<commit_message>
Implement top navigation layout with hamburger project selector and collapsible integrated checklist
</commit_message>
<xml_diff>
--- a/Schedule Preparation.xlsx
+++ b/Schedule Preparation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0. WtE Power Plant\Tools Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A863649-78B6-4609-A5C4-F5B39C8E3EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1077BE90-D0D1-42F6-B39D-73371F52DA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14303" yWindow="-98" windowWidth="28995" windowHeight="15675" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -601,7 +601,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -716,8 +716,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -810,11 +822,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -889,11 +916,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -914,7 +936,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -980,18 +1001,14 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1010,6 +1027,29 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1351,12 +1391,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D47"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="24"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="24.6"/>
   <cols>
-    <col min="1" max="1" width="69.36328125" style="1" customWidth="1"/>
-    <col min="2" max="4" width="13.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.90625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="1"/>
+    <col min="1" max="1" width="69.33203125" style="1" customWidth="1"/>
+    <col min="2" max="4" width="13.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.88671875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2026,592 +2066,592 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:PM48"/>
-  <sheetFormatPr defaultRowHeight="10"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="10.199999999999999"/>
   <cols>
-    <col min="1" max="1" width="5.36328125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="48.1796875" style="12" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="55" style="12" customWidth="1"/>
     <col min="3" max="3" width="19" style="12" customWidth="1"/>
-    <col min="4" max="4" width="2.6328125" style="14" customWidth="1"/>
-    <col min="5" max="10" width="2.6328125" style="13" customWidth="1"/>
-    <col min="11" max="11" width="2.6328125" style="14" customWidth="1"/>
-    <col min="12" max="17" width="2.6328125" style="13" customWidth="1"/>
-    <col min="18" max="18" width="2.6328125" style="14" customWidth="1"/>
-    <col min="19" max="24" width="2.6328125" style="13" customWidth="1"/>
-    <col min="25" max="25" width="2.6328125" style="15" customWidth="1"/>
-    <col min="26" max="31" width="2.6328125" style="12" customWidth="1"/>
-    <col min="32" max="32" width="2.6328125" style="15" customWidth="1"/>
-    <col min="33" max="38" width="2.6328125" style="12" customWidth="1"/>
-    <col min="39" max="39" width="2.6328125" style="15" customWidth="1"/>
-    <col min="40" max="45" width="2.6328125" style="12" customWidth="1"/>
-    <col min="46" max="46" width="2.6328125" style="15" customWidth="1"/>
-    <col min="47" max="52" width="2.6328125" style="12" customWidth="1"/>
-    <col min="53" max="53" width="2.6328125" style="15" customWidth="1"/>
-    <col min="54" max="59" width="2.6328125" style="12" customWidth="1"/>
-    <col min="60" max="60" width="2.6328125" style="15" customWidth="1"/>
-    <col min="61" max="66" width="2.6328125" style="12" customWidth="1"/>
-    <col min="67" max="67" width="2.6328125" style="15" customWidth="1"/>
-    <col min="68" max="73" width="2.6328125" style="12" customWidth="1"/>
-    <col min="74" max="74" width="2.6328125" style="15" customWidth="1"/>
-    <col min="75" max="80" width="2.6328125" style="12" customWidth="1"/>
-    <col min="81" max="81" width="2.6328125" style="15" customWidth="1"/>
-    <col min="82" max="87" width="2.6328125" style="12" customWidth="1"/>
-    <col min="88" max="88" width="2.6328125" style="15" customWidth="1"/>
-    <col min="89" max="94" width="2.6328125" style="12" customWidth="1"/>
-    <col min="95" max="95" width="2.6328125" style="15" customWidth="1"/>
-    <col min="96" max="101" width="2.6328125" style="12" customWidth="1"/>
-    <col min="102" max="102" width="2.6328125" style="15" customWidth="1"/>
-    <col min="103" max="108" width="2.6328125" style="12" customWidth="1"/>
-    <col min="109" max="109" width="2.6328125" style="15" customWidth="1"/>
-    <col min="110" max="115" width="2.6328125" style="12" customWidth="1"/>
-    <col min="116" max="116" width="2.6328125" style="15" customWidth="1"/>
-    <col min="117" max="122" width="2.6328125" style="12" customWidth="1"/>
-    <col min="123" max="123" width="2.6328125" style="15" customWidth="1"/>
-    <col min="124" max="129" width="2.6328125" style="12" customWidth="1"/>
-    <col min="130" max="130" width="2.6328125" style="15" customWidth="1"/>
-    <col min="131" max="136" width="2.6328125" style="12" customWidth="1"/>
-    <col min="137" max="137" width="2.6328125" style="15" customWidth="1"/>
-    <col min="138" max="143" width="2.6328125" style="12" customWidth="1"/>
-    <col min="144" max="144" width="2.6328125" style="15" customWidth="1"/>
-    <col min="145" max="150" width="2.6328125" style="12" customWidth="1"/>
-    <col min="151" max="151" width="2.6328125" style="15" customWidth="1"/>
-    <col min="152" max="157" width="2.6328125" style="12" customWidth="1"/>
-    <col min="158" max="158" width="2.6328125" style="15" customWidth="1"/>
-    <col min="159" max="164" width="2.6328125" style="12" customWidth="1"/>
-    <col min="165" max="165" width="2.6328125" style="15" customWidth="1"/>
-    <col min="166" max="171" width="2.6328125" style="12" customWidth="1"/>
-    <col min="172" max="172" width="2.6328125" style="15" customWidth="1"/>
-    <col min="173" max="178" width="2.6328125" style="12" customWidth="1"/>
-    <col min="179" max="179" width="2.6328125" style="15" customWidth="1"/>
-    <col min="180" max="185" width="2.6328125" style="12" customWidth="1"/>
-    <col min="186" max="186" width="2.6328125" style="15" customWidth="1"/>
-    <col min="187" max="192" width="2.6328125" style="12" customWidth="1"/>
-    <col min="193" max="193" width="2.6328125" style="15" customWidth="1"/>
-    <col min="194" max="199" width="2.6328125" style="12" customWidth="1"/>
-    <col min="200" max="200" width="2.6328125" style="15" customWidth="1"/>
-    <col min="201" max="206" width="2.6328125" style="12" customWidth="1"/>
-    <col min="207" max="207" width="2.6328125" style="15" customWidth="1"/>
-    <col min="208" max="213" width="2.6328125" style="12" customWidth="1"/>
-    <col min="214" max="214" width="2.6328125" style="15" customWidth="1"/>
-    <col min="215" max="220" width="2.6328125" style="12" customWidth="1"/>
-    <col min="221" max="221" width="2.6328125" style="15" customWidth="1"/>
-    <col min="222" max="227" width="2.6328125" style="12" customWidth="1"/>
-    <col min="228" max="228" width="2.6328125" style="15" customWidth="1"/>
-    <col min="229" max="234" width="2.6328125" style="12" customWidth="1"/>
-    <col min="235" max="235" width="2.6328125" style="15" customWidth="1"/>
-    <col min="236" max="241" width="2.6328125" style="12" customWidth="1"/>
-    <col min="242" max="242" width="2.6328125" style="15" customWidth="1"/>
-    <col min="243" max="248" width="2.6328125" style="12" customWidth="1"/>
-    <col min="249" max="249" width="2.6328125" style="15" customWidth="1"/>
-    <col min="250" max="255" width="2.6328125" style="12" customWidth="1"/>
-    <col min="256" max="256" width="2.6328125" style="15" customWidth="1"/>
-    <col min="257" max="262" width="2.6328125" style="12" customWidth="1"/>
-    <col min="263" max="263" width="2.6328125" style="15" customWidth="1"/>
-    <col min="264" max="269" width="2.6328125" style="12" customWidth="1"/>
-    <col min="270" max="270" width="2.6328125" style="15" customWidth="1"/>
-    <col min="271" max="276" width="2.6328125" style="12" customWidth="1"/>
-    <col min="277" max="277" width="2.6328125" style="15" customWidth="1"/>
-    <col min="278" max="283" width="2.6328125" style="12" customWidth="1"/>
-    <col min="284" max="284" width="2.6328125" style="15" customWidth="1"/>
-    <col min="285" max="290" width="2.6328125" style="12" customWidth="1"/>
-    <col min="291" max="291" width="2.6328125" style="15" customWidth="1"/>
-    <col min="292" max="297" width="2.6328125" style="12" customWidth="1"/>
-    <col min="298" max="298" width="2.6328125" style="15" customWidth="1"/>
-    <col min="299" max="304" width="2.6328125" style="12" customWidth="1"/>
-    <col min="305" max="305" width="2.6328125" style="15" customWidth="1"/>
-    <col min="306" max="311" width="2.6328125" style="12" customWidth="1"/>
-    <col min="312" max="312" width="2.6328125" style="15" customWidth="1"/>
-    <col min="313" max="318" width="2.6328125" style="12" customWidth="1"/>
-    <col min="319" max="319" width="2.6328125" style="15" customWidth="1"/>
-    <col min="320" max="325" width="2.6328125" style="12" customWidth="1"/>
-    <col min="326" max="326" width="2.6328125" style="15" customWidth="1"/>
-    <col min="327" max="332" width="2.6328125" style="12" customWidth="1"/>
-    <col min="333" max="333" width="2.6328125" style="15" customWidth="1"/>
-    <col min="334" max="339" width="2.6328125" style="12" customWidth="1"/>
-    <col min="340" max="340" width="2.6328125" style="15" customWidth="1"/>
-    <col min="341" max="346" width="2.6328125" style="12" customWidth="1"/>
-    <col min="347" max="347" width="2.6328125" style="15" customWidth="1"/>
-    <col min="348" max="353" width="2.6328125" style="12" customWidth="1"/>
-    <col min="354" max="354" width="2.6328125" style="15" customWidth="1"/>
-    <col min="355" max="360" width="2.6328125" style="12" customWidth="1"/>
-    <col min="361" max="361" width="2.6328125" style="15" customWidth="1"/>
-    <col min="362" max="367" width="2.6328125" style="12" customWidth="1"/>
-    <col min="368" max="368" width="2.6328125" style="15" customWidth="1"/>
-    <col min="369" max="374" width="2.6328125" style="12" customWidth="1"/>
-    <col min="375" max="375" width="2.6328125" style="15" customWidth="1"/>
-    <col min="376" max="381" width="2.6328125" style="12" customWidth="1"/>
-    <col min="382" max="382" width="2.6328125" style="15" customWidth="1"/>
-    <col min="383" max="388" width="2.6328125" style="12" customWidth="1"/>
-    <col min="389" max="389" width="2.6328125" style="15" customWidth="1"/>
-    <col min="390" max="395" width="2.6328125" style="12" customWidth="1"/>
-    <col min="396" max="396" width="2.6328125" style="15" customWidth="1"/>
-    <col min="397" max="402" width="2.6328125" style="12" customWidth="1"/>
-    <col min="403" max="403" width="2.6328125" style="15" customWidth="1"/>
-    <col min="404" max="409" width="2.6328125" style="12" customWidth="1"/>
-    <col min="410" max="410" width="2.6328125" style="15" customWidth="1"/>
-    <col min="411" max="416" width="2.6328125" style="12" customWidth="1"/>
-    <col min="417" max="417" width="2.6328125" style="15" customWidth="1"/>
-    <col min="418" max="423" width="2.6328125" style="12" customWidth="1"/>
-    <col min="424" max="424" width="2.6328125" style="15" customWidth="1"/>
-    <col min="425" max="429" width="2.6328125" style="12" customWidth="1"/>
-    <col min="430" max="430" width="8.7265625" style="12" customWidth="1"/>
-    <col min="431" max="16384" width="8.7265625" style="12"/>
+    <col min="4" max="4" width="2.6640625" style="14" customWidth="1"/>
+    <col min="5" max="10" width="2.6640625" style="13" customWidth="1"/>
+    <col min="11" max="11" width="2.6640625" style="14" customWidth="1"/>
+    <col min="12" max="17" width="2.6640625" style="13" customWidth="1"/>
+    <col min="18" max="18" width="2.6640625" style="14" customWidth="1"/>
+    <col min="19" max="24" width="2.6640625" style="13" customWidth="1"/>
+    <col min="25" max="25" width="2.6640625" style="15" customWidth="1"/>
+    <col min="26" max="31" width="2.6640625" style="12" customWidth="1"/>
+    <col min="32" max="32" width="2.6640625" style="15" customWidth="1"/>
+    <col min="33" max="38" width="2.6640625" style="12" customWidth="1"/>
+    <col min="39" max="39" width="2.6640625" style="15" customWidth="1"/>
+    <col min="40" max="45" width="2.6640625" style="12" customWidth="1"/>
+    <col min="46" max="46" width="2.6640625" style="15" customWidth="1"/>
+    <col min="47" max="52" width="2.6640625" style="12" customWidth="1"/>
+    <col min="53" max="53" width="2.6640625" style="15" customWidth="1"/>
+    <col min="54" max="59" width="2.6640625" style="12" customWidth="1"/>
+    <col min="60" max="60" width="2.6640625" style="15" customWidth="1"/>
+    <col min="61" max="66" width="2.6640625" style="12" customWidth="1"/>
+    <col min="67" max="67" width="2.6640625" style="15" customWidth="1"/>
+    <col min="68" max="73" width="2.6640625" style="12" customWidth="1"/>
+    <col min="74" max="74" width="2.6640625" style="15" customWidth="1"/>
+    <col min="75" max="80" width="2.6640625" style="12" customWidth="1"/>
+    <col min="81" max="81" width="2.6640625" style="15" customWidth="1"/>
+    <col min="82" max="87" width="2.6640625" style="12" customWidth="1"/>
+    <col min="88" max="88" width="2.6640625" style="15" customWidth="1"/>
+    <col min="89" max="94" width="2.6640625" style="12" customWidth="1"/>
+    <col min="95" max="95" width="2.6640625" style="15" customWidth="1"/>
+    <col min="96" max="101" width="2.6640625" style="12" customWidth="1"/>
+    <col min="102" max="102" width="2.6640625" style="15" customWidth="1"/>
+    <col min="103" max="108" width="2.6640625" style="12" customWidth="1"/>
+    <col min="109" max="109" width="2.6640625" style="15" customWidth="1"/>
+    <col min="110" max="115" width="2.6640625" style="12" customWidth="1"/>
+    <col min="116" max="116" width="2.6640625" style="15" customWidth="1"/>
+    <col min="117" max="122" width="2.6640625" style="12" customWidth="1"/>
+    <col min="123" max="123" width="2.6640625" style="15" customWidth="1"/>
+    <col min="124" max="129" width="2.6640625" style="12" customWidth="1"/>
+    <col min="130" max="130" width="2.6640625" style="15" customWidth="1"/>
+    <col min="131" max="136" width="2.6640625" style="12" customWidth="1"/>
+    <col min="137" max="137" width="2.6640625" style="15" customWidth="1"/>
+    <col min="138" max="143" width="2.6640625" style="12" customWidth="1"/>
+    <col min="144" max="144" width="2.6640625" style="15" customWidth="1"/>
+    <col min="145" max="150" width="2.6640625" style="12" customWidth="1"/>
+    <col min="151" max="151" width="2.6640625" style="15" customWidth="1"/>
+    <col min="152" max="157" width="2.6640625" style="12" customWidth="1"/>
+    <col min="158" max="158" width="2.6640625" style="15" customWidth="1"/>
+    <col min="159" max="164" width="2.6640625" style="12" customWidth="1"/>
+    <col min="165" max="165" width="2.6640625" style="15" customWidth="1"/>
+    <col min="166" max="171" width="2.6640625" style="12" customWidth="1"/>
+    <col min="172" max="172" width="2.6640625" style="15" customWidth="1"/>
+    <col min="173" max="178" width="2.6640625" style="12" customWidth="1"/>
+    <col min="179" max="179" width="2.6640625" style="15" customWidth="1"/>
+    <col min="180" max="185" width="2.6640625" style="12" customWidth="1"/>
+    <col min="186" max="186" width="2.6640625" style="15" customWidth="1"/>
+    <col min="187" max="192" width="2.6640625" style="12" customWidth="1"/>
+    <col min="193" max="193" width="2.6640625" style="15" customWidth="1"/>
+    <col min="194" max="199" width="2.6640625" style="12" customWidth="1"/>
+    <col min="200" max="200" width="2.6640625" style="15" customWidth="1"/>
+    <col min="201" max="206" width="2.6640625" style="12" customWidth="1"/>
+    <col min="207" max="207" width="2.6640625" style="15" customWidth="1"/>
+    <col min="208" max="213" width="2.6640625" style="12" customWidth="1"/>
+    <col min="214" max="214" width="2.6640625" style="15" customWidth="1"/>
+    <col min="215" max="220" width="2.6640625" style="12" customWidth="1"/>
+    <col min="221" max="221" width="2.6640625" style="15" customWidth="1"/>
+    <col min="222" max="227" width="2.6640625" style="12" customWidth="1"/>
+    <col min="228" max="228" width="2.6640625" style="15" customWidth="1"/>
+    <col min="229" max="234" width="2.6640625" style="12" customWidth="1"/>
+    <col min="235" max="235" width="2.6640625" style="15" customWidth="1"/>
+    <col min="236" max="241" width="2.6640625" style="12" customWidth="1"/>
+    <col min="242" max="242" width="2.6640625" style="15" customWidth="1"/>
+    <col min="243" max="248" width="2.6640625" style="12" customWidth="1"/>
+    <col min="249" max="249" width="2.6640625" style="15" customWidth="1"/>
+    <col min="250" max="255" width="2.6640625" style="12" customWidth="1"/>
+    <col min="256" max="256" width="2.6640625" style="15" customWidth="1"/>
+    <col min="257" max="262" width="2.6640625" style="12" customWidth="1"/>
+    <col min="263" max="263" width="2.6640625" style="15" customWidth="1"/>
+    <col min="264" max="269" width="2.6640625" style="12" customWidth="1"/>
+    <col min="270" max="270" width="2.6640625" style="15" customWidth="1"/>
+    <col min="271" max="276" width="2.6640625" style="12" customWidth="1"/>
+    <col min="277" max="277" width="2.6640625" style="15" customWidth="1"/>
+    <col min="278" max="283" width="2.6640625" style="12" customWidth="1"/>
+    <col min="284" max="284" width="2.6640625" style="15" customWidth="1"/>
+    <col min="285" max="290" width="2.6640625" style="12" customWidth="1"/>
+    <col min="291" max="291" width="2.6640625" style="15" customWidth="1"/>
+    <col min="292" max="297" width="2.6640625" style="12" customWidth="1"/>
+    <col min="298" max="298" width="2.6640625" style="15" customWidth="1"/>
+    <col min="299" max="304" width="2.6640625" style="12" customWidth="1"/>
+    <col min="305" max="305" width="2.6640625" style="15" customWidth="1"/>
+    <col min="306" max="311" width="2.6640625" style="12" customWidth="1"/>
+    <col min="312" max="312" width="2.6640625" style="15" customWidth="1"/>
+    <col min="313" max="318" width="2.6640625" style="12" customWidth="1"/>
+    <col min="319" max="319" width="2.6640625" style="15" customWidth="1"/>
+    <col min="320" max="325" width="2.6640625" style="12" customWidth="1"/>
+    <col min="326" max="326" width="2.6640625" style="15" customWidth="1"/>
+    <col min="327" max="332" width="2.6640625" style="12" customWidth="1"/>
+    <col min="333" max="333" width="2.6640625" style="15" customWidth="1"/>
+    <col min="334" max="339" width="2.6640625" style="12" customWidth="1"/>
+    <col min="340" max="340" width="2.6640625" style="15" customWidth="1"/>
+    <col min="341" max="346" width="2.6640625" style="12" customWidth="1"/>
+    <col min="347" max="347" width="2.6640625" style="15" customWidth="1"/>
+    <col min="348" max="353" width="2.6640625" style="12" customWidth="1"/>
+    <col min="354" max="354" width="2.6640625" style="15" customWidth="1"/>
+    <col min="355" max="360" width="2.6640625" style="12" customWidth="1"/>
+    <col min="361" max="361" width="2.6640625" style="15" customWidth="1"/>
+    <col min="362" max="367" width="2.6640625" style="12" customWidth="1"/>
+    <col min="368" max="368" width="2.6640625" style="15" customWidth="1"/>
+    <col min="369" max="374" width="2.6640625" style="12" customWidth="1"/>
+    <col min="375" max="375" width="2.6640625" style="15" customWidth="1"/>
+    <col min="376" max="381" width="2.6640625" style="12" customWidth="1"/>
+    <col min="382" max="382" width="2.6640625" style="15" customWidth="1"/>
+    <col min="383" max="388" width="2.6640625" style="12" customWidth="1"/>
+    <col min="389" max="389" width="2.6640625" style="15" customWidth="1"/>
+    <col min="390" max="395" width="2.6640625" style="12" customWidth="1"/>
+    <col min="396" max="396" width="2.6640625" style="15" customWidth="1"/>
+    <col min="397" max="402" width="2.6640625" style="12" customWidth="1"/>
+    <col min="403" max="403" width="2.6640625" style="15" customWidth="1"/>
+    <col min="404" max="409" width="2.6640625" style="12" customWidth="1"/>
+    <col min="410" max="410" width="2.6640625" style="15" customWidth="1"/>
+    <col min="411" max="416" width="2.6640625" style="12" customWidth="1"/>
+    <col min="417" max="417" width="2.6640625" style="15" customWidth="1"/>
+    <col min="418" max="423" width="2.6640625" style="12" customWidth="1"/>
+    <col min="424" max="424" width="2.6640625" style="15" customWidth="1"/>
+    <col min="425" max="429" width="2.6640625" style="12" customWidth="1"/>
+    <col min="430" max="430" width="8.77734375" style="12" customWidth="1"/>
+    <col min="431" max="16384" width="8.77734375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:429" ht="20" customHeight="1">
-      <c r="D1" s="30">
+    <row r="1" spans="2:429" ht="19.95" customHeight="1">
+      <c r="D1" s="70">
         <v>46327</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="32"/>
-      <c r="AH1" s="30">
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="71"/>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="71"/>
+      <c r="AD1" s="71"/>
+      <c r="AE1" s="71"/>
+      <c r="AF1" s="71"/>
+      <c r="AG1" s="72"/>
+      <c r="AH1" s="70">
         <v>46357</v>
       </c>
-      <c r="AI1" s="31"/>
-      <c r="AJ1" s="31"/>
-      <c r="AK1" s="31"/>
-      <c r="AL1" s="31"/>
-      <c r="AM1" s="31"/>
-      <c r="AN1" s="31"/>
-      <c r="AO1" s="31"/>
-      <c r="AP1" s="31"/>
-      <c r="AQ1" s="31"/>
-      <c r="AR1" s="31"/>
-      <c r="AS1" s="31"/>
-      <c r="AT1" s="31"/>
-      <c r="AU1" s="31"/>
-      <c r="AV1" s="31"/>
-      <c r="AW1" s="31"/>
-      <c r="AX1" s="31"/>
-      <c r="AY1" s="31"/>
-      <c r="AZ1" s="31"/>
-      <c r="BA1" s="31"/>
-      <c r="BB1" s="31"/>
-      <c r="BC1" s="31"/>
-      <c r="BD1" s="31"/>
-      <c r="BE1" s="31"/>
-      <c r="BF1" s="31"/>
-      <c r="BG1" s="31"/>
-      <c r="BH1" s="31"/>
-      <c r="BI1" s="31"/>
-      <c r="BJ1" s="31"/>
-      <c r="BK1" s="31"/>
-      <c r="BL1" s="32"/>
-      <c r="BM1" s="30">
+      <c r="AI1" s="71"/>
+      <c r="AJ1" s="71"/>
+      <c r="AK1" s="71"/>
+      <c r="AL1" s="71"/>
+      <c r="AM1" s="71"/>
+      <c r="AN1" s="71"/>
+      <c r="AO1" s="71"/>
+      <c r="AP1" s="71"/>
+      <c r="AQ1" s="71"/>
+      <c r="AR1" s="71"/>
+      <c r="AS1" s="71"/>
+      <c r="AT1" s="71"/>
+      <c r="AU1" s="71"/>
+      <c r="AV1" s="71"/>
+      <c r="AW1" s="71"/>
+      <c r="AX1" s="71"/>
+      <c r="AY1" s="71"/>
+      <c r="AZ1" s="71"/>
+      <c r="BA1" s="71"/>
+      <c r="BB1" s="71"/>
+      <c r="BC1" s="71"/>
+      <c r="BD1" s="71"/>
+      <c r="BE1" s="71"/>
+      <c r="BF1" s="71"/>
+      <c r="BG1" s="71"/>
+      <c r="BH1" s="71"/>
+      <c r="BI1" s="71"/>
+      <c r="BJ1" s="71"/>
+      <c r="BK1" s="71"/>
+      <c r="BL1" s="72"/>
+      <c r="BM1" s="70">
         <v>46388</v>
       </c>
-      <c r="BN1" s="31"/>
-      <c r="BO1" s="31"/>
-      <c r="BP1" s="31"/>
-      <c r="BQ1" s="31"/>
-      <c r="BR1" s="31"/>
-      <c r="BS1" s="31"/>
-      <c r="BT1" s="31"/>
-      <c r="BU1" s="31"/>
-      <c r="BV1" s="31"/>
-      <c r="BW1" s="31"/>
-      <c r="BX1" s="31"/>
-      <c r="BY1" s="31"/>
-      <c r="BZ1" s="31"/>
-      <c r="CA1" s="31"/>
-      <c r="CB1" s="31"/>
-      <c r="CC1" s="31"/>
-      <c r="CD1" s="31"/>
-      <c r="CE1" s="31"/>
-      <c r="CF1" s="31"/>
-      <c r="CG1" s="31"/>
-      <c r="CH1" s="31"/>
-      <c r="CI1" s="31"/>
-      <c r="CJ1" s="31"/>
-      <c r="CK1" s="31"/>
-      <c r="CL1" s="31"/>
-      <c r="CM1" s="31"/>
-      <c r="CN1" s="31"/>
-      <c r="CO1" s="31"/>
-      <c r="CP1" s="31"/>
-      <c r="CQ1" s="32"/>
-      <c r="CR1" s="30">
+      <c r="BN1" s="71"/>
+      <c r="BO1" s="71"/>
+      <c r="BP1" s="71"/>
+      <c r="BQ1" s="71"/>
+      <c r="BR1" s="71"/>
+      <c r="BS1" s="71"/>
+      <c r="BT1" s="71"/>
+      <c r="BU1" s="71"/>
+      <c r="BV1" s="71"/>
+      <c r="BW1" s="71"/>
+      <c r="BX1" s="71"/>
+      <c r="BY1" s="71"/>
+      <c r="BZ1" s="71"/>
+      <c r="CA1" s="71"/>
+      <c r="CB1" s="71"/>
+      <c r="CC1" s="71"/>
+      <c r="CD1" s="71"/>
+      <c r="CE1" s="71"/>
+      <c r="CF1" s="71"/>
+      <c r="CG1" s="71"/>
+      <c r="CH1" s="71"/>
+      <c r="CI1" s="71"/>
+      <c r="CJ1" s="71"/>
+      <c r="CK1" s="71"/>
+      <c r="CL1" s="71"/>
+      <c r="CM1" s="71"/>
+      <c r="CN1" s="71"/>
+      <c r="CO1" s="71"/>
+      <c r="CP1" s="71"/>
+      <c r="CQ1" s="72"/>
+      <c r="CR1" s="70">
         <v>46419</v>
       </c>
-      <c r="CS1" s="31"/>
-      <c r="CT1" s="31"/>
-      <c r="CU1" s="31"/>
-      <c r="CV1" s="31"/>
-      <c r="CW1" s="31"/>
-      <c r="CX1" s="31"/>
-      <c r="CY1" s="31"/>
-      <c r="CZ1" s="31"/>
-      <c r="DA1" s="31"/>
-      <c r="DB1" s="31"/>
-      <c r="DC1" s="31"/>
-      <c r="DD1" s="31"/>
-      <c r="DE1" s="31"/>
-      <c r="DF1" s="31"/>
-      <c r="DG1" s="31"/>
-      <c r="DH1" s="31"/>
-      <c r="DI1" s="31"/>
-      <c r="DJ1" s="31"/>
-      <c r="DK1" s="31"/>
-      <c r="DL1" s="31"/>
-      <c r="DM1" s="31"/>
-      <c r="DN1" s="31"/>
-      <c r="DO1" s="31"/>
-      <c r="DP1" s="31"/>
-      <c r="DQ1" s="31"/>
-      <c r="DR1" s="31"/>
-      <c r="DS1" s="32"/>
-      <c r="DT1" s="30">
+      <c r="CS1" s="71"/>
+      <c r="CT1" s="71"/>
+      <c r="CU1" s="71"/>
+      <c r="CV1" s="71"/>
+      <c r="CW1" s="71"/>
+      <c r="CX1" s="71"/>
+      <c r="CY1" s="71"/>
+      <c r="CZ1" s="71"/>
+      <c r="DA1" s="71"/>
+      <c r="DB1" s="71"/>
+      <c r="DC1" s="71"/>
+      <c r="DD1" s="71"/>
+      <c r="DE1" s="71"/>
+      <c r="DF1" s="71"/>
+      <c r="DG1" s="71"/>
+      <c r="DH1" s="71"/>
+      <c r="DI1" s="71"/>
+      <c r="DJ1" s="71"/>
+      <c r="DK1" s="71"/>
+      <c r="DL1" s="71"/>
+      <c r="DM1" s="71"/>
+      <c r="DN1" s="71"/>
+      <c r="DO1" s="71"/>
+      <c r="DP1" s="71"/>
+      <c r="DQ1" s="71"/>
+      <c r="DR1" s="71"/>
+      <c r="DS1" s="72"/>
+      <c r="DT1" s="70">
         <v>46447</v>
       </c>
-      <c r="DU1" s="31"/>
-      <c r="DV1" s="31"/>
-      <c r="DW1" s="31"/>
-      <c r="DX1" s="31"/>
-      <c r="DY1" s="31"/>
-      <c r="DZ1" s="31"/>
-      <c r="EA1" s="31"/>
-      <c r="EB1" s="31"/>
-      <c r="EC1" s="31"/>
-      <c r="ED1" s="31"/>
-      <c r="EE1" s="31"/>
-      <c r="EF1" s="31"/>
-      <c r="EG1" s="31"/>
-      <c r="EH1" s="31"/>
-      <c r="EI1" s="31"/>
-      <c r="EJ1" s="31"/>
-      <c r="EK1" s="31"/>
-      <c r="EL1" s="31"/>
-      <c r="EM1" s="31"/>
-      <c r="EN1" s="31"/>
-      <c r="EO1" s="31"/>
-      <c r="EP1" s="31"/>
-      <c r="EQ1" s="31"/>
-      <c r="ER1" s="31"/>
-      <c r="ES1" s="31"/>
-      <c r="ET1" s="31"/>
-      <c r="EU1" s="31"/>
-      <c r="EV1" s="31"/>
-      <c r="EW1" s="31"/>
-      <c r="EX1" s="32"/>
-      <c r="EY1" s="30">
+      <c r="DU1" s="71"/>
+      <c r="DV1" s="71"/>
+      <c r="DW1" s="71"/>
+      <c r="DX1" s="71"/>
+      <c r="DY1" s="71"/>
+      <c r="DZ1" s="71"/>
+      <c r="EA1" s="71"/>
+      <c r="EB1" s="71"/>
+      <c r="EC1" s="71"/>
+      <c r="ED1" s="71"/>
+      <c r="EE1" s="71"/>
+      <c r="EF1" s="71"/>
+      <c r="EG1" s="71"/>
+      <c r="EH1" s="71"/>
+      <c r="EI1" s="71"/>
+      <c r="EJ1" s="71"/>
+      <c r="EK1" s="71"/>
+      <c r="EL1" s="71"/>
+      <c r="EM1" s="71"/>
+      <c r="EN1" s="71"/>
+      <c r="EO1" s="71"/>
+      <c r="EP1" s="71"/>
+      <c r="EQ1" s="71"/>
+      <c r="ER1" s="71"/>
+      <c r="ES1" s="71"/>
+      <c r="ET1" s="71"/>
+      <c r="EU1" s="71"/>
+      <c r="EV1" s="71"/>
+      <c r="EW1" s="71"/>
+      <c r="EX1" s="72"/>
+      <c r="EY1" s="70">
         <v>46478</v>
       </c>
-      <c r="EZ1" s="31"/>
-      <c r="FA1" s="31"/>
-      <c r="FB1" s="31"/>
-      <c r="FC1" s="31"/>
-      <c r="FD1" s="31"/>
-      <c r="FE1" s="31"/>
-      <c r="FF1" s="31"/>
-      <c r="FG1" s="31"/>
-      <c r="FH1" s="31"/>
-      <c r="FI1" s="31"/>
-      <c r="FJ1" s="31"/>
-      <c r="FK1" s="31"/>
-      <c r="FL1" s="31"/>
-      <c r="FM1" s="31"/>
-      <c r="FN1" s="31"/>
-      <c r="FO1" s="31"/>
-      <c r="FP1" s="31"/>
-      <c r="FQ1" s="31"/>
-      <c r="FR1" s="31"/>
-      <c r="FS1" s="31"/>
-      <c r="FT1" s="31"/>
-      <c r="FU1" s="31"/>
-      <c r="FV1" s="31"/>
-      <c r="FW1" s="31"/>
-      <c r="FX1" s="31"/>
-      <c r="FY1" s="31"/>
-      <c r="FZ1" s="31"/>
-      <c r="GA1" s="31"/>
-      <c r="GB1" s="32"/>
-      <c r="GC1" s="30">
+      <c r="EZ1" s="71"/>
+      <c r="FA1" s="71"/>
+      <c r="FB1" s="71"/>
+      <c r="FC1" s="71"/>
+      <c r="FD1" s="71"/>
+      <c r="FE1" s="71"/>
+      <c r="FF1" s="71"/>
+      <c r="FG1" s="71"/>
+      <c r="FH1" s="71"/>
+      <c r="FI1" s="71"/>
+      <c r="FJ1" s="71"/>
+      <c r="FK1" s="71"/>
+      <c r="FL1" s="71"/>
+      <c r="FM1" s="71"/>
+      <c r="FN1" s="71"/>
+      <c r="FO1" s="71"/>
+      <c r="FP1" s="71"/>
+      <c r="FQ1" s="71"/>
+      <c r="FR1" s="71"/>
+      <c r="FS1" s="71"/>
+      <c r="FT1" s="71"/>
+      <c r="FU1" s="71"/>
+      <c r="FV1" s="71"/>
+      <c r="FW1" s="71"/>
+      <c r="FX1" s="71"/>
+      <c r="FY1" s="71"/>
+      <c r="FZ1" s="71"/>
+      <c r="GA1" s="71"/>
+      <c r="GB1" s="72"/>
+      <c r="GC1" s="70">
         <v>46508</v>
       </c>
-      <c r="GD1" s="31"/>
-      <c r="GE1" s="31"/>
-      <c r="GF1" s="31"/>
-      <c r="GG1" s="31"/>
-      <c r="GH1" s="31"/>
-      <c r="GI1" s="31"/>
-      <c r="GJ1" s="31"/>
-      <c r="GK1" s="31"/>
-      <c r="GL1" s="31"/>
-      <c r="GM1" s="31"/>
-      <c r="GN1" s="31"/>
-      <c r="GO1" s="31"/>
-      <c r="GP1" s="31"/>
-      <c r="GQ1" s="31"/>
-      <c r="GR1" s="31"/>
-      <c r="GS1" s="31"/>
-      <c r="GT1" s="31"/>
-      <c r="GU1" s="31"/>
-      <c r="GV1" s="31"/>
-      <c r="GW1" s="31"/>
-      <c r="GX1" s="31"/>
-      <c r="GY1" s="31"/>
-      <c r="GZ1" s="31"/>
-      <c r="HA1" s="31"/>
-      <c r="HB1" s="31"/>
-      <c r="HC1" s="31"/>
-      <c r="HD1" s="31"/>
-      <c r="HE1" s="31"/>
-      <c r="HF1" s="31"/>
-      <c r="HG1" s="32"/>
-      <c r="HH1" s="30">
+      <c r="GD1" s="71"/>
+      <c r="GE1" s="71"/>
+      <c r="GF1" s="71"/>
+      <c r="GG1" s="71"/>
+      <c r="GH1" s="71"/>
+      <c r="GI1" s="71"/>
+      <c r="GJ1" s="71"/>
+      <c r="GK1" s="71"/>
+      <c r="GL1" s="71"/>
+      <c r="GM1" s="71"/>
+      <c r="GN1" s="71"/>
+      <c r="GO1" s="71"/>
+      <c r="GP1" s="71"/>
+      <c r="GQ1" s="71"/>
+      <c r="GR1" s="71"/>
+      <c r="GS1" s="71"/>
+      <c r="GT1" s="71"/>
+      <c r="GU1" s="71"/>
+      <c r="GV1" s="71"/>
+      <c r="GW1" s="71"/>
+      <c r="GX1" s="71"/>
+      <c r="GY1" s="71"/>
+      <c r="GZ1" s="71"/>
+      <c r="HA1" s="71"/>
+      <c r="HB1" s="71"/>
+      <c r="HC1" s="71"/>
+      <c r="HD1" s="71"/>
+      <c r="HE1" s="71"/>
+      <c r="HF1" s="71"/>
+      <c r="HG1" s="72"/>
+      <c r="HH1" s="70">
         <v>46539</v>
       </c>
-      <c r="HI1" s="31"/>
-      <c r="HJ1" s="31"/>
-      <c r="HK1" s="31"/>
-      <c r="HL1" s="31"/>
-      <c r="HM1" s="31"/>
-      <c r="HN1" s="31"/>
-      <c r="HO1" s="31"/>
-      <c r="HP1" s="31"/>
-      <c r="HQ1" s="31"/>
-      <c r="HR1" s="31"/>
-      <c r="HS1" s="31"/>
-      <c r="HT1" s="31"/>
-      <c r="HU1" s="31"/>
-      <c r="HV1" s="31"/>
-      <c r="HW1" s="31"/>
-      <c r="HX1" s="31"/>
-      <c r="HY1" s="31"/>
-      <c r="HZ1" s="31"/>
-      <c r="IA1" s="31"/>
-      <c r="IB1" s="31"/>
-      <c r="IC1" s="31"/>
-      <c r="ID1" s="31"/>
-      <c r="IE1" s="31"/>
-      <c r="IF1" s="31"/>
-      <c r="IG1" s="31"/>
-      <c r="IH1" s="31"/>
-      <c r="II1" s="31"/>
-      <c r="IJ1" s="31"/>
-      <c r="IK1" s="32"/>
-      <c r="IL1" s="30">
+      <c r="HI1" s="71"/>
+      <c r="HJ1" s="71"/>
+      <c r="HK1" s="71"/>
+      <c r="HL1" s="71"/>
+      <c r="HM1" s="71"/>
+      <c r="HN1" s="71"/>
+      <c r="HO1" s="71"/>
+      <c r="HP1" s="71"/>
+      <c r="HQ1" s="71"/>
+      <c r="HR1" s="71"/>
+      <c r="HS1" s="71"/>
+      <c r="HT1" s="71"/>
+      <c r="HU1" s="71"/>
+      <c r="HV1" s="71"/>
+      <c r="HW1" s="71"/>
+      <c r="HX1" s="71"/>
+      <c r="HY1" s="71"/>
+      <c r="HZ1" s="71"/>
+      <c r="IA1" s="71"/>
+      <c r="IB1" s="71"/>
+      <c r="IC1" s="71"/>
+      <c r="ID1" s="71"/>
+      <c r="IE1" s="71"/>
+      <c r="IF1" s="71"/>
+      <c r="IG1" s="71"/>
+      <c r="IH1" s="71"/>
+      <c r="II1" s="71"/>
+      <c r="IJ1" s="71"/>
+      <c r="IK1" s="72"/>
+      <c r="IL1" s="70">
         <v>46569</v>
       </c>
-      <c r="IM1" s="31"/>
-      <c r="IN1" s="31"/>
-      <c r="IO1" s="31"/>
-      <c r="IP1" s="31"/>
-      <c r="IQ1" s="31"/>
-      <c r="IR1" s="31"/>
-      <c r="IS1" s="31"/>
-      <c r="IT1" s="31"/>
-      <c r="IU1" s="31"/>
-      <c r="IV1" s="31"/>
-      <c r="IW1" s="31"/>
-      <c r="IX1" s="31"/>
-      <c r="IY1" s="31"/>
-      <c r="IZ1" s="31"/>
-      <c r="JA1" s="31"/>
-      <c r="JB1" s="31"/>
-      <c r="JC1" s="31"/>
-      <c r="JD1" s="31"/>
-      <c r="JE1" s="31"/>
-      <c r="JF1" s="31"/>
-      <c r="JG1" s="31"/>
-      <c r="JH1" s="31"/>
-      <c r="JI1" s="31"/>
-      <c r="JJ1" s="31"/>
-      <c r="JK1" s="31"/>
-      <c r="JL1" s="31"/>
-      <c r="JM1" s="31"/>
-      <c r="JN1" s="31"/>
-      <c r="JO1" s="31"/>
-      <c r="JP1" s="32"/>
-      <c r="JQ1" s="30">
+      <c r="IM1" s="71"/>
+      <c r="IN1" s="71"/>
+      <c r="IO1" s="71"/>
+      <c r="IP1" s="71"/>
+      <c r="IQ1" s="71"/>
+      <c r="IR1" s="71"/>
+      <c r="IS1" s="71"/>
+      <c r="IT1" s="71"/>
+      <c r="IU1" s="71"/>
+      <c r="IV1" s="71"/>
+      <c r="IW1" s="71"/>
+      <c r="IX1" s="71"/>
+      <c r="IY1" s="71"/>
+      <c r="IZ1" s="71"/>
+      <c r="JA1" s="71"/>
+      <c r="JB1" s="71"/>
+      <c r="JC1" s="71"/>
+      <c r="JD1" s="71"/>
+      <c r="JE1" s="71"/>
+      <c r="JF1" s="71"/>
+      <c r="JG1" s="71"/>
+      <c r="JH1" s="71"/>
+      <c r="JI1" s="71"/>
+      <c r="JJ1" s="71"/>
+      <c r="JK1" s="71"/>
+      <c r="JL1" s="71"/>
+      <c r="JM1" s="71"/>
+      <c r="JN1" s="71"/>
+      <c r="JO1" s="71"/>
+      <c r="JP1" s="72"/>
+      <c r="JQ1" s="70">
         <v>46600</v>
       </c>
-      <c r="JR1" s="31"/>
-      <c r="JS1" s="31"/>
-      <c r="JT1" s="31"/>
-      <c r="JU1" s="31"/>
-      <c r="JV1" s="31"/>
-      <c r="JW1" s="31"/>
-      <c r="JX1" s="31"/>
-      <c r="JY1" s="31"/>
-      <c r="JZ1" s="31"/>
-      <c r="KA1" s="31"/>
-      <c r="KB1" s="31"/>
-      <c r="KC1" s="31"/>
-      <c r="KD1" s="31"/>
-      <c r="KE1" s="31"/>
-      <c r="KF1" s="31"/>
-      <c r="KG1" s="31"/>
-      <c r="KH1" s="31"/>
-      <c r="KI1" s="31"/>
-      <c r="KJ1" s="31"/>
-      <c r="KK1" s="31"/>
-      <c r="KL1" s="31"/>
-      <c r="KM1" s="31"/>
-      <c r="KN1" s="31"/>
-      <c r="KO1" s="31"/>
-      <c r="KP1" s="31"/>
-      <c r="KQ1" s="31"/>
-      <c r="KR1" s="31"/>
-      <c r="KS1" s="31"/>
-      <c r="KT1" s="31"/>
-      <c r="KU1" s="32"/>
-      <c r="KV1" s="30">
+      <c r="JR1" s="71"/>
+      <c r="JS1" s="71"/>
+      <c r="JT1" s="71"/>
+      <c r="JU1" s="71"/>
+      <c r="JV1" s="71"/>
+      <c r="JW1" s="71"/>
+      <c r="JX1" s="71"/>
+      <c r="JY1" s="71"/>
+      <c r="JZ1" s="71"/>
+      <c r="KA1" s="71"/>
+      <c r="KB1" s="71"/>
+      <c r="KC1" s="71"/>
+      <c r="KD1" s="71"/>
+      <c r="KE1" s="71"/>
+      <c r="KF1" s="71"/>
+      <c r="KG1" s="71"/>
+      <c r="KH1" s="71"/>
+      <c r="KI1" s="71"/>
+      <c r="KJ1" s="71"/>
+      <c r="KK1" s="71"/>
+      <c r="KL1" s="71"/>
+      <c r="KM1" s="71"/>
+      <c r="KN1" s="71"/>
+      <c r="KO1" s="71"/>
+      <c r="KP1" s="71"/>
+      <c r="KQ1" s="71"/>
+      <c r="KR1" s="71"/>
+      <c r="KS1" s="71"/>
+      <c r="KT1" s="71"/>
+      <c r="KU1" s="72"/>
+      <c r="KV1" s="70">
         <v>46631</v>
       </c>
-      <c r="KW1" s="31"/>
-      <c r="KX1" s="31"/>
-      <c r="KY1" s="31"/>
-      <c r="KZ1" s="31"/>
-      <c r="LA1" s="31"/>
-      <c r="LB1" s="31"/>
-      <c r="LC1" s="31"/>
-      <c r="LD1" s="31"/>
-      <c r="LE1" s="31"/>
-      <c r="LF1" s="31"/>
-      <c r="LG1" s="31"/>
-      <c r="LH1" s="31"/>
-      <c r="LI1" s="31"/>
-      <c r="LJ1" s="31"/>
-      <c r="LK1" s="31"/>
-      <c r="LL1" s="31"/>
-      <c r="LM1" s="31"/>
-      <c r="LN1" s="31"/>
-      <c r="LO1" s="31"/>
-      <c r="LP1" s="31"/>
-      <c r="LQ1" s="31"/>
-      <c r="LR1" s="31"/>
-      <c r="LS1" s="31"/>
-      <c r="LT1" s="31"/>
-      <c r="LU1" s="31"/>
-      <c r="LV1" s="31"/>
-      <c r="LW1" s="31"/>
-      <c r="LX1" s="31"/>
-      <c r="LY1" s="32"/>
-      <c r="LZ1" s="30">
+      <c r="KW1" s="71"/>
+      <c r="KX1" s="71"/>
+      <c r="KY1" s="71"/>
+      <c r="KZ1" s="71"/>
+      <c r="LA1" s="71"/>
+      <c r="LB1" s="71"/>
+      <c r="LC1" s="71"/>
+      <c r="LD1" s="71"/>
+      <c r="LE1" s="71"/>
+      <c r="LF1" s="71"/>
+      <c r="LG1" s="71"/>
+      <c r="LH1" s="71"/>
+      <c r="LI1" s="71"/>
+      <c r="LJ1" s="71"/>
+      <c r="LK1" s="71"/>
+      <c r="LL1" s="71"/>
+      <c r="LM1" s="71"/>
+      <c r="LN1" s="71"/>
+      <c r="LO1" s="71"/>
+      <c r="LP1" s="71"/>
+      <c r="LQ1" s="71"/>
+      <c r="LR1" s="71"/>
+      <c r="LS1" s="71"/>
+      <c r="LT1" s="71"/>
+      <c r="LU1" s="71"/>
+      <c r="LV1" s="71"/>
+      <c r="LW1" s="71"/>
+      <c r="LX1" s="71"/>
+      <c r="LY1" s="72"/>
+      <c r="LZ1" s="70">
         <v>46661</v>
       </c>
-      <c r="MA1" s="31"/>
-      <c r="MB1" s="31"/>
-      <c r="MC1" s="31"/>
-      <c r="MD1" s="31"/>
-      <c r="ME1" s="31"/>
-      <c r="MF1" s="31"/>
-      <c r="MG1" s="31"/>
-      <c r="MH1" s="31"/>
-      <c r="MI1" s="31"/>
-      <c r="MJ1" s="31"/>
-      <c r="MK1" s="31"/>
-      <c r="ML1" s="31"/>
-      <c r="MM1" s="31"/>
-      <c r="MN1" s="31"/>
-      <c r="MO1" s="31"/>
-      <c r="MP1" s="31"/>
-      <c r="MQ1" s="31"/>
-      <c r="MR1" s="31"/>
-      <c r="MS1" s="31"/>
-      <c r="MT1" s="31"/>
-      <c r="MU1" s="31"/>
-      <c r="MV1" s="31"/>
-      <c r="MW1" s="31"/>
-      <c r="MX1" s="31"/>
-      <c r="MY1" s="31"/>
-      <c r="MZ1" s="31"/>
-      <c r="NA1" s="31"/>
-      <c r="NB1" s="31"/>
-      <c r="NC1" s="31"/>
-      <c r="ND1" s="32"/>
-      <c r="NE1" s="30">
+      <c r="MA1" s="71"/>
+      <c r="MB1" s="71"/>
+      <c r="MC1" s="71"/>
+      <c r="MD1" s="71"/>
+      <c r="ME1" s="71"/>
+      <c r="MF1" s="71"/>
+      <c r="MG1" s="71"/>
+      <c r="MH1" s="71"/>
+      <c r="MI1" s="71"/>
+      <c r="MJ1" s="71"/>
+      <c r="MK1" s="71"/>
+      <c r="ML1" s="71"/>
+      <c r="MM1" s="71"/>
+      <c r="MN1" s="71"/>
+      <c r="MO1" s="71"/>
+      <c r="MP1" s="71"/>
+      <c r="MQ1" s="71"/>
+      <c r="MR1" s="71"/>
+      <c r="MS1" s="71"/>
+      <c r="MT1" s="71"/>
+      <c r="MU1" s="71"/>
+      <c r="MV1" s="71"/>
+      <c r="MW1" s="71"/>
+      <c r="MX1" s="71"/>
+      <c r="MY1" s="71"/>
+      <c r="MZ1" s="71"/>
+      <c r="NA1" s="71"/>
+      <c r="NB1" s="71"/>
+      <c r="NC1" s="71"/>
+      <c r="ND1" s="72"/>
+      <c r="NE1" s="70">
         <v>46692</v>
       </c>
-      <c r="NF1" s="31"/>
-      <c r="NG1" s="31"/>
-      <c r="NH1" s="31"/>
-      <c r="NI1" s="31"/>
-      <c r="NJ1" s="31"/>
-      <c r="NK1" s="31"/>
-      <c r="NL1" s="31"/>
-      <c r="NM1" s="31"/>
-      <c r="NN1" s="31"/>
-      <c r="NO1" s="31"/>
-      <c r="NP1" s="31"/>
-      <c r="NQ1" s="31"/>
-      <c r="NR1" s="31"/>
-      <c r="NS1" s="31"/>
-      <c r="NT1" s="31"/>
-      <c r="NU1" s="31"/>
-      <c r="NV1" s="31"/>
-      <c r="NW1" s="31"/>
-      <c r="NX1" s="31"/>
-      <c r="NY1" s="31"/>
-      <c r="NZ1" s="31"/>
-      <c r="OA1" s="31"/>
-      <c r="OB1" s="31"/>
-      <c r="OC1" s="31"/>
-      <c r="OD1" s="31"/>
-      <c r="OE1" s="31"/>
-      <c r="OF1" s="31"/>
-      <c r="OG1" s="31"/>
-      <c r="OH1" s="32"/>
-      <c r="OI1" s="30">
+      <c r="NF1" s="71"/>
+      <c r="NG1" s="71"/>
+      <c r="NH1" s="71"/>
+      <c r="NI1" s="71"/>
+      <c r="NJ1" s="71"/>
+      <c r="NK1" s="71"/>
+      <c r="NL1" s="71"/>
+      <c r="NM1" s="71"/>
+      <c r="NN1" s="71"/>
+      <c r="NO1" s="71"/>
+      <c r="NP1" s="71"/>
+      <c r="NQ1" s="71"/>
+      <c r="NR1" s="71"/>
+      <c r="NS1" s="71"/>
+      <c r="NT1" s="71"/>
+      <c r="NU1" s="71"/>
+      <c r="NV1" s="71"/>
+      <c r="NW1" s="71"/>
+      <c r="NX1" s="71"/>
+      <c r="NY1" s="71"/>
+      <c r="NZ1" s="71"/>
+      <c r="OA1" s="71"/>
+      <c r="OB1" s="71"/>
+      <c r="OC1" s="71"/>
+      <c r="OD1" s="71"/>
+      <c r="OE1" s="71"/>
+      <c r="OF1" s="71"/>
+      <c r="OG1" s="71"/>
+      <c r="OH1" s="72"/>
+      <c r="OI1" s="70">
         <v>46722</v>
       </c>
-      <c r="OJ1" s="31"/>
-      <c r="OK1" s="31"/>
-      <c r="OL1" s="31"/>
-      <c r="OM1" s="31"/>
-      <c r="ON1" s="31"/>
-      <c r="OO1" s="31"/>
-      <c r="OP1" s="31"/>
-      <c r="OQ1" s="31"/>
-      <c r="OR1" s="31"/>
-      <c r="OS1" s="31"/>
-      <c r="OT1" s="31"/>
-      <c r="OU1" s="31"/>
-      <c r="OV1" s="31"/>
-      <c r="OW1" s="31"/>
-      <c r="OX1" s="31"/>
-      <c r="OY1" s="31"/>
-      <c r="OZ1" s="31"/>
-      <c r="PA1" s="31"/>
-      <c r="PB1" s="31"/>
-      <c r="PC1" s="31"/>
-      <c r="PD1" s="31"/>
-      <c r="PE1" s="31"/>
-      <c r="PF1" s="31"/>
-      <c r="PG1" s="31"/>
-      <c r="PH1" s="31"/>
-      <c r="PI1" s="31"/>
-      <c r="PJ1" s="31"/>
-      <c r="PK1" s="31"/>
-      <c r="PL1" s="31"/>
-      <c r="PM1" s="32"/>
+      <c r="OJ1" s="71"/>
+      <c r="OK1" s="71"/>
+      <c r="OL1" s="71"/>
+      <c r="OM1" s="71"/>
+      <c r="ON1" s="71"/>
+      <c r="OO1" s="71"/>
+      <c r="OP1" s="71"/>
+      <c r="OQ1" s="71"/>
+      <c r="OR1" s="71"/>
+      <c r="OS1" s="71"/>
+      <c r="OT1" s="71"/>
+      <c r="OU1" s="71"/>
+      <c r="OV1" s="71"/>
+      <c r="OW1" s="71"/>
+      <c r="OX1" s="71"/>
+      <c r="OY1" s="71"/>
+      <c r="OZ1" s="71"/>
+      <c r="PA1" s="71"/>
+      <c r="PB1" s="71"/>
+      <c r="PC1" s="71"/>
+      <c r="PD1" s="71"/>
+      <c r="PE1" s="71"/>
+      <c r="PF1" s="71"/>
+      <c r="PG1" s="71"/>
+      <c r="PH1" s="71"/>
+      <c r="PI1" s="71"/>
+      <c r="PJ1" s="71"/>
+      <c r="PK1" s="71"/>
+      <c r="PL1" s="71"/>
+      <c r="PM1" s="72"/>
     </row>
     <row r="2" spans="2:429" ht="10.5" customHeight="1">
       <c r="B2" s="25" t="s">
@@ -3906,7 +3946,7 @@
       <c r="C3" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="26"/>
+      <c r="AE3" s="37"/>
       <c r="AF3" s="26"/>
       <c r="AG3" s="26"/>
       <c r="AH3" s="26"/>
@@ -4235,7 +4275,7 @@
       <c r="C4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AE4" s="26"/>
+      <c r="AE4" s="37"/>
       <c r="AF4" s="26"/>
       <c r="AG4" s="26"/>
       <c r="AH4" s="26"/>
@@ -4456,13 +4496,13 @@
       <c r="CU5" s="26"/>
     </row>
     <row r="6" spans="2:429" ht="15" customHeight="1">
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="BQ6" s="40"/>
+      <c r="BQ6" s="37"/>
       <c r="BR6" s="26"/>
       <c r="BS6" s="26"/>
       <c r="BT6" s="26"/>
@@ -4472,13 +4512,13 @@
       <c r="BX6" s="26"/>
     </row>
     <row r="7" spans="2:429" ht="15" customHeight="1">
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="AQ7" s="40"/>
+      <c r="AQ7" s="37"/>
       <c r="AR7" s="26"/>
       <c r="AS7" s="26"/>
       <c r="AT7" s="26"/>
@@ -4503,9 +4543,9 @@
       <c r="C8" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="BY8" s="33"/>
-      <c r="BZ8" s="33"/>
-      <c r="CA8" s="33"/>
+      <c r="BY8" s="30"/>
+      <c r="BZ8" s="30"/>
+      <c r="CA8" s="30"/>
     </row>
     <row r="9" spans="2:429" ht="15" customHeight="1">
       <c r="B9" s="21" t="s">
@@ -4514,7 +4554,7 @@
       <c r="C9" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="CB9" s="40"/>
+      <c r="CB9" s="37"/>
       <c r="CC9" s="26"/>
       <c r="CD9" s="26"/>
       <c r="CE9" s="26"/>
@@ -4530,7 +4570,7 @@
       <c r="C10" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="CZ10" s="40"/>
+      <c r="CZ10" s="37"/>
       <c r="DA10" s="26"/>
       <c r="DB10" s="26"/>
       <c r="DC10" s="26"/>
@@ -4549,7 +4589,7 @@
       <c r="C11" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="CS11" s="40"/>
+      <c r="CS11" s="37"/>
       <c r="CT11" s="26"/>
       <c r="CU11" s="26"/>
       <c r="CV11" s="26"/>
@@ -4564,7 +4604,7 @@
       <c r="C12" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="DK12" s="40"/>
+      <c r="DK12" s="37"/>
       <c r="DL12" s="26"/>
       <c r="DM12" s="26"/>
       <c r="DN12" s="26"/>
@@ -4596,7 +4636,7 @@
       <c r="C13" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="EI13" s="40"/>
+      <c r="EI13" s="37"/>
       <c r="EJ13" s="26"/>
       <c r="EK13" s="26"/>
       <c r="EL13" s="26"/>
@@ -4618,7 +4658,7 @@
       <c r="C14" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="CF14" s="40"/>
+      <c r="CF14" s="37"/>
       <c r="CG14" s="26"/>
       <c r="CH14" s="26"/>
       <c r="CI14" s="26"/>
@@ -4725,7 +4765,7 @@
       <c r="C15" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="CB15" s="40"/>
+      <c r="CB15" s="37"/>
       <c r="CC15" s="26"/>
       <c r="CD15" s="26"/>
       <c r="CE15" s="26"/>
@@ -4768,7 +4808,7 @@
       <c r="C16" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="CR16" s="40"/>
+      <c r="CR16" s="37"/>
       <c r="CS16" s="26"/>
       <c r="CT16" s="26"/>
       <c r="CU16" s="26"/>
@@ -4784,7 +4824,7 @@
       <c r="C17" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="CR17" s="40"/>
+      <c r="CR17" s="37"/>
       <c r="CS17" s="26"/>
       <c r="CT17" s="26"/>
       <c r="CU17" s="26"/>
@@ -4826,7 +4866,7 @@
       <c r="C18" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="AE18" s="40"/>
+      <c r="AE18" s="37"/>
       <c r="AF18" s="26"/>
       <c r="AG18" s="26"/>
       <c r="AH18" s="26"/>
@@ -5011,13 +5051,13 @@
       <c r="HE18" s="26"/>
     </row>
     <row r="19" spans="2:215" ht="15" customHeight="1">
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="AE19" s="40"/>
+      <c r="AE19" s="37"/>
       <c r="AF19" s="26"/>
       <c r="AG19" s="26"/>
       <c r="AH19" s="26"/>
@@ -5054,7 +5094,7 @@
       <c r="C21" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="EZ21" s="40"/>
+      <c r="EZ21" s="37"/>
       <c r="FA21" s="26"/>
       <c r="FB21" s="26"/>
       <c r="FC21" s="26"/>
@@ -5074,7 +5114,7 @@
       <c r="C22" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="CI22" s="40"/>
+      <c r="CI22" s="37"/>
       <c r="CJ22" s="26"/>
       <c r="CK22" s="26"/>
       <c r="CL22" s="26"/>
@@ -5102,7 +5142,7 @@
       <c r="C23" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="EI23" s="40"/>
+      <c r="EI23" s="37"/>
       <c r="EJ23" s="26"/>
       <c r="EK23" s="26"/>
       <c r="EL23" s="26"/>
@@ -5124,7 +5164,7 @@
       <c r="C24" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="EI24" s="40"/>
+      <c r="EI24" s="37"/>
       <c r="EJ24" s="26"/>
       <c r="EK24" s="26"/>
       <c r="EL24" s="26"/>
@@ -5142,7 +5182,7 @@
       <c r="C25" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="FL25" s="40"/>
+      <c r="FL25" s="37"/>
       <c r="FM25" s="26"/>
       <c r="FN25" s="26"/>
       <c r="FO25" s="26"/>
@@ -5152,13 +5192,13 @@
       <c r="FS25" s="26"/>
     </row>
     <row r="26" spans="2:215" ht="15" customHeight="1">
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="78" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="78" t="s">
         <v>48</v>
       </c>
-      <c r="FT26" s="41"/>
+      <c r="FT26" s="37"/>
       <c r="FU26" s="26"/>
       <c r="FV26" s="26"/>
       <c r="FW26" s="26"/>
@@ -5183,7 +5223,7 @@
       <c r="C27" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="GL27" s="40"/>
+      <c r="GL27" s="37"/>
       <c r="GM27" s="26"/>
       <c r="GN27" s="26"/>
       <c r="GO27" s="26"/>
@@ -5199,7 +5239,7 @@
       <c r="C28" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="GT28" s="40"/>
+      <c r="GT28" s="37"/>
       <c r="GU28" s="26"/>
       <c r="GV28" s="26"/>
       <c r="GW28" s="26"/>
@@ -5216,7 +5256,7 @@
       <c r="C29" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="GE29" s="40"/>
+      <c r="GE29" s="37"/>
       <c r="GF29" s="26"/>
       <c r="GG29" s="26"/>
       <c r="GH29" s="26"/>
@@ -5248,7 +5288,7 @@
       <c r="C30" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="HC30" s="40"/>
+      <c r="HC30" s="37"/>
       <c r="HD30" s="26"/>
     </row>
     <row r="31" spans="2:215" ht="15" customHeight="1">
@@ -5258,7 +5298,7 @@
       <c r="C31" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="HB31" s="40"/>
+      <c r="HB31" s="37"/>
       <c r="HC31" s="26"/>
       <c r="HD31" s="26"/>
     </row>
@@ -5269,7 +5309,7 @@
       <c r="C32" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="HE32" s="40"/>
+      <c r="HE32" s="37"/>
       <c r="HF32" s="26"/>
       <c r="HG32" s="26"/>
     </row>
@@ -5280,7 +5320,7 @@
       <c r="C33" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="BN33" s="40"/>
+      <c r="BN33" s="37"/>
       <c r="BO33" s="26"/>
       <c r="BP33" s="26"/>
       <c r="BQ33" s="26"/>
@@ -5323,7 +5363,7 @@
       <c r="C34" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="HH34" s="40"/>
+      <c r="HH34" s="37"/>
       <c r="HI34" s="26"/>
       <c r="HJ34" s="26"/>
     </row>
@@ -5334,7 +5374,7 @@
       <c r="C35" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="HK35" s="40"/>
+      <c r="HK35" s="37"/>
       <c r="HL35" s="26"/>
       <c r="HM35" s="26"/>
       <c r="HN35" s="26"/>
@@ -5346,7 +5386,7 @@
       <c r="C36" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="HO36" s="40"/>
+      <c r="HO36" s="37"/>
       <c r="HP36" s="26"/>
       <c r="HQ36" s="26"/>
       <c r="HR36" s="26"/>
@@ -5362,7 +5402,7 @@
       <c r="C37" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="HW37" s="44"/>
+      <c r="HW37" s="40"/>
       <c r="HX37" s="26"/>
       <c r="HY37" s="26"/>
       <c r="HZ37" s="26"/>
@@ -5430,7 +5470,7 @@
       <c r="C38" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="HW38" s="44"/>
+      <c r="HW38" s="40"/>
       <c r="HX38" s="26"/>
       <c r="HY38" s="26"/>
       <c r="HZ38" s="26"/>
@@ -5444,7 +5484,7 @@
       <c r="C39" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="IC39" s="44"/>
+      <c r="IC39" s="40"/>
       <c r="ID39" s="26"/>
       <c r="IE39" s="26"/>
       <c r="IF39" s="26"/>
@@ -5457,7 +5497,7 @@
       <c r="C40" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="II40" s="44"/>
+      <c r="II40" s="40"/>
       <c r="IJ40" s="26"/>
       <c r="IK40" s="26"/>
       <c r="IL40" s="26"/>
@@ -5470,7 +5510,7 @@
       <c r="C41" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="IN41" s="44"/>
+      <c r="IN41" s="40"/>
       <c r="IO41" s="26"/>
       <c r="IP41" s="26"/>
       <c r="IQ41" s="26"/>
@@ -5496,7 +5536,7 @@
       <c r="C42" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="JF42" s="44"/>
+      <c r="JF42" s="40"/>
       <c r="JG42" s="26"/>
       <c r="JH42" s="26"/>
       <c r="JI42" s="26"/>
@@ -5529,7 +5569,7 @@
       <c r="C43" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="KD43" s="45"/>
+      <c r="KD43" s="41"/>
     </row>
     <row r="44" spans="2:351" ht="15" customHeight="1">
       <c r="B44" s="20" t="s">
@@ -5538,7 +5578,7 @@
       <c r="C44" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="KE44" s="45"/>
+      <c r="KE44" s="41"/>
       <c r="KF44" s="26"/>
       <c r="KG44" s="26"/>
       <c r="KH44" s="26"/>
@@ -5607,7 +5647,7 @@
       <c r="C45" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="KE45" s="45"/>
+      <c r="KE45" s="41"/>
       <c r="KF45" s="26"/>
       <c r="KG45" s="26"/>
       <c r="KH45" s="26"/>
@@ -5629,7 +5669,7 @@
       <c r="C46" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="KS46" s="45"/>
+      <c r="KS46" s="41"/>
       <c r="KT46" s="26"/>
       <c r="KU46" s="26"/>
       <c r="KV46" s="26"/>
@@ -5667,7 +5707,7 @@
       <c r="C47" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="LW47" s="45"/>
+      <c r="LW47" s="41"/>
       <c r="LX47" s="26"/>
       <c r="LY47" s="26"/>
       <c r="LZ47" s="26"/>
@@ -5692,10 +5732,17 @@
       <c r="C48" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="MM48" s="45"/>
+      <c r="MM48" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="OI1:PM1"/>
+    <mergeCell ref="EY1:GB1"/>
+    <mergeCell ref="BM1:CQ1"/>
+    <mergeCell ref="AH1:BL1"/>
+    <mergeCell ref="GC1:HG1"/>
+    <mergeCell ref="LZ1:ND1"/>
+    <mergeCell ref="NE1:OH1"/>
     <mergeCell ref="D1:AG1"/>
     <mergeCell ref="IL1:JP1"/>
     <mergeCell ref="KV1:LY1"/>
@@ -5703,13 +5750,6 @@
     <mergeCell ref="HH1:IK1"/>
     <mergeCell ref="JQ1:KU1"/>
     <mergeCell ref="DT1:EX1"/>
-    <mergeCell ref="OI1:PM1"/>
-    <mergeCell ref="EY1:GB1"/>
-    <mergeCell ref="BM1:CQ1"/>
-    <mergeCell ref="AH1:BL1"/>
-    <mergeCell ref="GC1:HG1"/>
-    <mergeCell ref="LZ1:ND1"/>
-    <mergeCell ref="NE1:OH1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5717,385 +5757,402 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7DAE1D-59BF-444C-AB6B-E4987E444A19}">
-  <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6.81640625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="47" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" style="36" customWidth="1"/>
-    <col min="4" max="16384" width="8.7265625" style="36"/>
+    <col min="1" max="1" width="6.77734375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="47" style="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" style="33" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="33"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" customHeight="1">
-      <c r="A1" s="74" t="s">
+    <row r="1" spans="1:4" ht="15" customHeight="1">
+      <c r="A1" s="68" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="75"/>
-    </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1">
-      <c r="A2" s="38">
+      <c r="C1" s="69"/>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1">
+      <c r="A2" s="35">
         <v>1</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="36" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1">
-      <c r="A3" s="38">
+      <c r="D2" s="73"/>
+    </row>
+    <row r="3" spans="1:4" ht="15" customHeight="1">
+      <c r="A3" s="35">
         <v>2</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="36" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1">
-      <c r="A4" s="38"/>
-      <c r="B4" s="34" t="s">
+      <c r="D3" s="73"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" customHeight="1">
+      <c r="A4" s="35"/>
+      <c r="B4" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="39"/>
-    </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1">
-      <c r="A5" s="38">
+      <c r="C4" s="36"/>
+      <c r="D4" s="73"/>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1">
+      <c r="A5" s="35">
         <v>3</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="39"/>
-    </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1">
-      <c r="A6" s="63">
+      <c r="C5" s="36"/>
+      <c r="D5" s="73"/>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1">
+      <c r="A6" s="59">
         <v>4</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="60" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1">
-      <c r="A7" s="42">
+    <row r="7" spans="1:4" ht="15" customHeight="1">
+      <c r="A7" s="38">
         <v>5</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="43"/>
-    </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1">
-      <c r="A8" s="42">
+      <c r="C7" s="39"/>
+      <c r="D7" s="73"/>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1">
+      <c r="A8" s="38">
         <v>6</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="43"/>
-    </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1">
-      <c r="A9" s="42">
+      <c r="C8" s="39"/>
+      <c r="D8" s="73"/>
+    </row>
+    <row r="9" spans="1:4" ht="15" customHeight="1">
+      <c r="A9" s="38">
         <v>7</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="43"/>
-    </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1">
-      <c r="A10" s="42">
+      <c r="C9" s="39"/>
+      <c r="D9" s="73"/>
+    </row>
+    <row r="10" spans="1:4" ht="15" customHeight="1">
+      <c r="A10" s="38">
         <v>8</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="43"/>
-    </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1">
-      <c r="A11" s="42">
+      <c r="C10" s="39"/>
+      <c r="D10" s="73"/>
+    </row>
+    <row r="11" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A11" s="75">
         <v>9</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="43"/>
-    </row>
-    <row r="12" spans="1:3" ht="15" customHeight="1">
-      <c r="A12" s="42">
+      <c r="C11" s="77"/>
+      <c r="D11" s="73"/>
+    </row>
+    <row r="12" spans="1:4" ht="15" customHeight="1" thickTop="1">
+      <c r="A12" s="47">
         <v>10</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="43"/>
-    </row>
-    <row r="13" spans="1:3" ht="15" customHeight="1">
-      <c r="A13" s="42">
+      <c r="C12" s="49"/>
+      <c r="D12" s="73"/>
+    </row>
+    <row r="13" spans="1:4" ht="15" customHeight="1">
+      <c r="A13" s="38">
         <v>11</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="43"/>
-    </row>
-    <row r="14" spans="1:3" ht="15" customHeight="1">
-      <c r="A14" s="42">
+      <c r="C13" s="39"/>
+      <c r="D13" s="73"/>
+    </row>
+    <row r="14" spans="1:4" ht="15" customHeight="1">
+      <c r="A14" s="38">
         <v>12</v>
       </c>
       <c r="B14" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="43"/>
-    </row>
-    <row r="15" spans="1:3" ht="15" customHeight="1">
-      <c r="A15" s="42">
+      <c r="C14" s="39"/>
+      <c r="D14" s="73"/>
+    </row>
+    <row r="15" spans="1:4" ht="15" customHeight="1">
+      <c r="A15" s="38">
         <v>13</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="43"/>
-    </row>
-    <row r="16" spans="1:3" ht="15" customHeight="1">
-      <c r="A16" s="42">
+      <c r="C15" s="39"/>
+      <c r="D15" s="73"/>
+    </row>
+    <row r="16" spans="1:4" ht="15" customHeight="1">
+      <c r="A16" s="38">
         <v>14</v>
       </c>
       <c r="B16" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="43"/>
-    </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1">
-      <c r="A17" s="42">
+      <c r="C16" s="39"/>
+      <c r="D16" s="73"/>
+    </row>
+    <row r="17" spans="1:4" ht="15" customHeight="1">
+      <c r="A17" s="38">
         <v>15</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="43"/>
-    </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1">
-      <c r="A18" s="42">
+      <c r="C17" s="39"/>
+      <c r="D17" s="73"/>
+    </row>
+    <row r="18" spans="1:4" ht="15" customHeight="1">
+      <c r="A18" s="38">
         <v>16</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="43"/>
-    </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1">
-      <c r="A19" s="42">
+      <c r="C18" s="39"/>
+      <c r="D18" s="73"/>
+    </row>
+    <row r="19" spans="1:4" ht="15" customHeight="1">
+      <c r="A19" s="38">
         <v>17</v>
       </c>
       <c r="B19" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="43"/>
-    </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1">
-      <c r="A20" s="42">
+      <c r="C19" s="39"/>
+      <c r="D19" s="73"/>
+    </row>
+    <row r="20" spans="1:4" ht="15" customHeight="1">
+      <c r="A20" s="38">
         <v>18</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="43"/>
-    </row>
-    <row r="21" spans="1:3" ht="15" customHeight="1">
-      <c r="A21" s="42">
+      <c r="C20" s="39"/>
+    </row>
+    <row r="21" spans="1:4" ht="15" customHeight="1">
+      <c r="A21" s="38">
         <v>19</v>
       </c>
       <c r="B21" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="43"/>
-    </row>
-    <row r="22" spans="1:3" ht="15" customHeight="1">
-      <c r="A22" s="42">
+      <c r="C21" s="39"/>
+    </row>
+    <row r="22" spans="1:4" ht="15" customHeight="1">
+      <c r="A22" s="38">
         <v>20</v>
       </c>
       <c r="B22" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="43"/>
-    </row>
-    <row r="23" spans="1:3" ht="15" customHeight="1">
-      <c r="A23" s="42">
+      <c r="C22" s="39"/>
+    </row>
+    <row r="23" spans="1:4" ht="15" customHeight="1">
+      <c r="A23" s="38">
         <v>21</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="43"/>
-    </row>
-    <row r="24" spans="1:3" ht="15" customHeight="1">
-      <c r="A24" s="42">
+      <c r="C23" s="39"/>
+    </row>
+    <row r="24" spans="1:4" ht="15" customHeight="1">
+      <c r="A24" s="38">
         <v>22</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="43"/>
-    </row>
-    <row r="25" spans="1:3" ht="15" customHeight="1">
-      <c r="A25" s="42">
+      <c r="C24" s="39"/>
+    </row>
+    <row r="25" spans="1:4" ht="15" customHeight="1">
+      <c r="A25" s="38">
         <v>23</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="43"/>
-    </row>
-    <row r="26" spans="1:3" ht="15" customHeight="1">
-      <c r="A26" s="42">
+      <c r="C25" s="39"/>
+    </row>
+    <row r="26" spans="1:4" ht="15" customHeight="1">
+      <c r="A26" s="38">
         <v>24</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="43"/>
-    </row>
-    <row r="27" spans="1:3" ht="15" customHeight="1">
-      <c r="A27" s="42">
+      <c r="C26" s="39"/>
+    </row>
+    <row r="27" spans="1:4" ht="15" customHeight="1">
+      <c r="A27" s="38">
         <v>25</v>
       </c>
       <c r="B27" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="43"/>
-    </row>
-    <row r="28" spans="1:3" ht="15" customHeight="1">
-      <c r="A28" s="42">
+      <c r="C27" s="39"/>
+    </row>
+    <row r="28" spans="1:4" ht="15" customHeight="1">
+      <c r="A28" s="38">
         <v>26</v>
       </c>
       <c r="B28" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="43"/>
-    </row>
-    <row r="29" spans="1:3" ht="15" customHeight="1">
-      <c r="A29" s="42">
+      <c r="C28" s="39"/>
+    </row>
+    <row r="29" spans="1:4" ht="15" customHeight="1">
+      <c r="A29" s="38">
         <v>27</v>
       </c>
       <c r="B29" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="43"/>
-    </row>
-    <row r="30" spans="1:3" ht="15" customHeight="1">
-      <c r="A30" s="42">
+      <c r="C29" s="39"/>
+    </row>
+    <row r="30" spans="1:4" ht="15" customHeight="1">
+      <c r="A30" s="38">
         <v>28</v>
       </c>
       <c r="B30" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="43"/>
-    </row>
-    <row r="31" spans="1:3" ht="15" customHeight="1">
-      <c r="A31" s="48">
+      <c r="C30" s="39"/>
+    </row>
+    <row r="31" spans="1:4" ht="15" customHeight="1">
+      <c r="A31" s="44">
         <v>29</v>
       </c>
-      <c r="B31" s="49" t="s">
+      <c r="B31" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="50"/>
-    </row>
-    <row r="32" spans="1:3" ht="15" customHeight="1">
-      <c r="A32" s="61">
+      <c r="C31" s="46"/>
+    </row>
+    <row r="32" spans="1:4" ht="15" customHeight="1">
+      <c r="A32" s="57">
         <v>30</v>
       </c>
       <c r="B32" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="62" t="s">
+      <c r="C32" s="58" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" customHeight="1">
-      <c r="A33" s="51">
+      <c r="A33" s="47">
         <v>31</v>
       </c>
-      <c r="B33" s="52" t="s">
+      <c r="B33" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="53"/>
+      <c r="C33" s="49"/>
     </row>
     <row r="34" spans="1:3" ht="15" customHeight="1">
-      <c r="A34" s="42">
+      <c r="A34" s="38">
         <v>32</v>
       </c>
       <c r="B34" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="43"/>
+      <c r="C34" s="39"/>
     </row>
     <row r="35" spans="1:3" ht="15" customHeight="1">
-      <c r="A35" s="42">
+      <c r="A35" s="38">
         <v>33</v>
       </c>
       <c r="B35" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="43"/>
+      <c r="C35" s="39"/>
     </row>
     <row r="36" spans="1:3" ht="15" customHeight="1">
-      <c r="A36" s="42">
+      <c r="A36" s="38">
         <v>34</v>
       </c>
       <c r="B36" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="43"/>
+      <c r="C36" s="39"/>
     </row>
     <row r="37" spans="1:3" ht="15" customHeight="1">
-      <c r="A37" s="42">
+      <c r="A37" s="38">
         <v>35</v>
       </c>
       <c r="B37" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C37" s="43"/>
+      <c r="C37" s="39"/>
     </row>
     <row r="38" spans="1:3" ht="15" customHeight="1">
-      <c r="A38" s="59">
+      <c r="A38" s="55">
         <v>36</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="46"/>
+      <c r="C38" s="42"/>
     </row>
     <row r="39" spans="1:3" ht="15" customHeight="1">
-      <c r="A39" s="70">
+      <c r="A39" s="64">
         <v>37</v>
       </c>
-      <c r="B39" s="71" t="s">
+      <c r="B39" s="65" t="s">
         <v>83</v>
       </c>
-      <c r="C39" s="71" t="s">
+      <c r="C39" s="65" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="15" customHeight="1">
-      <c r="A40" s="56">
+      <c r="A40" s="52">
         <v>38</v>
       </c>
-      <c r="B40" s="52" t="s">
+      <c r="B40" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="C40" s="52"/>
+      <c r="C40" s="48"/>
     </row>
     <row r="41" spans="1:3" ht="15" customHeight="1">
-      <c r="A41" s="47">
+      <c r="A41" s="43">
         <v>39</v>
       </c>
       <c r="B41" s="22" t="s">
@@ -6104,7 +6161,7 @@
       <c r="C41" s="22"/>
     </row>
     <row r="42" spans="1:3" ht="15" customHeight="1">
-      <c r="A42" s="47">
+      <c r="A42" s="43">
         <v>40</v>
       </c>
       <c r="B42" s="22" t="s">
@@ -6113,13 +6170,13 @@
       <c r="C42" s="22"/>
     </row>
     <row r="43" spans="1:3" ht="15" customHeight="1">
-      <c r="A43" s="72">
+      <c r="A43" s="66">
         <v>41</v>
       </c>
-      <c r="B43" s="73" t="s">
+      <c r="B43" s="67" t="s">
         <v>91</v>
       </c>
-      <c r="C43" s="73"/>
+      <c r="C43" s="67"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6129,592 +6186,592 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:PM48"/>
-  <sheetFormatPr defaultRowHeight="10"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="10.199999999999999"/>
   <cols>
-    <col min="1" max="1" width="5.36328125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="48.1796875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="21" style="69" customWidth="1"/>
-    <col min="4" max="9" width="2.6328125" style="13" customWidth="1"/>
-    <col min="10" max="10" width="2.6328125" style="14" customWidth="1"/>
-    <col min="11" max="16" width="2.6328125" style="13" customWidth="1"/>
-    <col min="17" max="17" width="2.6328125" style="14" customWidth="1"/>
-    <col min="18" max="23" width="2.6328125" style="13" customWidth="1"/>
-    <col min="24" max="24" width="2.6328125" style="15" customWidth="1"/>
-    <col min="25" max="30" width="2.6328125" style="12" customWidth="1"/>
-    <col min="31" max="31" width="2.6328125" style="15" customWidth="1"/>
-    <col min="32" max="37" width="2.6328125" style="12" customWidth="1"/>
-    <col min="38" max="38" width="2.6328125" style="15" customWidth="1"/>
-    <col min="39" max="44" width="2.6328125" style="12" customWidth="1"/>
-    <col min="45" max="45" width="2.6328125" style="15" customWidth="1"/>
-    <col min="46" max="51" width="2.6328125" style="12" customWidth="1"/>
-    <col min="52" max="52" width="2.6328125" style="15" customWidth="1"/>
-    <col min="53" max="58" width="2.6328125" style="12" customWidth="1"/>
-    <col min="59" max="59" width="2.6328125" style="15" customWidth="1"/>
-    <col min="60" max="65" width="2.6328125" style="12" customWidth="1"/>
-    <col min="66" max="66" width="2.6328125" style="15" customWidth="1"/>
-    <col min="67" max="72" width="2.6328125" style="12" customWidth="1"/>
-    <col min="73" max="73" width="2.6328125" style="15" customWidth="1"/>
-    <col min="74" max="79" width="2.6328125" style="12" customWidth="1"/>
-    <col min="80" max="80" width="2.6328125" style="15" customWidth="1"/>
-    <col min="81" max="86" width="2.6328125" style="12" customWidth="1"/>
-    <col min="87" max="87" width="2.6328125" style="15" customWidth="1"/>
-    <col min="88" max="93" width="2.6328125" style="12" customWidth="1"/>
-    <col min="94" max="94" width="2.6328125" style="15" customWidth="1"/>
-    <col min="95" max="100" width="2.6328125" style="12" customWidth="1"/>
-    <col min="101" max="101" width="2.6328125" style="15" customWidth="1"/>
-    <col min="102" max="107" width="2.6328125" style="12" customWidth="1"/>
-    <col min="108" max="108" width="2.6328125" style="15" customWidth="1"/>
-    <col min="109" max="114" width="2.6328125" style="12" customWidth="1"/>
-    <col min="115" max="115" width="2.6328125" style="15" customWidth="1"/>
-    <col min="116" max="121" width="2.6328125" style="12" customWidth="1"/>
-    <col min="122" max="122" width="2.6328125" style="15" customWidth="1"/>
-    <col min="123" max="128" width="2.6328125" style="12" customWidth="1"/>
-    <col min="129" max="129" width="2.6328125" style="15" customWidth="1"/>
-    <col min="130" max="135" width="2.6328125" style="12" customWidth="1"/>
-    <col min="136" max="136" width="2.6328125" style="15" customWidth="1"/>
-    <col min="137" max="142" width="2.6328125" style="12" customWidth="1"/>
-    <col min="143" max="143" width="2.6328125" style="15" customWidth="1"/>
-    <col min="144" max="149" width="2.6328125" style="12" customWidth="1"/>
-    <col min="150" max="150" width="2.6328125" style="15" customWidth="1"/>
-    <col min="151" max="156" width="2.6328125" style="12" customWidth="1"/>
-    <col min="157" max="157" width="2.6328125" style="15" customWidth="1"/>
-    <col min="158" max="163" width="2.6328125" style="12" customWidth="1"/>
-    <col min="164" max="164" width="2.6328125" style="15" customWidth="1"/>
-    <col min="165" max="170" width="2.6328125" style="12" customWidth="1"/>
-    <col min="171" max="171" width="2.6328125" style="15" customWidth="1"/>
-    <col min="172" max="177" width="2.6328125" style="12" customWidth="1"/>
-    <col min="178" max="178" width="2.6328125" style="15" customWidth="1"/>
-    <col min="179" max="184" width="2.6328125" style="12" customWidth="1"/>
-    <col min="185" max="185" width="2.6328125" style="15" customWidth="1"/>
-    <col min="186" max="191" width="2.6328125" style="12" customWidth="1"/>
-    <col min="192" max="192" width="2.6328125" style="15" customWidth="1"/>
-    <col min="193" max="198" width="2.6328125" style="12" customWidth="1"/>
-    <col min="199" max="199" width="2.6328125" style="15" customWidth="1"/>
-    <col min="200" max="205" width="2.6328125" style="12" customWidth="1"/>
-    <col min="206" max="206" width="2.6328125" style="15" customWidth="1"/>
-    <col min="207" max="212" width="2.6328125" style="12" customWidth="1"/>
-    <col min="213" max="213" width="2.6328125" style="15" customWidth="1"/>
-    <col min="214" max="219" width="2.6328125" style="12" customWidth="1"/>
-    <col min="220" max="220" width="2.6328125" style="15" customWidth="1"/>
-    <col min="221" max="226" width="2.6328125" style="12" customWidth="1"/>
-    <col min="227" max="227" width="2.6328125" style="15" customWidth="1"/>
-    <col min="228" max="233" width="2.6328125" style="12" customWidth="1"/>
-    <col min="234" max="234" width="2.6328125" style="15" customWidth="1"/>
-    <col min="235" max="240" width="2.6328125" style="12" customWidth="1"/>
-    <col min="241" max="241" width="2.6328125" style="15" customWidth="1"/>
-    <col min="242" max="247" width="2.6328125" style="12" customWidth="1"/>
-    <col min="248" max="248" width="2.6328125" style="15" customWidth="1"/>
-    <col min="249" max="254" width="2.6328125" style="12" customWidth="1"/>
-    <col min="255" max="255" width="2.6328125" style="15" customWidth="1"/>
-    <col min="256" max="261" width="2.6328125" style="12" customWidth="1"/>
-    <col min="262" max="262" width="2.6328125" style="15" customWidth="1"/>
-    <col min="263" max="268" width="2.6328125" style="12" customWidth="1"/>
-    <col min="269" max="269" width="2.6328125" style="15" customWidth="1"/>
-    <col min="270" max="275" width="2.6328125" style="12" customWidth="1"/>
-    <col min="276" max="276" width="2.6328125" style="15" customWidth="1"/>
-    <col min="277" max="282" width="2.6328125" style="12" customWidth="1"/>
-    <col min="283" max="283" width="2.6328125" style="15" customWidth="1"/>
-    <col min="284" max="289" width="2.6328125" style="12" customWidth="1"/>
-    <col min="290" max="290" width="2.6328125" style="15" customWidth="1"/>
-    <col min="291" max="296" width="2.6328125" style="12" customWidth="1"/>
-    <col min="297" max="297" width="2.6328125" style="15" customWidth="1"/>
-    <col min="298" max="303" width="2.6328125" style="12" customWidth="1"/>
-    <col min="304" max="304" width="2.6328125" style="15" customWidth="1"/>
-    <col min="305" max="310" width="2.6328125" style="12" customWidth="1"/>
-    <col min="311" max="311" width="2.6328125" style="15" customWidth="1"/>
-    <col min="312" max="317" width="2.6328125" style="12" customWidth="1"/>
-    <col min="318" max="318" width="2.6328125" style="15" customWidth="1"/>
-    <col min="319" max="324" width="2.6328125" style="12" customWidth="1"/>
-    <col min="325" max="325" width="2.6328125" style="15" customWidth="1"/>
-    <col min="326" max="331" width="2.6328125" style="12" customWidth="1"/>
-    <col min="332" max="332" width="2.6328125" style="15" customWidth="1"/>
-    <col min="333" max="338" width="2.6328125" style="12" customWidth="1"/>
-    <col min="339" max="339" width="2.6328125" style="15" customWidth="1"/>
-    <col min="340" max="345" width="2.6328125" style="12" customWidth="1"/>
-    <col min="346" max="346" width="2.6328125" style="15" customWidth="1"/>
-    <col min="347" max="352" width="2.6328125" style="12" customWidth="1"/>
-    <col min="353" max="353" width="2.6328125" style="15" customWidth="1"/>
-    <col min="354" max="359" width="2.6328125" style="12" customWidth="1"/>
-    <col min="360" max="360" width="2.6328125" style="15" customWidth="1"/>
-    <col min="361" max="366" width="2.6328125" style="12" customWidth="1"/>
-    <col min="367" max="367" width="2.6328125" style="15" customWidth="1"/>
-    <col min="368" max="373" width="2.6328125" style="12" customWidth="1"/>
-    <col min="374" max="374" width="2.6328125" style="15" customWidth="1"/>
-    <col min="375" max="380" width="2.6328125" style="12" customWidth="1"/>
-    <col min="381" max="381" width="2.6328125" style="15" customWidth="1"/>
-    <col min="382" max="387" width="2.6328125" style="12" customWidth="1"/>
-    <col min="388" max="388" width="2.6328125" style="15" customWidth="1"/>
-    <col min="389" max="394" width="2.6328125" style="12" customWidth="1"/>
-    <col min="395" max="395" width="2.6328125" style="15" customWidth="1"/>
-    <col min="396" max="401" width="2.6328125" style="12" customWidth="1"/>
-    <col min="402" max="402" width="2.6328125" style="15" customWidth="1"/>
-    <col min="403" max="408" width="2.6328125" style="12" customWidth="1"/>
-    <col min="409" max="409" width="2.6328125" style="15" customWidth="1"/>
-    <col min="410" max="415" width="2.6328125" style="12" customWidth="1"/>
-    <col min="416" max="416" width="2.6328125" style="15" customWidth="1"/>
-    <col min="417" max="422" width="2.6328125" style="12" customWidth="1"/>
-    <col min="423" max="423" width="2.6328125" style="15" customWidth="1"/>
-    <col min="424" max="428" width="2.6328125" style="12" customWidth="1"/>
-    <col min="429" max="429" width="8.7265625" style="12" customWidth="1"/>
-    <col min="430" max="16384" width="8.7265625" style="12"/>
+    <col min="1" max="1" width="5.33203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="48.21875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="21" style="13" customWidth="1"/>
+    <col min="4" max="9" width="2.6640625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" style="14" customWidth="1"/>
+    <col min="11" max="16" width="2.6640625" style="13" customWidth="1"/>
+    <col min="17" max="17" width="2.6640625" style="14" customWidth="1"/>
+    <col min="18" max="23" width="2.6640625" style="13" customWidth="1"/>
+    <col min="24" max="24" width="2.6640625" style="15" customWidth="1"/>
+    <col min="25" max="30" width="2.6640625" style="12" customWidth="1"/>
+    <col min="31" max="31" width="2.6640625" style="15" customWidth="1"/>
+    <col min="32" max="37" width="2.6640625" style="12" customWidth="1"/>
+    <col min="38" max="38" width="2.6640625" style="15" customWidth="1"/>
+    <col min="39" max="44" width="2.6640625" style="12" customWidth="1"/>
+    <col min="45" max="45" width="2.6640625" style="15" customWidth="1"/>
+    <col min="46" max="51" width="2.6640625" style="12" customWidth="1"/>
+    <col min="52" max="52" width="2.6640625" style="15" customWidth="1"/>
+    <col min="53" max="58" width="2.6640625" style="12" customWidth="1"/>
+    <col min="59" max="59" width="2.6640625" style="15" customWidth="1"/>
+    <col min="60" max="65" width="2.6640625" style="12" customWidth="1"/>
+    <col min="66" max="66" width="2.6640625" style="15" customWidth="1"/>
+    <col min="67" max="72" width="2.6640625" style="12" customWidth="1"/>
+    <col min="73" max="73" width="2.6640625" style="15" customWidth="1"/>
+    <col min="74" max="79" width="2.6640625" style="12" customWidth="1"/>
+    <col min="80" max="80" width="2.6640625" style="15" customWidth="1"/>
+    <col min="81" max="86" width="2.6640625" style="12" customWidth="1"/>
+    <col min="87" max="87" width="2.6640625" style="15" customWidth="1"/>
+    <col min="88" max="93" width="2.6640625" style="12" customWidth="1"/>
+    <col min="94" max="94" width="2.6640625" style="15" customWidth="1"/>
+    <col min="95" max="100" width="2.6640625" style="12" customWidth="1"/>
+    <col min="101" max="101" width="2.6640625" style="15" customWidth="1"/>
+    <col min="102" max="107" width="2.6640625" style="12" customWidth="1"/>
+    <col min="108" max="108" width="2.6640625" style="15" customWidth="1"/>
+    <col min="109" max="114" width="2.6640625" style="12" customWidth="1"/>
+    <col min="115" max="115" width="2.6640625" style="15" customWidth="1"/>
+    <col min="116" max="121" width="2.6640625" style="12" customWidth="1"/>
+    <col min="122" max="122" width="2.6640625" style="15" customWidth="1"/>
+    <col min="123" max="128" width="2.6640625" style="12" customWidth="1"/>
+    <col min="129" max="129" width="2.6640625" style="15" customWidth="1"/>
+    <col min="130" max="135" width="2.6640625" style="12" customWidth="1"/>
+    <col min="136" max="136" width="2.6640625" style="15" customWidth="1"/>
+    <col min="137" max="142" width="2.6640625" style="12" customWidth="1"/>
+    <col min="143" max="143" width="2.6640625" style="15" customWidth="1"/>
+    <col min="144" max="149" width="2.6640625" style="12" customWidth="1"/>
+    <col min="150" max="150" width="2.6640625" style="15" customWidth="1"/>
+    <col min="151" max="156" width="2.6640625" style="12" customWidth="1"/>
+    <col min="157" max="157" width="2.6640625" style="15" customWidth="1"/>
+    <col min="158" max="163" width="2.6640625" style="12" customWidth="1"/>
+    <col min="164" max="164" width="2.6640625" style="15" customWidth="1"/>
+    <col min="165" max="170" width="2.6640625" style="12" customWidth="1"/>
+    <col min="171" max="171" width="2.6640625" style="15" customWidth="1"/>
+    <col min="172" max="177" width="2.6640625" style="12" customWidth="1"/>
+    <col min="178" max="178" width="2.6640625" style="15" customWidth="1"/>
+    <col min="179" max="184" width="2.6640625" style="12" customWidth="1"/>
+    <col min="185" max="185" width="2.6640625" style="15" customWidth="1"/>
+    <col min="186" max="191" width="2.6640625" style="12" customWidth="1"/>
+    <col min="192" max="192" width="2.6640625" style="15" customWidth="1"/>
+    <col min="193" max="198" width="2.6640625" style="12" customWidth="1"/>
+    <col min="199" max="199" width="2.6640625" style="15" customWidth="1"/>
+    <col min="200" max="205" width="2.6640625" style="12" customWidth="1"/>
+    <col min="206" max="206" width="2.6640625" style="15" customWidth="1"/>
+    <col min="207" max="212" width="2.6640625" style="12" customWidth="1"/>
+    <col min="213" max="213" width="2.6640625" style="15" customWidth="1"/>
+    <col min="214" max="219" width="2.6640625" style="12" customWidth="1"/>
+    <col min="220" max="220" width="2.6640625" style="15" customWidth="1"/>
+    <col min="221" max="226" width="2.6640625" style="12" customWidth="1"/>
+    <col min="227" max="227" width="2.6640625" style="15" customWidth="1"/>
+    <col min="228" max="233" width="2.6640625" style="12" customWidth="1"/>
+    <col min="234" max="234" width="2.6640625" style="15" customWidth="1"/>
+    <col min="235" max="240" width="2.6640625" style="12" customWidth="1"/>
+    <col min="241" max="241" width="2.6640625" style="15" customWidth="1"/>
+    <col min="242" max="247" width="2.6640625" style="12" customWidth="1"/>
+    <col min="248" max="248" width="2.6640625" style="15" customWidth="1"/>
+    <col min="249" max="254" width="2.6640625" style="12" customWidth="1"/>
+    <col min="255" max="255" width="2.6640625" style="15" customWidth="1"/>
+    <col min="256" max="261" width="2.6640625" style="12" customWidth="1"/>
+    <col min="262" max="262" width="2.6640625" style="15" customWidth="1"/>
+    <col min="263" max="268" width="2.6640625" style="12" customWidth="1"/>
+    <col min="269" max="269" width="2.6640625" style="15" customWidth="1"/>
+    <col min="270" max="275" width="2.6640625" style="12" customWidth="1"/>
+    <col min="276" max="276" width="2.6640625" style="15" customWidth="1"/>
+    <col min="277" max="282" width="2.6640625" style="12" customWidth="1"/>
+    <col min="283" max="283" width="2.6640625" style="15" customWidth="1"/>
+    <col min="284" max="289" width="2.6640625" style="12" customWidth="1"/>
+    <col min="290" max="290" width="2.6640625" style="15" customWidth="1"/>
+    <col min="291" max="296" width="2.6640625" style="12" customWidth="1"/>
+    <col min="297" max="297" width="2.6640625" style="15" customWidth="1"/>
+    <col min="298" max="303" width="2.6640625" style="12" customWidth="1"/>
+    <col min="304" max="304" width="2.6640625" style="15" customWidth="1"/>
+    <col min="305" max="310" width="2.6640625" style="12" customWidth="1"/>
+    <col min="311" max="311" width="2.6640625" style="15" customWidth="1"/>
+    <col min="312" max="317" width="2.6640625" style="12" customWidth="1"/>
+    <col min="318" max="318" width="2.6640625" style="15" customWidth="1"/>
+    <col min="319" max="324" width="2.6640625" style="12" customWidth="1"/>
+    <col min="325" max="325" width="2.6640625" style="15" customWidth="1"/>
+    <col min="326" max="331" width="2.6640625" style="12" customWidth="1"/>
+    <col min="332" max="332" width="2.6640625" style="15" customWidth="1"/>
+    <col min="333" max="338" width="2.6640625" style="12" customWidth="1"/>
+    <col min="339" max="339" width="2.6640625" style="15" customWidth="1"/>
+    <col min="340" max="345" width="2.6640625" style="12" customWidth="1"/>
+    <col min="346" max="346" width="2.6640625" style="15" customWidth="1"/>
+    <col min="347" max="352" width="2.6640625" style="12" customWidth="1"/>
+    <col min="353" max="353" width="2.6640625" style="15" customWidth="1"/>
+    <col min="354" max="359" width="2.6640625" style="12" customWidth="1"/>
+    <col min="360" max="360" width="2.6640625" style="15" customWidth="1"/>
+    <col min="361" max="366" width="2.6640625" style="12" customWidth="1"/>
+    <col min="367" max="367" width="2.6640625" style="15" customWidth="1"/>
+    <col min="368" max="373" width="2.6640625" style="12" customWidth="1"/>
+    <col min="374" max="374" width="2.6640625" style="15" customWidth="1"/>
+    <col min="375" max="380" width="2.6640625" style="12" customWidth="1"/>
+    <col min="381" max="381" width="2.6640625" style="15" customWidth="1"/>
+    <col min="382" max="387" width="2.6640625" style="12" customWidth="1"/>
+    <col min="388" max="388" width="2.6640625" style="15" customWidth="1"/>
+    <col min="389" max="394" width="2.6640625" style="12" customWidth="1"/>
+    <col min="395" max="395" width="2.6640625" style="15" customWidth="1"/>
+    <col min="396" max="401" width="2.6640625" style="12" customWidth="1"/>
+    <col min="402" max="402" width="2.6640625" style="15" customWidth="1"/>
+    <col min="403" max="408" width="2.6640625" style="12" customWidth="1"/>
+    <col min="409" max="409" width="2.6640625" style="15" customWidth="1"/>
+    <col min="410" max="415" width="2.6640625" style="12" customWidth="1"/>
+    <col min="416" max="416" width="2.6640625" style="15" customWidth="1"/>
+    <col min="417" max="422" width="2.6640625" style="12" customWidth="1"/>
+    <col min="423" max="423" width="2.6640625" style="15" customWidth="1"/>
+    <col min="424" max="428" width="2.6640625" style="12" customWidth="1"/>
+    <col min="429" max="429" width="8.77734375" style="12" customWidth="1"/>
+    <col min="430" max="16384" width="8.77734375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:429" ht="20" customHeight="1">
-      <c r="C1" s="65"/>
-      <c r="D1" s="30">
+    <row r="1" spans="2:429" ht="19.95" customHeight="1">
+      <c r="C1" s="27"/>
+      <c r="D1" s="70">
         <v>46327</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="32"/>
-      <c r="AH1" s="30">
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="71"/>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="71"/>
+      <c r="AD1" s="71"/>
+      <c r="AE1" s="71"/>
+      <c r="AF1" s="71"/>
+      <c r="AG1" s="72"/>
+      <c r="AH1" s="70">
         <v>46357</v>
       </c>
-      <c r="AI1" s="31"/>
-      <c r="AJ1" s="31"/>
-      <c r="AK1" s="31"/>
-      <c r="AL1" s="31"/>
-      <c r="AM1" s="31"/>
-      <c r="AN1" s="31"/>
-      <c r="AO1" s="31"/>
-      <c r="AP1" s="31"/>
-      <c r="AQ1" s="31"/>
-      <c r="AR1" s="31"/>
-      <c r="AS1" s="31"/>
-      <c r="AT1" s="31"/>
-      <c r="AU1" s="31"/>
-      <c r="AV1" s="31"/>
-      <c r="AW1" s="31"/>
-      <c r="AX1" s="31"/>
-      <c r="AY1" s="31"/>
-      <c r="AZ1" s="31"/>
-      <c r="BA1" s="31"/>
-      <c r="BB1" s="31"/>
-      <c r="BC1" s="31"/>
-      <c r="BD1" s="31"/>
-      <c r="BE1" s="31"/>
-      <c r="BF1" s="31"/>
-      <c r="BG1" s="31"/>
-      <c r="BH1" s="31"/>
-      <c r="BI1" s="31"/>
-      <c r="BJ1" s="31"/>
-      <c r="BK1" s="31"/>
-      <c r="BL1" s="32"/>
-      <c r="BM1" s="30">
+      <c r="AI1" s="71"/>
+      <c r="AJ1" s="71"/>
+      <c r="AK1" s="71"/>
+      <c r="AL1" s="71"/>
+      <c r="AM1" s="71"/>
+      <c r="AN1" s="71"/>
+      <c r="AO1" s="71"/>
+      <c r="AP1" s="71"/>
+      <c r="AQ1" s="71"/>
+      <c r="AR1" s="71"/>
+      <c r="AS1" s="71"/>
+      <c r="AT1" s="71"/>
+      <c r="AU1" s="71"/>
+      <c r="AV1" s="71"/>
+      <c r="AW1" s="71"/>
+      <c r="AX1" s="71"/>
+      <c r="AY1" s="71"/>
+      <c r="AZ1" s="71"/>
+      <c r="BA1" s="71"/>
+      <c r="BB1" s="71"/>
+      <c r="BC1" s="71"/>
+      <c r="BD1" s="71"/>
+      <c r="BE1" s="71"/>
+      <c r="BF1" s="71"/>
+      <c r="BG1" s="71"/>
+      <c r="BH1" s="71"/>
+      <c r="BI1" s="71"/>
+      <c r="BJ1" s="71"/>
+      <c r="BK1" s="71"/>
+      <c r="BL1" s="72"/>
+      <c r="BM1" s="70">
         <v>46388</v>
       </c>
-      <c r="BN1" s="31"/>
-      <c r="BO1" s="31"/>
-      <c r="BP1" s="31"/>
-      <c r="BQ1" s="31"/>
-      <c r="BR1" s="31"/>
-      <c r="BS1" s="31"/>
-      <c r="BT1" s="31"/>
-      <c r="BU1" s="31"/>
-      <c r="BV1" s="31"/>
-      <c r="BW1" s="31"/>
-      <c r="BX1" s="31"/>
-      <c r="BY1" s="31"/>
-      <c r="BZ1" s="31"/>
-      <c r="CA1" s="31"/>
-      <c r="CB1" s="31"/>
-      <c r="CC1" s="31"/>
-      <c r="CD1" s="31"/>
-      <c r="CE1" s="31"/>
-      <c r="CF1" s="31"/>
-      <c r="CG1" s="31"/>
-      <c r="CH1" s="31"/>
-      <c r="CI1" s="31"/>
-      <c r="CJ1" s="31"/>
-      <c r="CK1" s="31"/>
-      <c r="CL1" s="31"/>
-      <c r="CM1" s="31"/>
-      <c r="CN1" s="31"/>
-      <c r="CO1" s="31"/>
-      <c r="CP1" s="31"/>
-      <c r="CQ1" s="32"/>
-      <c r="CR1" s="30">
+      <c r="BN1" s="71"/>
+      <c r="BO1" s="71"/>
+      <c r="BP1" s="71"/>
+      <c r="BQ1" s="71"/>
+      <c r="BR1" s="71"/>
+      <c r="BS1" s="71"/>
+      <c r="BT1" s="71"/>
+      <c r="BU1" s="71"/>
+      <c r="BV1" s="71"/>
+      <c r="BW1" s="71"/>
+      <c r="BX1" s="71"/>
+      <c r="BY1" s="71"/>
+      <c r="BZ1" s="71"/>
+      <c r="CA1" s="71"/>
+      <c r="CB1" s="71"/>
+      <c r="CC1" s="71"/>
+      <c r="CD1" s="71"/>
+      <c r="CE1" s="71"/>
+      <c r="CF1" s="71"/>
+      <c r="CG1" s="71"/>
+      <c r="CH1" s="71"/>
+      <c r="CI1" s="71"/>
+      <c r="CJ1" s="71"/>
+      <c r="CK1" s="71"/>
+      <c r="CL1" s="71"/>
+      <c r="CM1" s="71"/>
+      <c r="CN1" s="71"/>
+      <c r="CO1" s="71"/>
+      <c r="CP1" s="71"/>
+      <c r="CQ1" s="72"/>
+      <c r="CR1" s="70">
         <v>46419</v>
       </c>
-      <c r="CS1" s="31"/>
-      <c r="CT1" s="31"/>
-      <c r="CU1" s="31"/>
-      <c r="CV1" s="31"/>
-      <c r="CW1" s="31"/>
-      <c r="CX1" s="31"/>
-      <c r="CY1" s="31"/>
-      <c r="CZ1" s="31"/>
-      <c r="DA1" s="31"/>
-      <c r="DB1" s="31"/>
-      <c r="DC1" s="31"/>
-      <c r="DD1" s="31"/>
-      <c r="DE1" s="31"/>
-      <c r="DF1" s="31"/>
-      <c r="DG1" s="31"/>
-      <c r="DH1" s="31"/>
-      <c r="DI1" s="31"/>
-      <c r="DJ1" s="31"/>
-      <c r="DK1" s="31"/>
-      <c r="DL1" s="31"/>
-      <c r="DM1" s="31"/>
-      <c r="DN1" s="31"/>
-      <c r="DO1" s="31"/>
-      <c r="DP1" s="31"/>
-      <c r="DQ1" s="31"/>
-      <c r="DR1" s="31"/>
-      <c r="DS1" s="32"/>
-      <c r="DT1" s="30">
+      <c r="CS1" s="71"/>
+      <c r="CT1" s="71"/>
+      <c r="CU1" s="71"/>
+      <c r="CV1" s="71"/>
+      <c r="CW1" s="71"/>
+      <c r="CX1" s="71"/>
+      <c r="CY1" s="71"/>
+      <c r="CZ1" s="71"/>
+      <c r="DA1" s="71"/>
+      <c r="DB1" s="71"/>
+      <c r="DC1" s="71"/>
+      <c r="DD1" s="71"/>
+      <c r="DE1" s="71"/>
+      <c r="DF1" s="71"/>
+      <c r="DG1" s="71"/>
+      <c r="DH1" s="71"/>
+      <c r="DI1" s="71"/>
+      <c r="DJ1" s="71"/>
+      <c r="DK1" s="71"/>
+      <c r="DL1" s="71"/>
+      <c r="DM1" s="71"/>
+      <c r="DN1" s="71"/>
+      <c r="DO1" s="71"/>
+      <c r="DP1" s="71"/>
+      <c r="DQ1" s="71"/>
+      <c r="DR1" s="71"/>
+      <c r="DS1" s="72"/>
+      <c r="DT1" s="70">
         <v>46447</v>
       </c>
-      <c r="DU1" s="31"/>
-      <c r="DV1" s="31"/>
-      <c r="DW1" s="31"/>
-      <c r="DX1" s="31"/>
-      <c r="DY1" s="31"/>
-      <c r="DZ1" s="31"/>
-      <c r="EA1" s="31"/>
-      <c r="EB1" s="31"/>
-      <c r="EC1" s="31"/>
-      <c r="ED1" s="31"/>
-      <c r="EE1" s="31"/>
-      <c r="EF1" s="31"/>
-      <c r="EG1" s="31"/>
-      <c r="EH1" s="31"/>
-      <c r="EI1" s="31"/>
-      <c r="EJ1" s="31"/>
-      <c r="EK1" s="31"/>
-      <c r="EL1" s="31"/>
-      <c r="EM1" s="31"/>
-      <c r="EN1" s="31"/>
-      <c r="EO1" s="31"/>
-      <c r="EP1" s="31"/>
-      <c r="EQ1" s="31"/>
-      <c r="ER1" s="31"/>
-      <c r="ES1" s="31"/>
-      <c r="ET1" s="31"/>
-      <c r="EU1" s="31"/>
-      <c r="EV1" s="31"/>
-      <c r="EW1" s="31"/>
-      <c r="EX1" s="32"/>
-      <c r="EY1" s="30">
+      <c r="DU1" s="71"/>
+      <c r="DV1" s="71"/>
+      <c r="DW1" s="71"/>
+      <c r="DX1" s="71"/>
+      <c r="DY1" s="71"/>
+      <c r="DZ1" s="71"/>
+      <c r="EA1" s="71"/>
+      <c r="EB1" s="71"/>
+      <c r="EC1" s="71"/>
+      <c r="ED1" s="71"/>
+      <c r="EE1" s="71"/>
+      <c r="EF1" s="71"/>
+      <c r="EG1" s="71"/>
+      <c r="EH1" s="71"/>
+      <c r="EI1" s="71"/>
+      <c r="EJ1" s="71"/>
+      <c r="EK1" s="71"/>
+      <c r="EL1" s="71"/>
+      <c r="EM1" s="71"/>
+      <c r="EN1" s="71"/>
+      <c r="EO1" s="71"/>
+      <c r="EP1" s="71"/>
+      <c r="EQ1" s="71"/>
+      <c r="ER1" s="71"/>
+      <c r="ES1" s="71"/>
+      <c r="ET1" s="71"/>
+      <c r="EU1" s="71"/>
+      <c r="EV1" s="71"/>
+      <c r="EW1" s="71"/>
+      <c r="EX1" s="72"/>
+      <c r="EY1" s="70">
         <v>46478</v>
       </c>
-      <c r="EZ1" s="31"/>
-      <c r="FA1" s="31"/>
-      <c r="FB1" s="31"/>
-      <c r="FC1" s="31"/>
-      <c r="FD1" s="31"/>
-      <c r="FE1" s="31"/>
-      <c r="FF1" s="31"/>
-      <c r="FG1" s="31"/>
-      <c r="FH1" s="31"/>
-      <c r="FI1" s="31"/>
-      <c r="FJ1" s="31"/>
-      <c r="FK1" s="31"/>
-      <c r="FL1" s="31"/>
-      <c r="FM1" s="31"/>
-      <c r="FN1" s="31"/>
-      <c r="FO1" s="31"/>
-      <c r="FP1" s="31"/>
-      <c r="FQ1" s="31"/>
-      <c r="FR1" s="31"/>
-      <c r="FS1" s="31"/>
-      <c r="FT1" s="31"/>
-      <c r="FU1" s="31"/>
-      <c r="FV1" s="31"/>
-      <c r="FW1" s="31"/>
-      <c r="FX1" s="31"/>
-      <c r="FY1" s="31"/>
-      <c r="FZ1" s="31"/>
-      <c r="GA1" s="31"/>
-      <c r="GB1" s="32"/>
-      <c r="GC1" s="30">
+      <c r="EZ1" s="71"/>
+      <c r="FA1" s="71"/>
+      <c r="FB1" s="71"/>
+      <c r="FC1" s="71"/>
+      <c r="FD1" s="71"/>
+      <c r="FE1" s="71"/>
+      <c r="FF1" s="71"/>
+      <c r="FG1" s="71"/>
+      <c r="FH1" s="71"/>
+      <c r="FI1" s="71"/>
+      <c r="FJ1" s="71"/>
+      <c r="FK1" s="71"/>
+      <c r="FL1" s="71"/>
+      <c r="FM1" s="71"/>
+      <c r="FN1" s="71"/>
+      <c r="FO1" s="71"/>
+      <c r="FP1" s="71"/>
+      <c r="FQ1" s="71"/>
+      <c r="FR1" s="71"/>
+      <c r="FS1" s="71"/>
+      <c r="FT1" s="71"/>
+      <c r="FU1" s="71"/>
+      <c r="FV1" s="71"/>
+      <c r="FW1" s="71"/>
+      <c r="FX1" s="71"/>
+      <c r="FY1" s="71"/>
+      <c r="FZ1" s="71"/>
+      <c r="GA1" s="71"/>
+      <c r="GB1" s="72"/>
+      <c r="GC1" s="70">
         <v>46508</v>
       </c>
-      <c r="GD1" s="31"/>
-      <c r="GE1" s="31"/>
-      <c r="GF1" s="31"/>
-      <c r="GG1" s="31"/>
-      <c r="GH1" s="31"/>
-      <c r="GI1" s="31"/>
-      <c r="GJ1" s="31"/>
-      <c r="GK1" s="31"/>
-      <c r="GL1" s="31"/>
-      <c r="GM1" s="31"/>
-      <c r="GN1" s="31"/>
-      <c r="GO1" s="31"/>
-      <c r="GP1" s="31"/>
-      <c r="GQ1" s="31"/>
-      <c r="GR1" s="31"/>
-      <c r="GS1" s="31"/>
-      <c r="GT1" s="31"/>
-      <c r="GU1" s="31"/>
-      <c r="GV1" s="31"/>
-      <c r="GW1" s="31"/>
-      <c r="GX1" s="31"/>
-      <c r="GY1" s="31"/>
-      <c r="GZ1" s="31"/>
-      <c r="HA1" s="31"/>
-      <c r="HB1" s="31"/>
-      <c r="HC1" s="31"/>
-      <c r="HD1" s="31"/>
-      <c r="HE1" s="31"/>
-      <c r="HF1" s="31"/>
-      <c r="HG1" s="32"/>
-      <c r="HH1" s="30">
+      <c r="GD1" s="71"/>
+      <c r="GE1" s="71"/>
+      <c r="GF1" s="71"/>
+      <c r="GG1" s="71"/>
+      <c r="GH1" s="71"/>
+      <c r="GI1" s="71"/>
+      <c r="GJ1" s="71"/>
+      <c r="GK1" s="71"/>
+      <c r="GL1" s="71"/>
+      <c r="GM1" s="71"/>
+      <c r="GN1" s="71"/>
+      <c r="GO1" s="71"/>
+      <c r="GP1" s="71"/>
+      <c r="GQ1" s="71"/>
+      <c r="GR1" s="71"/>
+      <c r="GS1" s="71"/>
+      <c r="GT1" s="71"/>
+      <c r="GU1" s="71"/>
+      <c r="GV1" s="71"/>
+      <c r="GW1" s="71"/>
+      <c r="GX1" s="71"/>
+      <c r="GY1" s="71"/>
+      <c r="GZ1" s="71"/>
+      <c r="HA1" s="71"/>
+      <c r="HB1" s="71"/>
+      <c r="HC1" s="71"/>
+      <c r="HD1" s="71"/>
+      <c r="HE1" s="71"/>
+      <c r="HF1" s="71"/>
+      <c r="HG1" s="72"/>
+      <c r="HH1" s="70">
         <v>46539</v>
       </c>
-      <c r="HI1" s="31"/>
-      <c r="HJ1" s="31"/>
-      <c r="HK1" s="31"/>
-      <c r="HL1" s="31"/>
-      <c r="HM1" s="31"/>
-      <c r="HN1" s="31"/>
-      <c r="HO1" s="31"/>
-      <c r="HP1" s="31"/>
-      <c r="HQ1" s="31"/>
-      <c r="HR1" s="31"/>
-      <c r="HS1" s="31"/>
-      <c r="HT1" s="31"/>
-      <c r="HU1" s="31"/>
-      <c r="HV1" s="31"/>
-      <c r="HW1" s="31"/>
-      <c r="HX1" s="31"/>
-      <c r="HY1" s="31"/>
-      <c r="HZ1" s="31"/>
-      <c r="IA1" s="31"/>
-      <c r="IB1" s="31"/>
-      <c r="IC1" s="31"/>
-      <c r="ID1" s="31"/>
-      <c r="IE1" s="31"/>
-      <c r="IF1" s="31"/>
-      <c r="IG1" s="31"/>
-      <c r="IH1" s="31"/>
-      <c r="II1" s="31"/>
-      <c r="IJ1" s="31"/>
-      <c r="IK1" s="32"/>
-      <c r="IL1" s="30">
+      <c r="HI1" s="71"/>
+      <c r="HJ1" s="71"/>
+      <c r="HK1" s="71"/>
+      <c r="HL1" s="71"/>
+      <c r="HM1" s="71"/>
+      <c r="HN1" s="71"/>
+      <c r="HO1" s="71"/>
+      <c r="HP1" s="71"/>
+      <c r="HQ1" s="71"/>
+      <c r="HR1" s="71"/>
+      <c r="HS1" s="71"/>
+      <c r="HT1" s="71"/>
+      <c r="HU1" s="71"/>
+      <c r="HV1" s="71"/>
+      <c r="HW1" s="71"/>
+      <c r="HX1" s="71"/>
+      <c r="HY1" s="71"/>
+      <c r="HZ1" s="71"/>
+      <c r="IA1" s="71"/>
+      <c r="IB1" s="71"/>
+      <c r="IC1" s="71"/>
+      <c r="ID1" s="71"/>
+      <c r="IE1" s="71"/>
+      <c r="IF1" s="71"/>
+      <c r="IG1" s="71"/>
+      <c r="IH1" s="71"/>
+      <c r="II1" s="71"/>
+      <c r="IJ1" s="71"/>
+      <c r="IK1" s="72"/>
+      <c r="IL1" s="70">
         <v>46569</v>
       </c>
-      <c r="IM1" s="31"/>
-      <c r="IN1" s="31"/>
-      <c r="IO1" s="31"/>
-      <c r="IP1" s="31"/>
-      <c r="IQ1" s="31"/>
-      <c r="IR1" s="31"/>
-      <c r="IS1" s="31"/>
-      <c r="IT1" s="31"/>
-      <c r="IU1" s="31"/>
-      <c r="IV1" s="31"/>
-      <c r="IW1" s="31"/>
-      <c r="IX1" s="31"/>
-      <c r="IY1" s="31"/>
-      <c r="IZ1" s="31"/>
-      <c r="JA1" s="31"/>
-      <c r="JB1" s="31"/>
-      <c r="JC1" s="31"/>
-      <c r="JD1" s="31"/>
-      <c r="JE1" s="31"/>
-      <c r="JF1" s="31"/>
-      <c r="JG1" s="31"/>
-      <c r="JH1" s="31"/>
-      <c r="JI1" s="31"/>
-      <c r="JJ1" s="31"/>
-      <c r="JK1" s="31"/>
-      <c r="JL1" s="31"/>
-      <c r="JM1" s="31"/>
-      <c r="JN1" s="31"/>
-      <c r="JO1" s="31"/>
-      <c r="JP1" s="32"/>
-      <c r="JQ1" s="30">
+      <c r="IM1" s="71"/>
+      <c r="IN1" s="71"/>
+      <c r="IO1" s="71"/>
+      <c r="IP1" s="71"/>
+      <c r="IQ1" s="71"/>
+      <c r="IR1" s="71"/>
+      <c r="IS1" s="71"/>
+      <c r="IT1" s="71"/>
+      <c r="IU1" s="71"/>
+      <c r="IV1" s="71"/>
+      <c r="IW1" s="71"/>
+      <c r="IX1" s="71"/>
+      <c r="IY1" s="71"/>
+      <c r="IZ1" s="71"/>
+      <c r="JA1" s="71"/>
+      <c r="JB1" s="71"/>
+      <c r="JC1" s="71"/>
+      <c r="JD1" s="71"/>
+      <c r="JE1" s="71"/>
+      <c r="JF1" s="71"/>
+      <c r="JG1" s="71"/>
+      <c r="JH1" s="71"/>
+      <c r="JI1" s="71"/>
+      <c r="JJ1" s="71"/>
+      <c r="JK1" s="71"/>
+      <c r="JL1" s="71"/>
+      <c r="JM1" s="71"/>
+      <c r="JN1" s="71"/>
+      <c r="JO1" s="71"/>
+      <c r="JP1" s="72"/>
+      <c r="JQ1" s="70">
         <v>46600</v>
       </c>
-      <c r="JR1" s="31"/>
-      <c r="JS1" s="31"/>
-      <c r="JT1" s="31"/>
-      <c r="JU1" s="31"/>
-      <c r="JV1" s="31"/>
-      <c r="JW1" s="31"/>
-      <c r="JX1" s="31"/>
-      <c r="JY1" s="31"/>
-      <c r="JZ1" s="31"/>
-      <c r="KA1" s="31"/>
-      <c r="KB1" s="31"/>
-      <c r="KC1" s="31"/>
-      <c r="KD1" s="31"/>
-      <c r="KE1" s="31"/>
-      <c r="KF1" s="31"/>
-      <c r="KG1" s="31"/>
-      <c r="KH1" s="31"/>
-      <c r="KI1" s="31"/>
-      <c r="KJ1" s="31"/>
-      <c r="KK1" s="31"/>
-      <c r="KL1" s="31"/>
-      <c r="KM1" s="31"/>
-      <c r="KN1" s="31"/>
-      <c r="KO1" s="31"/>
-      <c r="KP1" s="31"/>
-      <c r="KQ1" s="31"/>
-      <c r="KR1" s="31"/>
-      <c r="KS1" s="31"/>
-      <c r="KT1" s="31"/>
-      <c r="KU1" s="32"/>
-      <c r="KV1" s="30">
+      <c r="JR1" s="71"/>
+      <c r="JS1" s="71"/>
+      <c r="JT1" s="71"/>
+      <c r="JU1" s="71"/>
+      <c r="JV1" s="71"/>
+      <c r="JW1" s="71"/>
+      <c r="JX1" s="71"/>
+      <c r="JY1" s="71"/>
+      <c r="JZ1" s="71"/>
+      <c r="KA1" s="71"/>
+      <c r="KB1" s="71"/>
+      <c r="KC1" s="71"/>
+      <c r="KD1" s="71"/>
+      <c r="KE1" s="71"/>
+      <c r="KF1" s="71"/>
+      <c r="KG1" s="71"/>
+      <c r="KH1" s="71"/>
+      <c r="KI1" s="71"/>
+      <c r="KJ1" s="71"/>
+      <c r="KK1" s="71"/>
+      <c r="KL1" s="71"/>
+      <c r="KM1" s="71"/>
+      <c r="KN1" s="71"/>
+      <c r="KO1" s="71"/>
+      <c r="KP1" s="71"/>
+      <c r="KQ1" s="71"/>
+      <c r="KR1" s="71"/>
+      <c r="KS1" s="71"/>
+      <c r="KT1" s="71"/>
+      <c r="KU1" s="72"/>
+      <c r="KV1" s="70">
         <v>46631</v>
       </c>
-      <c r="KW1" s="31"/>
-      <c r="KX1" s="31"/>
-      <c r="KY1" s="31"/>
-      <c r="KZ1" s="31"/>
-      <c r="LA1" s="31"/>
-      <c r="LB1" s="31"/>
-      <c r="LC1" s="31"/>
-      <c r="LD1" s="31"/>
-      <c r="LE1" s="31"/>
-      <c r="LF1" s="31"/>
-      <c r="LG1" s="31"/>
-      <c r="LH1" s="31"/>
-      <c r="LI1" s="31"/>
-      <c r="LJ1" s="31"/>
-      <c r="LK1" s="31"/>
-      <c r="LL1" s="31"/>
-      <c r="LM1" s="31"/>
-      <c r="LN1" s="31"/>
-      <c r="LO1" s="31"/>
-      <c r="LP1" s="31"/>
-      <c r="LQ1" s="31"/>
-      <c r="LR1" s="31"/>
-      <c r="LS1" s="31"/>
-      <c r="LT1" s="31"/>
-      <c r="LU1" s="31"/>
-      <c r="LV1" s="31"/>
-      <c r="LW1" s="31"/>
-      <c r="LX1" s="31"/>
-      <c r="LY1" s="32"/>
-      <c r="LZ1" s="30">
+      <c r="KW1" s="71"/>
+      <c r="KX1" s="71"/>
+      <c r="KY1" s="71"/>
+      <c r="KZ1" s="71"/>
+      <c r="LA1" s="71"/>
+      <c r="LB1" s="71"/>
+      <c r="LC1" s="71"/>
+      <c r="LD1" s="71"/>
+      <c r="LE1" s="71"/>
+      <c r="LF1" s="71"/>
+      <c r="LG1" s="71"/>
+      <c r="LH1" s="71"/>
+      <c r="LI1" s="71"/>
+      <c r="LJ1" s="71"/>
+      <c r="LK1" s="71"/>
+      <c r="LL1" s="71"/>
+      <c r="LM1" s="71"/>
+      <c r="LN1" s="71"/>
+      <c r="LO1" s="71"/>
+      <c r="LP1" s="71"/>
+      <c r="LQ1" s="71"/>
+      <c r="LR1" s="71"/>
+      <c r="LS1" s="71"/>
+      <c r="LT1" s="71"/>
+      <c r="LU1" s="71"/>
+      <c r="LV1" s="71"/>
+      <c r="LW1" s="71"/>
+      <c r="LX1" s="71"/>
+      <c r="LY1" s="72"/>
+      <c r="LZ1" s="70">
         <v>46661</v>
       </c>
-      <c r="MA1" s="31"/>
-      <c r="MB1" s="31"/>
-      <c r="MC1" s="31"/>
-      <c r="MD1" s="31"/>
-      <c r="ME1" s="31"/>
-      <c r="MF1" s="31"/>
-      <c r="MG1" s="31"/>
-      <c r="MH1" s="31"/>
-      <c r="MI1" s="31"/>
-      <c r="MJ1" s="31"/>
-      <c r="MK1" s="31"/>
-      <c r="ML1" s="31"/>
-      <c r="MM1" s="31"/>
-      <c r="MN1" s="31"/>
-      <c r="MO1" s="31"/>
-      <c r="MP1" s="31"/>
-      <c r="MQ1" s="31"/>
-      <c r="MR1" s="31"/>
-      <c r="MS1" s="31"/>
-      <c r="MT1" s="31"/>
-      <c r="MU1" s="31"/>
-      <c r="MV1" s="31"/>
-      <c r="MW1" s="31"/>
-      <c r="MX1" s="31"/>
-      <c r="MY1" s="31"/>
-      <c r="MZ1" s="31"/>
-      <c r="NA1" s="31"/>
-      <c r="NB1" s="31"/>
-      <c r="NC1" s="31"/>
-      <c r="ND1" s="32"/>
-      <c r="NE1" s="30">
+      <c r="MA1" s="71"/>
+      <c r="MB1" s="71"/>
+      <c r="MC1" s="71"/>
+      <c r="MD1" s="71"/>
+      <c r="ME1" s="71"/>
+      <c r="MF1" s="71"/>
+      <c r="MG1" s="71"/>
+      <c r="MH1" s="71"/>
+      <c r="MI1" s="71"/>
+      <c r="MJ1" s="71"/>
+      <c r="MK1" s="71"/>
+      <c r="ML1" s="71"/>
+      <c r="MM1" s="71"/>
+      <c r="MN1" s="71"/>
+      <c r="MO1" s="71"/>
+      <c r="MP1" s="71"/>
+      <c r="MQ1" s="71"/>
+      <c r="MR1" s="71"/>
+      <c r="MS1" s="71"/>
+      <c r="MT1" s="71"/>
+      <c r="MU1" s="71"/>
+      <c r="MV1" s="71"/>
+      <c r="MW1" s="71"/>
+      <c r="MX1" s="71"/>
+      <c r="MY1" s="71"/>
+      <c r="MZ1" s="71"/>
+      <c r="NA1" s="71"/>
+      <c r="NB1" s="71"/>
+      <c r="NC1" s="71"/>
+      <c r="ND1" s="72"/>
+      <c r="NE1" s="70">
         <v>46692</v>
       </c>
-      <c r="NF1" s="31"/>
-      <c r="NG1" s="31"/>
-      <c r="NH1" s="31"/>
-      <c r="NI1" s="31"/>
-      <c r="NJ1" s="31"/>
-      <c r="NK1" s="31"/>
-      <c r="NL1" s="31"/>
-      <c r="NM1" s="31"/>
-      <c r="NN1" s="31"/>
-      <c r="NO1" s="31"/>
-      <c r="NP1" s="31"/>
-      <c r="NQ1" s="31"/>
-      <c r="NR1" s="31"/>
-      <c r="NS1" s="31"/>
-      <c r="NT1" s="31"/>
-      <c r="NU1" s="31"/>
-      <c r="NV1" s="31"/>
-      <c r="NW1" s="31"/>
-      <c r="NX1" s="31"/>
-      <c r="NY1" s="31"/>
-      <c r="NZ1" s="31"/>
-      <c r="OA1" s="31"/>
-      <c r="OB1" s="31"/>
-      <c r="OC1" s="31"/>
-      <c r="OD1" s="31"/>
-      <c r="OE1" s="31"/>
-      <c r="OF1" s="31"/>
-      <c r="OG1" s="31"/>
-      <c r="OH1" s="32"/>
-      <c r="OI1" s="30">
+      <c r="NF1" s="71"/>
+      <c r="NG1" s="71"/>
+      <c r="NH1" s="71"/>
+      <c r="NI1" s="71"/>
+      <c r="NJ1" s="71"/>
+      <c r="NK1" s="71"/>
+      <c r="NL1" s="71"/>
+      <c r="NM1" s="71"/>
+      <c r="NN1" s="71"/>
+      <c r="NO1" s="71"/>
+      <c r="NP1" s="71"/>
+      <c r="NQ1" s="71"/>
+      <c r="NR1" s="71"/>
+      <c r="NS1" s="71"/>
+      <c r="NT1" s="71"/>
+      <c r="NU1" s="71"/>
+      <c r="NV1" s="71"/>
+      <c r="NW1" s="71"/>
+      <c r="NX1" s="71"/>
+      <c r="NY1" s="71"/>
+      <c r="NZ1" s="71"/>
+      <c r="OA1" s="71"/>
+      <c r="OB1" s="71"/>
+      <c r="OC1" s="71"/>
+      <c r="OD1" s="71"/>
+      <c r="OE1" s="71"/>
+      <c r="OF1" s="71"/>
+      <c r="OG1" s="71"/>
+      <c r="OH1" s="72"/>
+      <c r="OI1" s="70">
         <v>46722</v>
       </c>
-      <c r="OJ1" s="31"/>
-      <c r="OK1" s="31"/>
-      <c r="OL1" s="31"/>
-      <c r="OM1" s="31"/>
-      <c r="ON1" s="31"/>
-      <c r="OO1" s="31"/>
-      <c r="OP1" s="31"/>
-      <c r="OQ1" s="31"/>
-      <c r="OR1" s="31"/>
-      <c r="OS1" s="31"/>
-      <c r="OT1" s="31"/>
-      <c r="OU1" s="31"/>
-      <c r="OV1" s="31"/>
-      <c r="OW1" s="31"/>
-      <c r="OX1" s="31"/>
-      <c r="OY1" s="31"/>
-      <c r="OZ1" s="31"/>
-      <c r="PA1" s="31"/>
-      <c r="PB1" s="31"/>
-      <c r="PC1" s="31"/>
-      <c r="PD1" s="31"/>
-      <c r="PE1" s="31"/>
-      <c r="PF1" s="31"/>
-      <c r="PG1" s="31"/>
-      <c r="PH1" s="31"/>
-      <c r="PI1" s="31"/>
-      <c r="PJ1" s="31"/>
-      <c r="PK1" s="31"/>
-      <c r="PL1" s="31"/>
-      <c r="PM1" s="32"/>
+      <c r="OJ1" s="71"/>
+      <c r="OK1" s="71"/>
+      <c r="OL1" s="71"/>
+      <c r="OM1" s="71"/>
+      <c r="ON1" s="71"/>
+      <c r="OO1" s="71"/>
+      <c r="OP1" s="71"/>
+      <c r="OQ1" s="71"/>
+      <c r="OR1" s="71"/>
+      <c r="OS1" s="71"/>
+      <c r="OT1" s="71"/>
+      <c r="OU1" s="71"/>
+      <c r="OV1" s="71"/>
+      <c r="OW1" s="71"/>
+      <c r="OX1" s="71"/>
+      <c r="OY1" s="71"/>
+      <c r="OZ1" s="71"/>
+      <c r="PA1" s="71"/>
+      <c r="PB1" s="71"/>
+      <c r="PC1" s="71"/>
+      <c r="PD1" s="71"/>
+      <c r="PE1" s="71"/>
+      <c r="PF1" s="71"/>
+      <c r="PG1" s="71"/>
+      <c r="PH1" s="71"/>
+      <c r="PI1" s="71"/>
+      <c r="PJ1" s="71"/>
+      <c r="PK1" s="71"/>
+      <c r="PL1" s="71"/>
+      <c r="PM1" s="72"/>
     </row>
     <row r="2" spans="2:429" ht="10.5" customHeight="1">
       <c r="B2" s="25" t="s">
@@ -8339,7 +8396,7 @@
       <c r="B4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="61" t="s">
         <v>121</v>
       </c>
       <c r="BF4" s="28"/>
@@ -8550,7 +8607,7 @@
       <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="61" t="s">
         <v>122</v>
       </c>
       <c r="CI5" s="28"/>
@@ -8570,7 +8627,7 @@
       <c r="B6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="61" t="s">
         <v>123</v>
       </c>
       <c r="CY6" s="28"/>
@@ -8586,7 +8643,7 @@
       <c r="B7" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="66" t="s">
+      <c r="C7" s="61" t="s">
         <v>124</v>
       </c>
       <c r="BF7" s="28"/>
@@ -8612,7 +8669,7 @@
       <c r="B8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="61" t="s">
         <v>125</v>
       </c>
       <c r="DF8" s="27"/>
@@ -8624,7 +8681,7 @@
       <c r="B9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="66" t="s">
+      <c r="C9" s="61" t="s">
         <v>126</v>
       </c>
       <c r="DJ9" s="28"/>
@@ -8640,7 +8697,7 @@
       <c r="B10" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="66" t="s">
+      <c r="C10" s="61" t="s">
         <v>127</v>
       </c>
       <c r="EB10" s="28"/>
@@ -8659,7 +8716,7 @@
       <c r="B11" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="66" t="s">
+      <c r="C11" s="61" t="s">
         <v>19</v>
       </c>
       <c r="CS11" s="28"/>
@@ -8674,7 +8731,7 @@
       <c r="B12" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="66" t="s">
+      <c r="C12" s="61" t="s">
         <v>128</v>
       </c>
       <c r="EM12" s="28"/>
@@ -8706,7 +8763,7 @@
       <c r="B13" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="66" t="s">
+      <c r="C13" s="61" t="s">
         <v>129</v>
       </c>
       <c r="FK13" s="28"/>
@@ -8728,7 +8785,7 @@
       <c r="B14" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="66" t="s">
+      <c r="C14" s="61" t="s">
         <v>130</v>
       </c>
       <c r="DJ14" s="28"/>
@@ -8841,7 +8898,7 @@
       <c r="B15" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="66" t="s">
+      <c r="C15" s="61" t="s">
         <v>131</v>
       </c>
       <c r="DJ15" s="28"/>
@@ -8884,7 +8941,7 @@
       <c r="B16" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="66" t="s">
+      <c r="C16" s="61" t="s">
         <v>132</v>
       </c>
       <c r="EF16" s="28"/>
@@ -8900,7 +8957,7 @@
       <c r="B17" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="66" t="s">
+      <c r="C17" s="61" t="s">
         <v>133</v>
       </c>
       <c r="EF17" s="28"/>
@@ -8943,7 +9000,7 @@
       <c r="B18" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="66" t="s">
+      <c r="C18" s="61" t="s">
         <v>134</v>
       </c>
       <c r="CU18" s="28"/>
@@ -9092,7 +9149,7 @@
       <c r="B19" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="67" t="s">
+      <c r="C19" s="62" t="s">
         <v>135</v>
       </c>
       <c r="CU19" s="28"/>
@@ -9121,7 +9178,7 @@
       <c r="B20" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="62" t="s">
         <v>136</v>
       </c>
       <c r="IC20" s="28"/>
@@ -9132,7 +9189,7 @@
       <c r="B21" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="66" t="s">
+      <c r="C21" s="61" t="s">
         <v>137</v>
       </c>
       <c r="FK21" s="28"/>
@@ -9151,7 +9208,7 @@
       <c r="B22" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="66" t="s">
+      <c r="C22" s="61" t="s">
         <v>138</v>
       </c>
       <c r="EY22" s="28"/>
@@ -9179,7 +9236,7 @@
       <c r="B23" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="66" t="s">
+      <c r="C23" s="61" t="s">
         <v>129</v>
       </c>
       <c r="FK23" s="28"/>
@@ -9201,7 +9258,7 @@
       <c r="B24" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="66" t="s">
+      <c r="C24" s="61" t="s">
         <v>139</v>
       </c>
       <c r="FO24" s="28"/>
@@ -9220,7 +9277,7 @@
       <c r="B25" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="66" t="s">
+      <c r="C25" s="61" t="s">
         <v>140</v>
       </c>
       <c r="FZ25" s="28"/>
@@ -9236,7 +9293,7 @@
       <c r="B26" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="66" t="s">
+      <c r="C26" s="61" t="s">
         <v>141</v>
       </c>
       <c r="GT26" s="28"/>
@@ -9261,7 +9318,7 @@
       <c r="B27" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="66" t="s">
+      <c r="C27" s="61" t="s">
         <v>142</v>
       </c>
       <c r="HK27" s="28"/>
@@ -9277,7 +9334,7 @@
       <c r="B28" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="66" t="s">
+      <c r="C28" s="61" t="s">
         <v>143</v>
       </c>
       <c r="HS28" s="28"/>
@@ -9295,7 +9352,7 @@
       <c r="B29" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="66" t="s">
+      <c r="C29" s="61" t="s">
         <v>144</v>
       </c>
       <c r="GJ29" s="28"/>
@@ -9338,7 +9395,7 @@
       <c r="B30" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="66" t="s">
+      <c r="C30" s="61" t="s">
         <v>136</v>
       </c>
       <c r="IC30" s="28"/>
@@ -9349,7 +9406,7 @@
       <c r="B31" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C31" s="66" t="s">
+      <c r="C31" s="61" t="s">
         <v>136</v>
       </c>
       <c r="IC31" s="28"/>
@@ -9360,7 +9417,7 @@
       <c r="B32" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="66" t="s">
+      <c r="C32" s="61" t="s">
         <v>145</v>
       </c>
       <c r="IF32" s="28"/>
@@ -9372,7 +9429,7 @@
       <c r="B33" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="66" t="s">
+      <c r="C33" s="61" t="s">
         <v>146</v>
       </c>
       <c r="CG33" s="28"/>
@@ -9415,7 +9472,7 @@
       <c r="B34" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="66" t="s">
+      <c r="C34" s="61" t="s">
         <v>147</v>
       </c>
       <c r="IJ34" s="28"/>
@@ -9428,7 +9485,7 @@
       <c r="B35" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C35" s="66" t="s">
+      <c r="C35" s="61" t="s">
         <v>148</v>
       </c>
       <c r="IP35" s="28"/>
@@ -9439,7 +9496,7 @@
       <c r="B36" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C36" s="66" t="s">
+      <c r="C36" s="61" t="s">
         <v>149</v>
       </c>
       <c r="IS36" s="28"/>
@@ -9455,7 +9512,7 @@
       <c r="B37" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C37" s="66" t="s">
+      <c r="C37" s="61" t="s">
         <v>150</v>
       </c>
       <c r="JA37" s="28"/>
@@ -9524,7 +9581,7 @@
       <c r="B38" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="C38" s="68" t="s">
+      <c r="C38" s="63" t="s">
         <v>151</v>
       </c>
       <c r="JA38" s="28"/>
@@ -9538,7 +9595,7 @@
       <c r="B39" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="63" t="s">
         <v>152</v>
       </c>
       <c r="JG39" s="28"/>
@@ -9552,7 +9609,7 @@
       <c r="B40" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C40" s="68" t="s">
+      <c r="C40" s="63" t="s">
         <v>153</v>
       </c>
       <c r="JM40" s="28"/>
@@ -9566,7 +9623,7 @@
       <c r="B41" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="63" t="s">
         <v>154</v>
       </c>
       <c r="JS41" s="28"/>
@@ -9591,7 +9648,7 @@
       <c r="B42" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C42" s="68" t="s">
+      <c r="C42" s="63" t="s">
         <v>155</v>
       </c>
       <c r="KJ42" s="28"/>
@@ -9625,7 +9682,7 @@
       <c r="B43" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C43" s="68" t="s">
+      <c r="C43" s="63" t="s">
         <v>156</v>
       </c>
       <c r="LI43" s="28"/>
@@ -9634,7 +9691,7 @@
       <c r="B44" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="C44" s="66" t="s">
+      <c r="C44" s="61" t="s">
         <v>157</v>
       </c>
       <c r="LJ44" s="28"/>
@@ -9703,7 +9760,7 @@
       <c r="B45" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="63" t="s">
         <v>158</v>
       </c>
       <c r="LJ45" s="28"/>
@@ -9725,7 +9782,7 @@
       <c r="B46" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="68" t="s">
+      <c r="C46" s="63" t="s">
         <v>159</v>
       </c>
       <c r="LX46" s="28"/>
@@ -9763,7 +9820,7 @@
       <c r="B47" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="63" t="s">
         <v>160</v>
       </c>
       <c r="NB47" s="28"/>
@@ -9788,7 +9845,7 @@
       <c r="B48" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="C48" s="68" t="s">
+      <c r="C48" s="63" t="s">
         <v>161</v>
       </c>
       <c r="NR48" s="28"/>
@@ -9817,383 +9874,383 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38AFB97A-96F2-4583-ACB9-D6943AFDA3A8}">
   <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="6.81640625" customWidth="1"/>
+    <col min="1" max="1" width="6.77734375" customWidth="1"/>
     <col min="2" max="2" width="47" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="68" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="75"/>
+      <c r="C1" s="69"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="38">
+      <c r="A2" s="35">
         <v>1</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="36" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="38">
+    <row r="3" spans="1:3" ht="20.399999999999999">
+      <c r="A3" s="35">
         <v>2</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="36" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="38"/>
-      <c r="B4" s="34" t="s">
+      <c r="A4" s="35"/>
+      <c r="B4" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="39"/>
+      <c r="C4" s="36"/>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="38">
+      <c r="A5" s="35">
         <v>3</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="39"/>
+      <c r="C5" s="36"/>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="63">
+      <c r="A6" s="59">
         <v>4</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="60" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="42">
+      <c r="A7" s="38">
         <v>5</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="43"/>
+      <c r="C7" s="39"/>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="42">
+      <c r="A8" s="38">
         <v>6</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="43"/>
+      <c r="C8" s="39"/>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="42">
+      <c r="A9" s="38">
         <v>7</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="43"/>
+      <c r="C9" s="39"/>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="42">
+      <c r="A10" s="38">
         <v>8</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="43"/>
+      <c r="C10" s="39"/>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="42">
+      <c r="A11" s="38">
         <v>9</v>
       </c>
       <c r="B11" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="43"/>
+      <c r="C11" s="39"/>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="42">
+      <c r="A12" s="38">
         <v>10</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="43"/>
+      <c r="C12" s="39"/>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="42">
+      <c r="A13" s="38">
         <v>11</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="43"/>
+      <c r="C13" s="39"/>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="42">
+      <c r="A14" s="38">
         <v>12</v>
       </c>
       <c r="B14" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="43"/>
+      <c r="C14" s="39"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="42">
+      <c r="A15" s="38">
         <v>13</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="43"/>
+      <c r="C15" s="39"/>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="42">
+      <c r="A16" s="38">
         <v>14</v>
       </c>
       <c r="B16" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="43"/>
+      <c r="C16" s="39"/>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="42">
+      <c r="A17" s="38">
         <v>15</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="43"/>
+      <c r="C17" s="39"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="42">
+      <c r="A18" s="38">
         <v>16</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="43"/>
+      <c r="C18" s="39"/>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="42">
+      <c r="A19" s="38">
         <v>17</v>
       </c>
       <c r="B19" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="43"/>
+      <c r="C19" s="39"/>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="42">
+      <c r="A20" s="38">
         <v>18</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="43"/>
+      <c r="C20" s="39"/>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="42">
+      <c r="A21" s="38">
         <v>19</v>
       </c>
       <c r="B21" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="43"/>
+      <c r="C21" s="39"/>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="42">
+      <c r="A22" s="38">
         <v>20</v>
       </c>
       <c r="B22" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="43"/>
+      <c r="C22" s="39"/>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" s="42">
+      <c r="A23" s="38">
         <v>21</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="43"/>
+      <c r="C23" s="39"/>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="42">
+      <c r="A24" s="38">
         <v>22</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="43"/>
+      <c r="C24" s="39"/>
     </row>
     <row r="25" spans="1:3">
-      <c r="A25" s="42">
+      <c r="A25" s="38">
         <v>23</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="43"/>
+      <c r="C25" s="39"/>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" s="42">
+      <c r="A26" s="38">
         <v>24</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C26" s="43"/>
+      <c r="C26" s="39"/>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="42">
+      <c r="A27" s="38">
         <v>25</v>
       </c>
       <c r="B27" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="43"/>
+      <c r="C27" s="39"/>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" s="42">
+      <c r="A28" s="38">
         <v>26</v>
       </c>
       <c r="B28" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="43"/>
+      <c r="C28" s="39"/>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" s="42">
+      <c r="A29" s="38">
         <v>27</v>
       </c>
       <c r="B29" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="43"/>
+      <c r="C29" s="39"/>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" s="42">
+      <c r="A30" s="38">
         <v>28</v>
       </c>
       <c r="B30" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="43"/>
+      <c r="C30" s="39"/>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" s="48">
+      <c r="A31" s="44">
         <v>29</v>
       </c>
-      <c r="B31" s="49" t="s">
+      <c r="B31" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="50"/>
+      <c r="C31" s="46"/>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="61">
+      <c r="A32" s="57">
         <v>30</v>
       </c>
       <c r="B32" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="62" t="s">
+      <c r="C32" s="58" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="51">
+      <c r="A33" s="47">
         <v>31</v>
       </c>
-      <c r="B33" s="52" t="s">
+      <c r="B33" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="C33" s="53"/>
+      <c r="C33" s="49"/>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="42">
+      <c r="A34" s="38">
         <v>32</v>
       </c>
       <c r="B34" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="43"/>
+      <c r="C34" s="39"/>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="42">
+      <c r="A35" s="38">
         <v>33</v>
       </c>
       <c r="B35" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="43"/>
+      <c r="C35" s="39"/>
     </row>
     <row r="36" spans="1:3">
-      <c r="A36" s="42">
+      <c r="A36" s="38">
         <v>34</v>
       </c>
       <c r="B36" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="43"/>
+      <c r="C36" s="39"/>
     </row>
     <row r="37" spans="1:3">
-      <c r="A37" s="42">
+      <c r="A37" s="38">
         <v>35</v>
       </c>
       <c r="B37" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C37" s="43"/>
+      <c r="C37" s="39"/>
     </row>
     <row r="38" spans="1:3">
-      <c r="A38" s="59">
+      <c r="A38" s="55">
         <v>36</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="46"/>
+      <c r="C38" s="42"/>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" s="54">
+      <c r="A39" s="50">
         <v>37</v>
       </c>
-      <c r="B39" s="55" t="s">
+      <c r="B39" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="C39" s="55" t="s">
+      <c r="C39" s="51" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="56">
+      <c r="A40" s="52">
         <v>38</v>
       </c>
-      <c r="B40" s="52" t="s">
+      <c r="B40" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="C40" s="52"/>
+      <c r="C40" s="48"/>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="47">
+      <c r="A41" s="43">
         <v>39</v>
       </c>
       <c r="B41" s="22" t="s">
@@ -10202,7 +10259,7 @@
       <c r="C41" s="22"/>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="47">
+      <c r="A42" s="43">
         <v>40</v>
       </c>
       <c r="B42" s="22" t="s">
@@ -10211,13 +10268,13 @@
       <c r="C42" s="22"/>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="57">
+      <c r="A43" s="53">
         <v>41</v>
       </c>
-      <c r="B43" s="58" t="s">
+      <c r="B43" s="54" t="s">
         <v>91</v>
       </c>
-      <c r="C43" s="58"/>
+      <c r="C43" s="54"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update schedule preparation Excel and add print paper size configuration
</commit_message>
<xml_diff>
--- a/Schedule Preparation.xlsx
+++ b/Schedule Preparation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0. WtE Power Plant\Tools Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1077BE90-D0D1-42F6-B39D-73371F52DA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F619309-82AA-4501-9270-15364611B757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1028,11 +1028,6 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1051,6 +1046,11 @@
     <xf numFmtId="0" fontId="6" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1391,12 +1391,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D47"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="24.6"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="24"/>
   <cols>
-    <col min="1" max="1" width="69.33203125" style="1" customWidth="1"/>
-    <col min="2" max="4" width="13.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="69.36328125" style="1" customWidth="1"/>
+    <col min="2" max="4" width="13.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2066,592 +2066,592 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:PM48"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="10.199999999999999"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="10"/>
   <cols>
-    <col min="1" max="1" width="5.33203125" style="12" customWidth="1"/>
+    <col min="1" max="1" width="5.36328125" style="12" customWidth="1"/>
     <col min="2" max="2" width="55" style="12" customWidth="1"/>
     <col min="3" max="3" width="19" style="12" customWidth="1"/>
-    <col min="4" max="4" width="2.6640625" style="14" customWidth="1"/>
-    <col min="5" max="10" width="2.6640625" style="13" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" style="14" customWidth="1"/>
-    <col min="12" max="17" width="2.6640625" style="13" customWidth="1"/>
-    <col min="18" max="18" width="2.6640625" style="14" customWidth="1"/>
-    <col min="19" max="24" width="2.6640625" style="13" customWidth="1"/>
-    <col min="25" max="25" width="2.6640625" style="15" customWidth="1"/>
-    <col min="26" max="31" width="2.6640625" style="12" customWidth="1"/>
-    <col min="32" max="32" width="2.6640625" style="15" customWidth="1"/>
-    <col min="33" max="38" width="2.6640625" style="12" customWidth="1"/>
-    <col min="39" max="39" width="2.6640625" style="15" customWidth="1"/>
-    <col min="40" max="45" width="2.6640625" style="12" customWidth="1"/>
-    <col min="46" max="46" width="2.6640625" style="15" customWidth="1"/>
-    <col min="47" max="52" width="2.6640625" style="12" customWidth="1"/>
-    <col min="53" max="53" width="2.6640625" style="15" customWidth="1"/>
-    <col min="54" max="59" width="2.6640625" style="12" customWidth="1"/>
-    <col min="60" max="60" width="2.6640625" style="15" customWidth="1"/>
-    <col min="61" max="66" width="2.6640625" style="12" customWidth="1"/>
-    <col min="67" max="67" width="2.6640625" style="15" customWidth="1"/>
-    <col min="68" max="73" width="2.6640625" style="12" customWidth="1"/>
-    <col min="74" max="74" width="2.6640625" style="15" customWidth="1"/>
-    <col min="75" max="80" width="2.6640625" style="12" customWidth="1"/>
-    <col min="81" max="81" width="2.6640625" style="15" customWidth="1"/>
-    <col min="82" max="87" width="2.6640625" style="12" customWidth="1"/>
-    <col min="88" max="88" width="2.6640625" style="15" customWidth="1"/>
-    <col min="89" max="94" width="2.6640625" style="12" customWidth="1"/>
-    <col min="95" max="95" width="2.6640625" style="15" customWidth="1"/>
-    <col min="96" max="101" width="2.6640625" style="12" customWidth="1"/>
-    <col min="102" max="102" width="2.6640625" style="15" customWidth="1"/>
-    <col min="103" max="108" width="2.6640625" style="12" customWidth="1"/>
-    <col min="109" max="109" width="2.6640625" style="15" customWidth="1"/>
-    <col min="110" max="115" width="2.6640625" style="12" customWidth="1"/>
-    <col min="116" max="116" width="2.6640625" style="15" customWidth="1"/>
-    <col min="117" max="122" width="2.6640625" style="12" customWidth="1"/>
-    <col min="123" max="123" width="2.6640625" style="15" customWidth="1"/>
-    <col min="124" max="129" width="2.6640625" style="12" customWidth="1"/>
-    <col min="130" max="130" width="2.6640625" style="15" customWidth="1"/>
-    <col min="131" max="136" width="2.6640625" style="12" customWidth="1"/>
-    <col min="137" max="137" width="2.6640625" style="15" customWidth="1"/>
-    <col min="138" max="143" width="2.6640625" style="12" customWidth="1"/>
-    <col min="144" max="144" width="2.6640625" style="15" customWidth="1"/>
-    <col min="145" max="150" width="2.6640625" style="12" customWidth="1"/>
-    <col min="151" max="151" width="2.6640625" style="15" customWidth="1"/>
-    <col min="152" max="157" width="2.6640625" style="12" customWidth="1"/>
-    <col min="158" max="158" width="2.6640625" style="15" customWidth="1"/>
-    <col min="159" max="164" width="2.6640625" style="12" customWidth="1"/>
-    <col min="165" max="165" width="2.6640625" style="15" customWidth="1"/>
-    <col min="166" max="171" width="2.6640625" style="12" customWidth="1"/>
-    <col min="172" max="172" width="2.6640625" style="15" customWidth="1"/>
-    <col min="173" max="178" width="2.6640625" style="12" customWidth="1"/>
-    <col min="179" max="179" width="2.6640625" style="15" customWidth="1"/>
-    <col min="180" max="185" width="2.6640625" style="12" customWidth="1"/>
-    <col min="186" max="186" width="2.6640625" style="15" customWidth="1"/>
-    <col min="187" max="192" width="2.6640625" style="12" customWidth="1"/>
-    <col min="193" max="193" width="2.6640625" style="15" customWidth="1"/>
-    <col min="194" max="199" width="2.6640625" style="12" customWidth="1"/>
-    <col min="200" max="200" width="2.6640625" style="15" customWidth="1"/>
-    <col min="201" max="206" width="2.6640625" style="12" customWidth="1"/>
-    <col min="207" max="207" width="2.6640625" style="15" customWidth="1"/>
-    <col min="208" max="213" width="2.6640625" style="12" customWidth="1"/>
-    <col min="214" max="214" width="2.6640625" style="15" customWidth="1"/>
-    <col min="215" max="220" width="2.6640625" style="12" customWidth="1"/>
-    <col min="221" max="221" width="2.6640625" style="15" customWidth="1"/>
-    <col min="222" max="227" width="2.6640625" style="12" customWidth="1"/>
-    <col min="228" max="228" width="2.6640625" style="15" customWidth="1"/>
-    <col min="229" max="234" width="2.6640625" style="12" customWidth="1"/>
-    <col min="235" max="235" width="2.6640625" style="15" customWidth="1"/>
-    <col min="236" max="241" width="2.6640625" style="12" customWidth="1"/>
-    <col min="242" max="242" width="2.6640625" style="15" customWidth="1"/>
-    <col min="243" max="248" width="2.6640625" style="12" customWidth="1"/>
-    <col min="249" max="249" width="2.6640625" style="15" customWidth="1"/>
-    <col min="250" max="255" width="2.6640625" style="12" customWidth="1"/>
-    <col min="256" max="256" width="2.6640625" style="15" customWidth="1"/>
-    <col min="257" max="262" width="2.6640625" style="12" customWidth="1"/>
-    <col min="263" max="263" width="2.6640625" style="15" customWidth="1"/>
-    <col min="264" max="269" width="2.6640625" style="12" customWidth="1"/>
-    <col min="270" max="270" width="2.6640625" style="15" customWidth="1"/>
-    <col min="271" max="276" width="2.6640625" style="12" customWidth="1"/>
-    <col min="277" max="277" width="2.6640625" style="15" customWidth="1"/>
-    <col min="278" max="283" width="2.6640625" style="12" customWidth="1"/>
-    <col min="284" max="284" width="2.6640625" style="15" customWidth="1"/>
-    <col min="285" max="290" width="2.6640625" style="12" customWidth="1"/>
-    <col min="291" max="291" width="2.6640625" style="15" customWidth="1"/>
-    <col min="292" max="297" width="2.6640625" style="12" customWidth="1"/>
-    <col min="298" max="298" width="2.6640625" style="15" customWidth="1"/>
-    <col min="299" max="304" width="2.6640625" style="12" customWidth="1"/>
-    <col min="305" max="305" width="2.6640625" style="15" customWidth="1"/>
-    <col min="306" max="311" width="2.6640625" style="12" customWidth="1"/>
-    <col min="312" max="312" width="2.6640625" style="15" customWidth="1"/>
-    <col min="313" max="318" width="2.6640625" style="12" customWidth="1"/>
-    <col min="319" max="319" width="2.6640625" style="15" customWidth="1"/>
-    <col min="320" max="325" width="2.6640625" style="12" customWidth="1"/>
-    <col min="326" max="326" width="2.6640625" style="15" customWidth="1"/>
-    <col min="327" max="332" width="2.6640625" style="12" customWidth="1"/>
-    <col min="333" max="333" width="2.6640625" style="15" customWidth="1"/>
-    <col min="334" max="339" width="2.6640625" style="12" customWidth="1"/>
-    <col min="340" max="340" width="2.6640625" style="15" customWidth="1"/>
-    <col min="341" max="346" width="2.6640625" style="12" customWidth="1"/>
-    <col min="347" max="347" width="2.6640625" style="15" customWidth="1"/>
-    <col min="348" max="353" width="2.6640625" style="12" customWidth="1"/>
-    <col min="354" max="354" width="2.6640625" style="15" customWidth="1"/>
-    <col min="355" max="360" width="2.6640625" style="12" customWidth="1"/>
-    <col min="361" max="361" width="2.6640625" style="15" customWidth="1"/>
-    <col min="362" max="367" width="2.6640625" style="12" customWidth="1"/>
-    <col min="368" max="368" width="2.6640625" style="15" customWidth="1"/>
-    <col min="369" max="374" width="2.6640625" style="12" customWidth="1"/>
-    <col min="375" max="375" width="2.6640625" style="15" customWidth="1"/>
-    <col min="376" max="381" width="2.6640625" style="12" customWidth="1"/>
-    <col min="382" max="382" width="2.6640625" style="15" customWidth="1"/>
-    <col min="383" max="388" width="2.6640625" style="12" customWidth="1"/>
-    <col min="389" max="389" width="2.6640625" style="15" customWidth="1"/>
-    <col min="390" max="395" width="2.6640625" style="12" customWidth="1"/>
-    <col min="396" max="396" width="2.6640625" style="15" customWidth="1"/>
-    <col min="397" max="402" width="2.6640625" style="12" customWidth="1"/>
-    <col min="403" max="403" width="2.6640625" style="15" customWidth="1"/>
-    <col min="404" max="409" width="2.6640625" style="12" customWidth="1"/>
-    <col min="410" max="410" width="2.6640625" style="15" customWidth="1"/>
-    <col min="411" max="416" width="2.6640625" style="12" customWidth="1"/>
-    <col min="417" max="417" width="2.6640625" style="15" customWidth="1"/>
-    <col min="418" max="423" width="2.6640625" style="12" customWidth="1"/>
-    <col min="424" max="424" width="2.6640625" style="15" customWidth="1"/>
-    <col min="425" max="429" width="2.6640625" style="12" customWidth="1"/>
-    <col min="430" max="430" width="8.77734375" style="12" customWidth="1"/>
-    <col min="431" max="16384" width="8.77734375" style="12"/>
+    <col min="4" max="4" width="2.6328125" style="14" customWidth="1"/>
+    <col min="5" max="10" width="2.6328125" style="13" customWidth="1"/>
+    <col min="11" max="11" width="2.6328125" style="14" customWidth="1"/>
+    <col min="12" max="17" width="2.6328125" style="13" customWidth="1"/>
+    <col min="18" max="18" width="2.6328125" style="14" customWidth="1"/>
+    <col min="19" max="24" width="2.6328125" style="13" customWidth="1"/>
+    <col min="25" max="25" width="2.6328125" style="15" customWidth="1"/>
+    <col min="26" max="31" width="2.6328125" style="12" customWidth="1"/>
+    <col min="32" max="32" width="2.6328125" style="15" customWidth="1"/>
+    <col min="33" max="38" width="2.6328125" style="12" customWidth="1"/>
+    <col min="39" max="39" width="2.6328125" style="15" customWidth="1"/>
+    <col min="40" max="45" width="2.6328125" style="12" customWidth="1"/>
+    <col min="46" max="46" width="2.6328125" style="15" customWidth="1"/>
+    <col min="47" max="52" width="2.6328125" style="12" customWidth="1"/>
+    <col min="53" max="53" width="2.6328125" style="15" customWidth="1"/>
+    <col min="54" max="59" width="2.6328125" style="12" customWidth="1"/>
+    <col min="60" max="60" width="2.6328125" style="15" customWidth="1"/>
+    <col min="61" max="66" width="2.6328125" style="12" customWidth="1"/>
+    <col min="67" max="67" width="2.6328125" style="15" customWidth="1"/>
+    <col min="68" max="73" width="2.6328125" style="12" customWidth="1"/>
+    <col min="74" max="74" width="2.6328125" style="15" customWidth="1"/>
+    <col min="75" max="80" width="2.6328125" style="12" customWidth="1"/>
+    <col min="81" max="81" width="2.6328125" style="15" customWidth="1"/>
+    <col min="82" max="87" width="2.6328125" style="12" customWidth="1"/>
+    <col min="88" max="88" width="2.6328125" style="15" customWidth="1"/>
+    <col min="89" max="94" width="2.6328125" style="12" customWidth="1"/>
+    <col min="95" max="95" width="2.6328125" style="15" customWidth="1"/>
+    <col min="96" max="101" width="2.6328125" style="12" customWidth="1"/>
+    <col min="102" max="102" width="2.6328125" style="15" customWidth="1"/>
+    <col min="103" max="108" width="2.6328125" style="12" customWidth="1"/>
+    <col min="109" max="109" width="2.6328125" style="15" customWidth="1"/>
+    <col min="110" max="115" width="2.6328125" style="12" customWidth="1"/>
+    <col min="116" max="116" width="2.6328125" style="15" customWidth="1"/>
+    <col min="117" max="122" width="2.6328125" style="12" customWidth="1"/>
+    <col min="123" max="123" width="2.6328125" style="15" customWidth="1"/>
+    <col min="124" max="129" width="2.6328125" style="12" customWidth="1"/>
+    <col min="130" max="130" width="2.6328125" style="15" customWidth="1"/>
+    <col min="131" max="136" width="2.6328125" style="12" customWidth="1"/>
+    <col min="137" max="137" width="2.6328125" style="15" customWidth="1"/>
+    <col min="138" max="143" width="2.6328125" style="12" customWidth="1"/>
+    <col min="144" max="144" width="2.6328125" style="15" customWidth="1"/>
+    <col min="145" max="150" width="2.6328125" style="12" customWidth="1"/>
+    <col min="151" max="151" width="2.6328125" style="15" customWidth="1"/>
+    <col min="152" max="157" width="2.6328125" style="12" customWidth="1"/>
+    <col min="158" max="158" width="2.6328125" style="15" customWidth="1"/>
+    <col min="159" max="164" width="2.6328125" style="12" customWidth="1"/>
+    <col min="165" max="165" width="2.6328125" style="15" customWidth="1"/>
+    <col min="166" max="171" width="2.6328125" style="12" customWidth="1"/>
+    <col min="172" max="172" width="2.6328125" style="15" customWidth="1"/>
+    <col min="173" max="178" width="2.6328125" style="12" customWidth="1"/>
+    <col min="179" max="179" width="2.6328125" style="15" customWidth="1"/>
+    <col min="180" max="185" width="2.6328125" style="12" customWidth="1"/>
+    <col min="186" max="186" width="2.6328125" style="15" customWidth="1"/>
+    <col min="187" max="192" width="2.6328125" style="12" customWidth="1"/>
+    <col min="193" max="193" width="2.6328125" style="15" customWidth="1"/>
+    <col min="194" max="199" width="2.6328125" style="12" customWidth="1"/>
+    <col min="200" max="200" width="2.6328125" style="15" customWidth="1"/>
+    <col min="201" max="206" width="2.6328125" style="12" customWidth="1"/>
+    <col min="207" max="207" width="2.6328125" style="15" customWidth="1"/>
+    <col min="208" max="213" width="2.6328125" style="12" customWidth="1"/>
+    <col min="214" max="214" width="2.6328125" style="15" customWidth="1"/>
+    <col min="215" max="220" width="2.6328125" style="12" customWidth="1"/>
+    <col min="221" max="221" width="2.6328125" style="15" customWidth="1"/>
+    <col min="222" max="227" width="2.6328125" style="12" customWidth="1"/>
+    <col min="228" max="228" width="2.6328125" style="15" customWidth="1"/>
+    <col min="229" max="234" width="2.6328125" style="12" customWidth="1"/>
+    <col min="235" max="235" width="2.6328125" style="15" customWidth="1"/>
+    <col min="236" max="241" width="2.6328125" style="12" customWidth="1"/>
+    <col min="242" max="242" width="2.6328125" style="15" customWidth="1"/>
+    <col min="243" max="248" width="2.6328125" style="12" customWidth="1"/>
+    <col min="249" max="249" width="2.6328125" style="15" customWidth="1"/>
+    <col min="250" max="255" width="2.6328125" style="12" customWidth="1"/>
+    <col min="256" max="256" width="2.6328125" style="15" customWidth="1"/>
+    <col min="257" max="262" width="2.6328125" style="12" customWidth="1"/>
+    <col min="263" max="263" width="2.6328125" style="15" customWidth="1"/>
+    <col min="264" max="269" width="2.6328125" style="12" customWidth="1"/>
+    <col min="270" max="270" width="2.6328125" style="15" customWidth="1"/>
+    <col min="271" max="276" width="2.6328125" style="12" customWidth="1"/>
+    <col min="277" max="277" width="2.6328125" style="15" customWidth="1"/>
+    <col min="278" max="283" width="2.6328125" style="12" customWidth="1"/>
+    <col min="284" max="284" width="2.6328125" style="15" customWidth="1"/>
+    <col min="285" max="290" width="2.6328125" style="12" customWidth="1"/>
+    <col min="291" max="291" width="2.6328125" style="15" customWidth="1"/>
+    <col min="292" max="297" width="2.6328125" style="12" customWidth="1"/>
+    <col min="298" max="298" width="2.6328125" style="15" customWidth="1"/>
+    <col min="299" max="304" width="2.6328125" style="12" customWidth="1"/>
+    <col min="305" max="305" width="2.6328125" style="15" customWidth="1"/>
+    <col min="306" max="311" width="2.6328125" style="12" customWidth="1"/>
+    <col min="312" max="312" width="2.6328125" style="15" customWidth="1"/>
+    <col min="313" max="318" width="2.6328125" style="12" customWidth="1"/>
+    <col min="319" max="319" width="2.6328125" style="15" customWidth="1"/>
+    <col min="320" max="325" width="2.6328125" style="12" customWidth="1"/>
+    <col min="326" max="326" width="2.6328125" style="15" customWidth="1"/>
+    <col min="327" max="332" width="2.6328125" style="12" customWidth="1"/>
+    <col min="333" max="333" width="2.6328125" style="15" customWidth="1"/>
+    <col min="334" max="339" width="2.6328125" style="12" customWidth="1"/>
+    <col min="340" max="340" width="2.6328125" style="15" customWidth="1"/>
+    <col min="341" max="346" width="2.6328125" style="12" customWidth="1"/>
+    <col min="347" max="347" width="2.6328125" style="15" customWidth="1"/>
+    <col min="348" max="353" width="2.6328125" style="12" customWidth="1"/>
+    <col min="354" max="354" width="2.6328125" style="15" customWidth="1"/>
+    <col min="355" max="360" width="2.6328125" style="12" customWidth="1"/>
+    <col min="361" max="361" width="2.6328125" style="15" customWidth="1"/>
+    <col min="362" max="367" width="2.6328125" style="12" customWidth="1"/>
+    <col min="368" max="368" width="2.6328125" style="15" customWidth="1"/>
+    <col min="369" max="374" width="2.6328125" style="12" customWidth="1"/>
+    <col min="375" max="375" width="2.6328125" style="15" customWidth="1"/>
+    <col min="376" max="381" width="2.6328125" style="12" customWidth="1"/>
+    <col min="382" max="382" width="2.6328125" style="15" customWidth="1"/>
+    <col min="383" max="388" width="2.6328125" style="12" customWidth="1"/>
+    <col min="389" max="389" width="2.6328125" style="15" customWidth="1"/>
+    <col min="390" max="395" width="2.6328125" style="12" customWidth="1"/>
+    <col min="396" max="396" width="2.6328125" style="15" customWidth="1"/>
+    <col min="397" max="402" width="2.6328125" style="12" customWidth="1"/>
+    <col min="403" max="403" width="2.6328125" style="15" customWidth="1"/>
+    <col min="404" max="409" width="2.6328125" style="12" customWidth="1"/>
+    <col min="410" max="410" width="2.6328125" style="15" customWidth="1"/>
+    <col min="411" max="416" width="2.6328125" style="12" customWidth="1"/>
+    <col min="417" max="417" width="2.6328125" style="15" customWidth="1"/>
+    <col min="418" max="423" width="2.6328125" style="12" customWidth="1"/>
+    <col min="424" max="424" width="2.6328125" style="15" customWidth="1"/>
+    <col min="425" max="429" width="2.6328125" style="12" customWidth="1"/>
+    <col min="430" max="430" width="8.81640625" style="12" customWidth="1"/>
+    <col min="431" max="16384" width="8.81640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:429" ht="19.95" customHeight="1">
-      <c r="D1" s="70">
+    <row r="1" spans="2:429" ht="20" customHeight="1">
+      <c r="D1" s="76">
         <v>46327</v>
       </c>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="71"/>
-      <c r="AA1" s="71"/>
-      <c r="AB1" s="71"/>
-      <c r="AC1" s="71"/>
-      <c r="AD1" s="71"/>
-      <c r="AE1" s="71"/>
-      <c r="AF1" s="71"/>
-      <c r="AG1" s="72"/>
-      <c r="AH1" s="70">
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="77"/>
+      <c r="W1" s="77"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="77"/>
+      <c r="Z1" s="77"/>
+      <c r="AA1" s="77"/>
+      <c r="AB1" s="77"/>
+      <c r="AC1" s="77"/>
+      <c r="AD1" s="77"/>
+      <c r="AE1" s="77"/>
+      <c r="AF1" s="77"/>
+      <c r="AG1" s="78"/>
+      <c r="AH1" s="76">
         <v>46357</v>
       </c>
-      <c r="AI1" s="71"/>
-      <c r="AJ1" s="71"/>
-      <c r="AK1" s="71"/>
-      <c r="AL1" s="71"/>
-      <c r="AM1" s="71"/>
-      <c r="AN1" s="71"/>
-      <c r="AO1" s="71"/>
-      <c r="AP1" s="71"/>
-      <c r="AQ1" s="71"/>
-      <c r="AR1" s="71"/>
-      <c r="AS1" s="71"/>
-      <c r="AT1" s="71"/>
-      <c r="AU1" s="71"/>
-      <c r="AV1" s="71"/>
-      <c r="AW1" s="71"/>
-      <c r="AX1" s="71"/>
-      <c r="AY1" s="71"/>
-      <c r="AZ1" s="71"/>
-      <c r="BA1" s="71"/>
-      <c r="BB1" s="71"/>
-      <c r="BC1" s="71"/>
-      <c r="BD1" s="71"/>
-      <c r="BE1" s="71"/>
-      <c r="BF1" s="71"/>
-      <c r="BG1" s="71"/>
-      <c r="BH1" s="71"/>
-      <c r="BI1" s="71"/>
-      <c r="BJ1" s="71"/>
-      <c r="BK1" s="71"/>
-      <c r="BL1" s="72"/>
-      <c r="BM1" s="70">
+      <c r="AI1" s="77"/>
+      <c r="AJ1" s="77"/>
+      <c r="AK1" s="77"/>
+      <c r="AL1" s="77"/>
+      <c r="AM1" s="77"/>
+      <c r="AN1" s="77"/>
+      <c r="AO1" s="77"/>
+      <c r="AP1" s="77"/>
+      <c r="AQ1" s="77"/>
+      <c r="AR1" s="77"/>
+      <c r="AS1" s="77"/>
+      <c r="AT1" s="77"/>
+      <c r="AU1" s="77"/>
+      <c r="AV1" s="77"/>
+      <c r="AW1" s="77"/>
+      <c r="AX1" s="77"/>
+      <c r="AY1" s="77"/>
+      <c r="AZ1" s="77"/>
+      <c r="BA1" s="77"/>
+      <c r="BB1" s="77"/>
+      <c r="BC1" s="77"/>
+      <c r="BD1" s="77"/>
+      <c r="BE1" s="77"/>
+      <c r="BF1" s="77"/>
+      <c r="BG1" s="77"/>
+      <c r="BH1" s="77"/>
+      <c r="BI1" s="77"/>
+      <c r="BJ1" s="77"/>
+      <c r="BK1" s="77"/>
+      <c r="BL1" s="78"/>
+      <c r="BM1" s="76">
         <v>46388</v>
       </c>
-      <c r="BN1" s="71"/>
-      <c r="BO1" s="71"/>
-      <c r="BP1" s="71"/>
-      <c r="BQ1" s="71"/>
-      <c r="BR1" s="71"/>
-      <c r="BS1" s="71"/>
-      <c r="BT1" s="71"/>
-      <c r="BU1" s="71"/>
-      <c r="BV1" s="71"/>
-      <c r="BW1" s="71"/>
-      <c r="BX1" s="71"/>
-      <c r="BY1" s="71"/>
-      <c r="BZ1" s="71"/>
-      <c r="CA1" s="71"/>
-      <c r="CB1" s="71"/>
-      <c r="CC1" s="71"/>
-      <c r="CD1" s="71"/>
-      <c r="CE1" s="71"/>
-      <c r="CF1" s="71"/>
-      <c r="CG1" s="71"/>
-      <c r="CH1" s="71"/>
-      <c r="CI1" s="71"/>
-      <c r="CJ1" s="71"/>
-      <c r="CK1" s="71"/>
-      <c r="CL1" s="71"/>
-      <c r="CM1" s="71"/>
-      <c r="CN1" s="71"/>
-      <c r="CO1" s="71"/>
-      <c r="CP1" s="71"/>
-      <c r="CQ1" s="72"/>
-      <c r="CR1" s="70">
+      <c r="BN1" s="77"/>
+      <c r="BO1" s="77"/>
+      <c r="BP1" s="77"/>
+      <c r="BQ1" s="77"/>
+      <c r="BR1" s="77"/>
+      <c r="BS1" s="77"/>
+      <c r="BT1" s="77"/>
+      <c r="BU1" s="77"/>
+      <c r="BV1" s="77"/>
+      <c r="BW1" s="77"/>
+      <c r="BX1" s="77"/>
+      <c r="BY1" s="77"/>
+      <c r="BZ1" s="77"/>
+      <c r="CA1" s="77"/>
+      <c r="CB1" s="77"/>
+      <c r="CC1" s="77"/>
+      <c r="CD1" s="77"/>
+      <c r="CE1" s="77"/>
+      <c r="CF1" s="77"/>
+      <c r="CG1" s="77"/>
+      <c r="CH1" s="77"/>
+      <c r="CI1" s="77"/>
+      <c r="CJ1" s="77"/>
+      <c r="CK1" s="77"/>
+      <c r="CL1" s="77"/>
+      <c r="CM1" s="77"/>
+      <c r="CN1" s="77"/>
+      <c r="CO1" s="77"/>
+      <c r="CP1" s="77"/>
+      <c r="CQ1" s="78"/>
+      <c r="CR1" s="76">
         <v>46419</v>
       </c>
-      <c r="CS1" s="71"/>
-      <c r="CT1" s="71"/>
-      <c r="CU1" s="71"/>
-      <c r="CV1" s="71"/>
-      <c r="CW1" s="71"/>
-      <c r="CX1" s="71"/>
-      <c r="CY1" s="71"/>
-      <c r="CZ1" s="71"/>
-      <c r="DA1" s="71"/>
-      <c r="DB1" s="71"/>
-      <c r="DC1" s="71"/>
-      <c r="DD1" s="71"/>
-      <c r="DE1" s="71"/>
-      <c r="DF1" s="71"/>
-      <c r="DG1" s="71"/>
-      <c r="DH1" s="71"/>
-      <c r="DI1" s="71"/>
-      <c r="DJ1" s="71"/>
-      <c r="DK1" s="71"/>
-      <c r="DL1" s="71"/>
-      <c r="DM1" s="71"/>
-      <c r="DN1" s="71"/>
-      <c r="DO1" s="71"/>
-      <c r="DP1" s="71"/>
-      <c r="DQ1" s="71"/>
-      <c r="DR1" s="71"/>
-      <c r="DS1" s="72"/>
-      <c r="DT1" s="70">
+      <c r="CS1" s="77"/>
+      <c r="CT1" s="77"/>
+      <c r="CU1" s="77"/>
+      <c r="CV1" s="77"/>
+      <c r="CW1" s="77"/>
+      <c r="CX1" s="77"/>
+      <c r="CY1" s="77"/>
+      <c r="CZ1" s="77"/>
+      <c r="DA1" s="77"/>
+      <c r="DB1" s="77"/>
+      <c r="DC1" s="77"/>
+      <c r="DD1" s="77"/>
+      <c r="DE1" s="77"/>
+      <c r="DF1" s="77"/>
+      <c r="DG1" s="77"/>
+      <c r="DH1" s="77"/>
+      <c r="DI1" s="77"/>
+      <c r="DJ1" s="77"/>
+      <c r="DK1" s="77"/>
+      <c r="DL1" s="77"/>
+      <c r="DM1" s="77"/>
+      <c r="DN1" s="77"/>
+      <c r="DO1" s="77"/>
+      <c r="DP1" s="77"/>
+      <c r="DQ1" s="77"/>
+      <c r="DR1" s="77"/>
+      <c r="DS1" s="78"/>
+      <c r="DT1" s="76">
         <v>46447</v>
       </c>
-      <c r="DU1" s="71"/>
-      <c r="DV1" s="71"/>
-      <c r="DW1" s="71"/>
-      <c r="DX1" s="71"/>
-      <c r="DY1" s="71"/>
-      <c r="DZ1" s="71"/>
-      <c r="EA1" s="71"/>
-      <c r="EB1" s="71"/>
-      <c r="EC1" s="71"/>
-      <c r="ED1" s="71"/>
-      <c r="EE1" s="71"/>
-      <c r="EF1" s="71"/>
-      <c r="EG1" s="71"/>
-      <c r="EH1" s="71"/>
-      <c r="EI1" s="71"/>
-      <c r="EJ1" s="71"/>
-      <c r="EK1" s="71"/>
-      <c r="EL1" s="71"/>
-      <c r="EM1" s="71"/>
-      <c r="EN1" s="71"/>
-      <c r="EO1" s="71"/>
-      <c r="EP1" s="71"/>
-      <c r="EQ1" s="71"/>
-      <c r="ER1" s="71"/>
-      <c r="ES1" s="71"/>
-      <c r="ET1" s="71"/>
-      <c r="EU1" s="71"/>
-      <c r="EV1" s="71"/>
-      <c r="EW1" s="71"/>
-      <c r="EX1" s="72"/>
-      <c r="EY1" s="70">
+      <c r="DU1" s="77"/>
+      <c r="DV1" s="77"/>
+      <c r="DW1" s="77"/>
+      <c r="DX1" s="77"/>
+      <c r="DY1" s="77"/>
+      <c r="DZ1" s="77"/>
+      <c r="EA1" s="77"/>
+      <c r="EB1" s="77"/>
+      <c r="EC1" s="77"/>
+      <c r="ED1" s="77"/>
+      <c r="EE1" s="77"/>
+      <c r="EF1" s="77"/>
+      <c r="EG1" s="77"/>
+      <c r="EH1" s="77"/>
+      <c r="EI1" s="77"/>
+      <c r="EJ1" s="77"/>
+      <c r="EK1" s="77"/>
+      <c r="EL1" s="77"/>
+      <c r="EM1" s="77"/>
+      <c r="EN1" s="77"/>
+      <c r="EO1" s="77"/>
+      <c r="EP1" s="77"/>
+      <c r="EQ1" s="77"/>
+      <c r="ER1" s="77"/>
+      <c r="ES1" s="77"/>
+      <c r="ET1" s="77"/>
+      <c r="EU1" s="77"/>
+      <c r="EV1" s="77"/>
+      <c r="EW1" s="77"/>
+      <c r="EX1" s="78"/>
+      <c r="EY1" s="76">
         <v>46478</v>
       </c>
-      <c r="EZ1" s="71"/>
-      <c r="FA1" s="71"/>
-      <c r="FB1" s="71"/>
-      <c r="FC1" s="71"/>
-      <c r="FD1" s="71"/>
-      <c r="FE1" s="71"/>
-      <c r="FF1" s="71"/>
-      <c r="FG1" s="71"/>
-      <c r="FH1" s="71"/>
-      <c r="FI1" s="71"/>
-      <c r="FJ1" s="71"/>
-      <c r="FK1" s="71"/>
-      <c r="FL1" s="71"/>
-      <c r="FM1" s="71"/>
-      <c r="FN1" s="71"/>
-      <c r="FO1" s="71"/>
-      <c r="FP1" s="71"/>
-      <c r="FQ1" s="71"/>
-      <c r="FR1" s="71"/>
-      <c r="FS1" s="71"/>
-      <c r="FT1" s="71"/>
-      <c r="FU1" s="71"/>
-      <c r="FV1" s="71"/>
-      <c r="FW1" s="71"/>
-      <c r="FX1" s="71"/>
-      <c r="FY1" s="71"/>
-      <c r="FZ1" s="71"/>
-      <c r="GA1" s="71"/>
-      <c r="GB1" s="72"/>
-      <c r="GC1" s="70">
+      <c r="EZ1" s="77"/>
+      <c r="FA1" s="77"/>
+      <c r="FB1" s="77"/>
+      <c r="FC1" s="77"/>
+      <c r="FD1" s="77"/>
+      <c r="FE1" s="77"/>
+      <c r="FF1" s="77"/>
+      <c r="FG1" s="77"/>
+      <c r="FH1" s="77"/>
+      <c r="FI1" s="77"/>
+      <c r="FJ1" s="77"/>
+      <c r="FK1" s="77"/>
+      <c r="FL1" s="77"/>
+      <c r="FM1" s="77"/>
+      <c r="FN1" s="77"/>
+      <c r="FO1" s="77"/>
+      <c r="FP1" s="77"/>
+      <c r="FQ1" s="77"/>
+      <c r="FR1" s="77"/>
+      <c r="FS1" s="77"/>
+      <c r="FT1" s="77"/>
+      <c r="FU1" s="77"/>
+      <c r="FV1" s="77"/>
+      <c r="FW1" s="77"/>
+      <c r="FX1" s="77"/>
+      <c r="FY1" s="77"/>
+      <c r="FZ1" s="77"/>
+      <c r="GA1" s="77"/>
+      <c r="GB1" s="78"/>
+      <c r="GC1" s="76">
         <v>46508</v>
       </c>
-      <c r="GD1" s="71"/>
-      <c r="GE1" s="71"/>
-      <c r="GF1" s="71"/>
-      <c r="GG1" s="71"/>
-      <c r="GH1" s="71"/>
-      <c r="GI1" s="71"/>
-      <c r="GJ1" s="71"/>
-      <c r="GK1" s="71"/>
-      <c r="GL1" s="71"/>
-      <c r="GM1" s="71"/>
-      <c r="GN1" s="71"/>
-      <c r="GO1" s="71"/>
-      <c r="GP1" s="71"/>
-      <c r="GQ1" s="71"/>
-      <c r="GR1" s="71"/>
-      <c r="GS1" s="71"/>
-      <c r="GT1" s="71"/>
-      <c r="GU1" s="71"/>
-      <c r="GV1" s="71"/>
-      <c r="GW1" s="71"/>
-      <c r="GX1" s="71"/>
-      <c r="GY1" s="71"/>
-      <c r="GZ1" s="71"/>
-      <c r="HA1" s="71"/>
-      <c r="HB1" s="71"/>
-      <c r="HC1" s="71"/>
-      <c r="HD1" s="71"/>
-      <c r="HE1" s="71"/>
-      <c r="HF1" s="71"/>
-      <c r="HG1" s="72"/>
-      <c r="HH1" s="70">
+      <c r="GD1" s="77"/>
+      <c r="GE1" s="77"/>
+      <c r="GF1" s="77"/>
+      <c r="GG1" s="77"/>
+      <c r="GH1" s="77"/>
+      <c r="GI1" s="77"/>
+      <c r="GJ1" s="77"/>
+      <c r="GK1" s="77"/>
+      <c r="GL1" s="77"/>
+      <c r="GM1" s="77"/>
+      <c r="GN1" s="77"/>
+      <c r="GO1" s="77"/>
+      <c r="GP1" s="77"/>
+      <c r="GQ1" s="77"/>
+      <c r="GR1" s="77"/>
+      <c r="GS1" s="77"/>
+      <c r="GT1" s="77"/>
+      <c r="GU1" s="77"/>
+      <c r="GV1" s="77"/>
+      <c r="GW1" s="77"/>
+      <c r="GX1" s="77"/>
+      <c r="GY1" s="77"/>
+      <c r="GZ1" s="77"/>
+      <c r="HA1" s="77"/>
+      <c r="HB1" s="77"/>
+      <c r="HC1" s="77"/>
+      <c r="HD1" s="77"/>
+      <c r="HE1" s="77"/>
+      <c r="HF1" s="77"/>
+      <c r="HG1" s="78"/>
+      <c r="HH1" s="76">
         <v>46539</v>
       </c>
-      <c r="HI1" s="71"/>
-      <c r="HJ1" s="71"/>
-      <c r="HK1" s="71"/>
-      <c r="HL1" s="71"/>
-      <c r="HM1" s="71"/>
-      <c r="HN1" s="71"/>
-      <c r="HO1" s="71"/>
-      <c r="HP1" s="71"/>
-      <c r="HQ1" s="71"/>
-      <c r="HR1" s="71"/>
-      <c r="HS1" s="71"/>
-      <c r="HT1" s="71"/>
-      <c r="HU1" s="71"/>
-      <c r="HV1" s="71"/>
-      <c r="HW1" s="71"/>
-      <c r="HX1" s="71"/>
-      <c r="HY1" s="71"/>
-      <c r="HZ1" s="71"/>
-      <c r="IA1" s="71"/>
-      <c r="IB1" s="71"/>
-      <c r="IC1" s="71"/>
-      <c r="ID1" s="71"/>
-      <c r="IE1" s="71"/>
-      <c r="IF1" s="71"/>
-      <c r="IG1" s="71"/>
-      <c r="IH1" s="71"/>
-      <c r="II1" s="71"/>
-      <c r="IJ1" s="71"/>
-      <c r="IK1" s="72"/>
-      <c r="IL1" s="70">
+      <c r="HI1" s="77"/>
+      <c r="HJ1" s="77"/>
+      <c r="HK1" s="77"/>
+      <c r="HL1" s="77"/>
+      <c r="HM1" s="77"/>
+      <c r="HN1" s="77"/>
+      <c r="HO1" s="77"/>
+      <c r="HP1" s="77"/>
+      <c r="HQ1" s="77"/>
+      <c r="HR1" s="77"/>
+      <c r="HS1" s="77"/>
+      <c r="HT1" s="77"/>
+      <c r="HU1" s="77"/>
+      <c r="HV1" s="77"/>
+      <c r="HW1" s="77"/>
+      <c r="HX1" s="77"/>
+      <c r="HY1" s="77"/>
+      <c r="HZ1" s="77"/>
+      <c r="IA1" s="77"/>
+      <c r="IB1" s="77"/>
+      <c r="IC1" s="77"/>
+      <c r="ID1" s="77"/>
+      <c r="IE1" s="77"/>
+      <c r="IF1" s="77"/>
+      <c r="IG1" s="77"/>
+      <c r="IH1" s="77"/>
+      <c r="II1" s="77"/>
+      <c r="IJ1" s="77"/>
+      <c r="IK1" s="78"/>
+      <c r="IL1" s="76">
         <v>46569</v>
       </c>
-      <c r="IM1" s="71"/>
-      <c r="IN1" s="71"/>
-      <c r="IO1" s="71"/>
-      <c r="IP1" s="71"/>
-      <c r="IQ1" s="71"/>
-      <c r="IR1" s="71"/>
-      <c r="IS1" s="71"/>
-      <c r="IT1" s="71"/>
-      <c r="IU1" s="71"/>
-      <c r="IV1" s="71"/>
-      <c r="IW1" s="71"/>
-      <c r="IX1" s="71"/>
-      <c r="IY1" s="71"/>
-      <c r="IZ1" s="71"/>
-      <c r="JA1" s="71"/>
-      <c r="JB1" s="71"/>
-      <c r="JC1" s="71"/>
-      <c r="JD1" s="71"/>
-      <c r="JE1" s="71"/>
-      <c r="JF1" s="71"/>
-      <c r="JG1" s="71"/>
-      <c r="JH1" s="71"/>
-      <c r="JI1" s="71"/>
-      <c r="JJ1" s="71"/>
-      <c r="JK1" s="71"/>
-      <c r="JL1" s="71"/>
-      <c r="JM1" s="71"/>
-      <c r="JN1" s="71"/>
-      <c r="JO1" s="71"/>
-      <c r="JP1" s="72"/>
-      <c r="JQ1" s="70">
+      <c r="IM1" s="77"/>
+      <c r="IN1" s="77"/>
+      <c r="IO1" s="77"/>
+      <c r="IP1" s="77"/>
+      <c r="IQ1" s="77"/>
+      <c r="IR1" s="77"/>
+      <c r="IS1" s="77"/>
+      <c r="IT1" s="77"/>
+      <c r="IU1" s="77"/>
+      <c r="IV1" s="77"/>
+      <c r="IW1" s="77"/>
+      <c r="IX1" s="77"/>
+      <c r="IY1" s="77"/>
+      <c r="IZ1" s="77"/>
+      <c r="JA1" s="77"/>
+      <c r="JB1" s="77"/>
+      <c r="JC1" s="77"/>
+      <c r="JD1" s="77"/>
+      <c r="JE1" s="77"/>
+      <c r="JF1" s="77"/>
+      <c r="JG1" s="77"/>
+      <c r="JH1" s="77"/>
+      <c r="JI1" s="77"/>
+      <c r="JJ1" s="77"/>
+      <c r="JK1" s="77"/>
+      <c r="JL1" s="77"/>
+      <c r="JM1" s="77"/>
+      <c r="JN1" s="77"/>
+      <c r="JO1" s="77"/>
+      <c r="JP1" s="78"/>
+      <c r="JQ1" s="76">
         <v>46600</v>
       </c>
-      <c r="JR1" s="71"/>
-      <c r="JS1" s="71"/>
-      <c r="JT1" s="71"/>
-      <c r="JU1" s="71"/>
-      <c r="JV1" s="71"/>
-      <c r="JW1" s="71"/>
-      <c r="JX1" s="71"/>
-      <c r="JY1" s="71"/>
-      <c r="JZ1" s="71"/>
-      <c r="KA1" s="71"/>
-      <c r="KB1" s="71"/>
-      <c r="KC1" s="71"/>
-      <c r="KD1" s="71"/>
-      <c r="KE1" s="71"/>
-      <c r="KF1" s="71"/>
-      <c r="KG1" s="71"/>
-      <c r="KH1" s="71"/>
-      <c r="KI1" s="71"/>
-      <c r="KJ1" s="71"/>
-      <c r="KK1" s="71"/>
-      <c r="KL1" s="71"/>
-      <c r="KM1" s="71"/>
-      <c r="KN1" s="71"/>
-      <c r="KO1" s="71"/>
-      <c r="KP1" s="71"/>
-      <c r="KQ1" s="71"/>
-      <c r="KR1" s="71"/>
-      <c r="KS1" s="71"/>
-      <c r="KT1" s="71"/>
-      <c r="KU1" s="72"/>
-      <c r="KV1" s="70">
+      <c r="JR1" s="77"/>
+      <c r="JS1" s="77"/>
+      <c r="JT1" s="77"/>
+      <c r="JU1" s="77"/>
+      <c r="JV1" s="77"/>
+      <c r="JW1" s="77"/>
+      <c r="JX1" s="77"/>
+      <c r="JY1" s="77"/>
+      <c r="JZ1" s="77"/>
+      <c r="KA1" s="77"/>
+      <c r="KB1" s="77"/>
+      <c r="KC1" s="77"/>
+      <c r="KD1" s="77"/>
+      <c r="KE1" s="77"/>
+      <c r="KF1" s="77"/>
+      <c r="KG1" s="77"/>
+      <c r="KH1" s="77"/>
+      <c r="KI1" s="77"/>
+      <c r="KJ1" s="77"/>
+      <c r="KK1" s="77"/>
+      <c r="KL1" s="77"/>
+      <c r="KM1" s="77"/>
+      <c r="KN1" s="77"/>
+      <c r="KO1" s="77"/>
+      <c r="KP1" s="77"/>
+      <c r="KQ1" s="77"/>
+      <c r="KR1" s="77"/>
+      <c r="KS1" s="77"/>
+      <c r="KT1" s="77"/>
+      <c r="KU1" s="78"/>
+      <c r="KV1" s="76">
         <v>46631</v>
       </c>
-      <c r="KW1" s="71"/>
-      <c r="KX1" s="71"/>
-      <c r="KY1" s="71"/>
-      <c r="KZ1" s="71"/>
-      <c r="LA1" s="71"/>
-      <c r="LB1" s="71"/>
-      <c r="LC1" s="71"/>
-      <c r="LD1" s="71"/>
-      <c r="LE1" s="71"/>
-      <c r="LF1" s="71"/>
-      <c r="LG1" s="71"/>
-      <c r="LH1" s="71"/>
-      <c r="LI1" s="71"/>
-      <c r="LJ1" s="71"/>
-      <c r="LK1" s="71"/>
-      <c r="LL1" s="71"/>
-      <c r="LM1" s="71"/>
-      <c r="LN1" s="71"/>
-      <c r="LO1" s="71"/>
-      <c r="LP1" s="71"/>
-      <c r="LQ1" s="71"/>
-      <c r="LR1" s="71"/>
-      <c r="LS1" s="71"/>
-      <c r="LT1" s="71"/>
-      <c r="LU1" s="71"/>
-      <c r="LV1" s="71"/>
-      <c r="LW1" s="71"/>
-      <c r="LX1" s="71"/>
-      <c r="LY1" s="72"/>
-      <c r="LZ1" s="70">
+      <c r="KW1" s="77"/>
+      <c r="KX1" s="77"/>
+      <c r="KY1" s="77"/>
+      <c r="KZ1" s="77"/>
+      <c r="LA1" s="77"/>
+      <c r="LB1" s="77"/>
+      <c r="LC1" s="77"/>
+      <c r="LD1" s="77"/>
+      <c r="LE1" s="77"/>
+      <c r="LF1" s="77"/>
+      <c r="LG1" s="77"/>
+      <c r="LH1" s="77"/>
+      <c r="LI1" s="77"/>
+      <c r="LJ1" s="77"/>
+      <c r="LK1" s="77"/>
+      <c r="LL1" s="77"/>
+      <c r="LM1" s="77"/>
+      <c r="LN1" s="77"/>
+      <c r="LO1" s="77"/>
+      <c r="LP1" s="77"/>
+      <c r="LQ1" s="77"/>
+      <c r="LR1" s="77"/>
+      <c r="LS1" s="77"/>
+      <c r="LT1" s="77"/>
+      <c r="LU1" s="77"/>
+      <c r="LV1" s="77"/>
+      <c r="LW1" s="77"/>
+      <c r="LX1" s="77"/>
+      <c r="LY1" s="78"/>
+      <c r="LZ1" s="76">
         <v>46661</v>
       </c>
-      <c r="MA1" s="71"/>
-      <c r="MB1" s="71"/>
-      <c r="MC1" s="71"/>
-      <c r="MD1" s="71"/>
-      <c r="ME1" s="71"/>
-      <c r="MF1" s="71"/>
-      <c r="MG1" s="71"/>
-      <c r="MH1" s="71"/>
-      <c r="MI1" s="71"/>
-      <c r="MJ1" s="71"/>
-      <c r="MK1" s="71"/>
-      <c r="ML1" s="71"/>
-      <c r="MM1" s="71"/>
-      <c r="MN1" s="71"/>
-      <c r="MO1" s="71"/>
-      <c r="MP1" s="71"/>
-      <c r="MQ1" s="71"/>
-      <c r="MR1" s="71"/>
-      <c r="MS1" s="71"/>
-      <c r="MT1" s="71"/>
-      <c r="MU1" s="71"/>
-      <c r="MV1" s="71"/>
-      <c r="MW1" s="71"/>
-      <c r="MX1" s="71"/>
-      <c r="MY1" s="71"/>
-      <c r="MZ1" s="71"/>
-      <c r="NA1" s="71"/>
-      <c r="NB1" s="71"/>
-      <c r="NC1" s="71"/>
-      <c r="ND1" s="72"/>
-      <c r="NE1" s="70">
+      <c r="MA1" s="77"/>
+      <c r="MB1" s="77"/>
+      <c r="MC1" s="77"/>
+      <c r="MD1" s="77"/>
+      <c r="ME1" s="77"/>
+      <c r="MF1" s="77"/>
+      <c r="MG1" s="77"/>
+      <c r="MH1" s="77"/>
+      <c r="MI1" s="77"/>
+      <c r="MJ1" s="77"/>
+      <c r="MK1" s="77"/>
+      <c r="ML1" s="77"/>
+      <c r="MM1" s="77"/>
+      <c r="MN1" s="77"/>
+      <c r="MO1" s="77"/>
+      <c r="MP1" s="77"/>
+      <c r="MQ1" s="77"/>
+      <c r="MR1" s="77"/>
+      <c r="MS1" s="77"/>
+      <c r="MT1" s="77"/>
+      <c r="MU1" s="77"/>
+      <c r="MV1" s="77"/>
+      <c r="MW1" s="77"/>
+      <c r="MX1" s="77"/>
+      <c r="MY1" s="77"/>
+      <c r="MZ1" s="77"/>
+      <c r="NA1" s="77"/>
+      <c r="NB1" s="77"/>
+      <c r="NC1" s="77"/>
+      <c r="ND1" s="78"/>
+      <c r="NE1" s="76">
         <v>46692</v>
       </c>
-      <c r="NF1" s="71"/>
-      <c r="NG1" s="71"/>
-      <c r="NH1" s="71"/>
-      <c r="NI1" s="71"/>
-      <c r="NJ1" s="71"/>
-      <c r="NK1" s="71"/>
-      <c r="NL1" s="71"/>
-      <c r="NM1" s="71"/>
-      <c r="NN1" s="71"/>
-      <c r="NO1" s="71"/>
-      <c r="NP1" s="71"/>
-      <c r="NQ1" s="71"/>
-      <c r="NR1" s="71"/>
-      <c r="NS1" s="71"/>
-      <c r="NT1" s="71"/>
-      <c r="NU1" s="71"/>
-      <c r="NV1" s="71"/>
-      <c r="NW1" s="71"/>
-      <c r="NX1" s="71"/>
-      <c r="NY1" s="71"/>
-      <c r="NZ1" s="71"/>
-      <c r="OA1" s="71"/>
-      <c r="OB1" s="71"/>
-      <c r="OC1" s="71"/>
-      <c r="OD1" s="71"/>
-      <c r="OE1" s="71"/>
-      <c r="OF1" s="71"/>
-      <c r="OG1" s="71"/>
-      <c r="OH1" s="72"/>
-      <c r="OI1" s="70">
+      <c r="NF1" s="77"/>
+      <c r="NG1" s="77"/>
+      <c r="NH1" s="77"/>
+      <c r="NI1" s="77"/>
+      <c r="NJ1" s="77"/>
+      <c r="NK1" s="77"/>
+      <c r="NL1" s="77"/>
+      <c r="NM1" s="77"/>
+      <c r="NN1" s="77"/>
+      <c r="NO1" s="77"/>
+      <c r="NP1" s="77"/>
+      <c r="NQ1" s="77"/>
+      <c r="NR1" s="77"/>
+      <c r="NS1" s="77"/>
+      <c r="NT1" s="77"/>
+      <c r="NU1" s="77"/>
+      <c r="NV1" s="77"/>
+      <c r="NW1" s="77"/>
+      <c r="NX1" s="77"/>
+      <c r="NY1" s="77"/>
+      <c r="NZ1" s="77"/>
+      <c r="OA1" s="77"/>
+      <c r="OB1" s="77"/>
+      <c r="OC1" s="77"/>
+      <c r="OD1" s="77"/>
+      <c r="OE1" s="77"/>
+      <c r="OF1" s="77"/>
+      <c r="OG1" s="77"/>
+      <c r="OH1" s="78"/>
+      <c r="OI1" s="76">
         <v>46722</v>
       </c>
-      <c r="OJ1" s="71"/>
-      <c r="OK1" s="71"/>
-      <c r="OL1" s="71"/>
-      <c r="OM1" s="71"/>
-      <c r="ON1" s="71"/>
-      <c r="OO1" s="71"/>
-      <c r="OP1" s="71"/>
-      <c r="OQ1" s="71"/>
-      <c r="OR1" s="71"/>
-      <c r="OS1" s="71"/>
-      <c r="OT1" s="71"/>
-      <c r="OU1" s="71"/>
-      <c r="OV1" s="71"/>
-      <c r="OW1" s="71"/>
-      <c r="OX1" s="71"/>
-      <c r="OY1" s="71"/>
-      <c r="OZ1" s="71"/>
-      <c r="PA1" s="71"/>
-      <c r="PB1" s="71"/>
-      <c r="PC1" s="71"/>
-      <c r="PD1" s="71"/>
-      <c r="PE1" s="71"/>
-      <c r="PF1" s="71"/>
-      <c r="PG1" s="71"/>
-      <c r="PH1" s="71"/>
-      <c r="PI1" s="71"/>
-      <c r="PJ1" s="71"/>
-      <c r="PK1" s="71"/>
-      <c r="PL1" s="71"/>
-      <c r="PM1" s="72"/>
+      <c r="OJ1" s="77"/>
+      <c r="OK1" s="77"/>
+      <c r="OL1" s="77"/>
+      <c r="OM1" s="77"/>
+      <c r="ON1" s="77"/>
+      <c r="OO1" s="77"/>
+      <c r="OP1" s="77"/>
+      <c r="OQ1" s="77"/>
+      <c r="OR1" s="77"/>
+      <c r="OS1" s="77"/>
+      <c r="OT1" s="77"/>
+      <c r="OU1" s="77"/>
+      <c r="OV1" s="77"/>
+      <c r="OW1" s="77"/>
+      <c r="OX1" s="77"/>
+      <c r="OY1" s="77"/>
+      <c r="OZ1" s="77"/>
+      <c r="PA1" s="77"/>
+      <c r="PB1" s="77"/>
+      <c r="PC1" s="77"/>
+      <c r="PD1" s="77"/>
+      <c r="PE1" s="77"/>
+      <c r="PF1" s="77"/>
+      <c r="PG1" s="77"/>
+      <c r="PH1" s="77"/>
+      <c r="PI1" s="77"/>
+      <c r="PJ1" s="77"/>
+      <c r="PK1" s="77"/>
+      <c r="PL1" s="77"/>
+      <c r="PM1" s="78"/>
     </row>
     <row r="2" spans="2:429" ht="10.5" customHeight="1">
       <c r="B2" s="25" t="s">
@@ -5192,10 +5192,10 @@
       <c r="FS25" s="26"/>
     </row>
     <row r="26" spans="2:215" ht="15" customHeight="1">
-      <c r="B26" s="78" t="s">
+      <c r="B26" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="78" t="s">
+      <c r="C26" s="75" t="s">
         <v>48</v>
       </c>
       <c r="FT26" s="37"/>
@@ -5758,12 +5758,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7DAE1D-59BF-444C-AB6B-E4987E444A19}">
   <dimension ref="A1:D43"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="6.81640625" style="13" customWidth="1"/>
     <col min="2" max="2" width="47" style="33" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" style="33" customWidth="1"/>
-    <col min="4" max="16384" width="8.77734375" style="33"/>
+    <col min="3" max="3" width="18.81640625" style="33" customWidth="1"/>
+    <col min="4" max="16384" width="8.81640625" style="33"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
@@ -5785,7 +5785,7 @@
       <c r="C2" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="D2" s="73"/>
+      <c r="D2" s="70"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1">
       <c r="A3" s="35">
@@ -5797,7 +5797,7 @@
       <c r="C3" s="36" t="s">
         <v>167</v>
       </c>
-      <c r="D3" s="73"/>
+      <c r="D3" s="70"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
       <c r="A4" s="35"/>
@@ -5805,7 +5805,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="36"/>
-      <c r="D4" s="73"/>
+      <c r="D4" s="70"/>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1">
       <c r="A5" s="35">
@@ -5815,7 +5815,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="36"/>
-      <c r="D5" s="73"/>
+      <c r="D5" s="70"/>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1">
       <c r="A6" s="59">
@@ -5836,7 +5836,7 @@
         <v>61</v>
       </c>
       <c r="C7" s="39"/>
-      <c r="D7" s="73"/>
+      <c r="D7" s="70"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1">
       <c r="A8" s="38">
@@ -5846,7 +5846,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="39"/>
-      <c r="D8" s="73"/>
+      <c r="D8" s="70"/>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1">
       <c r="A9" s="38">
@@ -5856,7 +5856,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="39"/>
-      <c r="D9" s="73"/>
+      <c r="D9" s="70"/>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1">
       <c r="A10" s="38">
@@ -5866,27 +5866,27 @@
         <v>24</v>
       </c>
       <c r="C10" s="39"/>
-      <c r="D10" s="73"/>
+      <c r="D10" s="70"/>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A11" s="75">
+      <c r="A11" s="72">
         <v>9</v>
       </c>
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="77"/>
-      <c r="D11" s="73"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="70"/>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" thickTop="1">
       <c r="A12" s="47">
         <v>10</v>
       </c>
-      <c r="B12" s="74" t="s">
+      <c r="B12" s="71" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="49"/>
-      <c r="D12" s="73"/>
+      <c r="D12" s="70"/>
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1">
       <c r="A13" s="38">
@@ -5896,7 +5896,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="39"/>
-      <c r="D13" s="73"/>
+      <c r="D13" s="70"/>
     </row>
     <row r="14" spans="1:4" ht="15" customHeight="1">
       <c r="A14" s="38">
@@ -5906,7 +5906,7 @@
         <v>18</v>
       </c>
       <c r="C14" s="39"/>
-      <c r="D14" s="73"/>
+      <c r="D14" s="70"/>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1">
       <c r="A15" s="38">
@@ -5916,7 +5916,7 @@
         <v>16</v>
       </c>
       <c r="C15" s="39"/>
-      <c r="D15" s="73"/>
+      <c r="D15" s="70"/>
     </row>
     <row r="16" spans="1:4" ht="15" customHeight="1">
       <c r="A16" s="38">
@@ -5926,7 +5926,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="39"/>
-      <c r="D16" s="73"/>
+      <c r="D16" s="70"/>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
       <c r="A17" s="38">
@@ -5936,7 +5936,7 @@
         <v>22</v>
       </c>
       <c r="C17" s="39"/>
-      <c r="D17" s="73"/>
+      <c r="D17" s="70"/>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1">
       <c r="A18" s="38">
@@ -5946,7 +5946,7 @@
         <v>42</v>
       </c>
       <c r="C18" s="39"/>
-      <c r="D18" s="73"/>
+      <c r="D18" s="70"/>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1">
       <c r="A19" s="38">
@@ -5956,7 +5956,7 @@
         <v>43</v>
       </c>
       <c r="C19" s="39"/>
-      <c r="D19" s="73"/>
+      <c r="D19" s="70"/>
     </row>
     <row r="20" spans="1:4" ht="15" customHeight="1">
       <c r="A20" s="38">
@@ -6186,592 +6186,592 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:PM48"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="10.199999999999999"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="10"/>
   <cols>
-    <col min="1" max="1" width="5.33203125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="48.21875" style="12" customWidth="1"/>
+    <col min="1" max="1" width="5.36328125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="48.1796875" style="12" customWidth="1"/>
     <col min="3" max="3" width="21" style="13" customWidth="1"/>
-    <col min="4" max="9" width="2.6640625" style="13" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" style="14" customWidth="1"/>
-    <col min="11" max="16" width="2.6640625" style="13" customWidth="1"/>
-    <col min="17" max="17" width="2.6640625" style="14" customWidth="1"/>
-    <col min="18" max="23" width="2.6640625" style="13" customWidth="1"/>
-    <col min="24" max="24" width="2.6640625" style="15" customWidth="1"/>
-    <col min="25" max="30" width="2.6640625" style="12" customWidth="1"/>
-    <col min="31" max="31" width="2.6640625" style="15" customWidth="1"/>
-    <col min="32" max="37" width="2.6640625" style="12" customWidth="1"/>
-    <col min="38" max="38" width="2.6640625" style="15" customWidth="1"/>
-    <col min="39" max="44" width="2.6640625" style="12" customWidth="1"/>
-    <col min="45" max="45" width="2.6640625" style="15" customWidth="1"/>
-    <col min="46" max="51" width="2.6640625" style="12" customWidth="1"/>
-    <col min="52" max="52" width="2.6640625" style="15" customWidth="1"/>
-    <col min="53" max="58" width="2.6640625" style="12" customWidth="1"/>
-    <col min="59" max="59" width="2.6640625" style="15" customWidth="1"/>
-    <col min="60" max="65" width="2.6640625" style="12" customWidth="1"/>
-    <col min="66" max="66" width="2.6640625" style="15" customWidth="1"/>
-    <col min="67" max="72" width="2.6640625" style="12" customWidth="1"/>
-    <col min="73" max="73" width="2.6640625" style="15" customWidth="1"/>
-    <col min="74" max="79" width="2.6640625" style="12" customWidth="1"/>
-    <col min="80" max="80" width="2.6640625" style="15" customWidth="1"/>
-    <col min="81" max="86" width="2.6640625" style="12" customWidth="1"/>
-    <col min="87" max="87" width="2.6640625" style="15" customWidth="1"/>
-    <col min="88" max="93" width="2.6640625" style="12" customWidth="1"/>
-    <col min="94" max="94" width="2.6640625" style="15" customWidth="1"/>
-    <col min="95" max="100" width="2.6640625" style="12" customWidth="1"/>
-    <col min="101" max="101" width="2.6640625" style="15" customWidth="1"/>
-    <col min="102" max="107" width="2.6640625" style="12" customWidth="1"/>
-    <col min="108" max="108" width="2.6640625" style="15" customWidth="1"/>
-    <col min="109" max="114" width="2.6640625" style="12" customWidth="1"/>
-    <col min="115" max="115" width="2.6640625" style="15" customWidth="1"/>
-    <col min="116" max="121" width="2.6640625" style="12" customWidth="1"/>
-    <col min="122" max="122" width="2.6640625" style="15" customWidth="1"/>
-    <col min="123" max="128" width="2.6640625" style="12" customWidth="1"/>
-    <col min="129" max="129" width="2.6640625" style="15" customWidth="1"/>
-    <col min="130" max="135" width="2.6640625" style="12" customWidth="1"/>
-    <col min="136" max="136" width="2.6640625" style="15" customWidth="1"/>
-    <col min="137" max="142" width="2.6640625" style="12" customWidth="1"/>
-    <col min="143" max="143" width="2.6640625" style="15" customWidth="1"/>
-    <col min="144" max="149" width="2.6640625" style="12" customWidth="1"/>
-    <col min="150" max="150" width="2.6640625" style="15" customWidth="1"/>
-    <col min="151" max="156" width="2.6640625" style="12" customWidth="1"/>
-    <col min="157" max="157" width="2.6640625" style="15" customWidth="1"/>
-    <col min="158" max="163" width="2.6640625" style="12" customWidth="1"/>
-    <col min="164" max="164" width="2.6640625" style="15" customWidth="1"/>
-    <col min="165" max="170" width="2.6640625" style="12" customWidth="1"/>
-    <col min="171" max="171" width="2.6640625" style="15" customWidth="1"/>
-    <col min="172" max="177" width="2.6640625" style="12" customWidth="1"/>
-    <col min="178" max="178" width="2.6640625" style="15" customWidth="1"/>
-    <col min="179" max="184" width="2.6640625" style="12" customWidth="1"/>
-    <col min="185" max="185" width="2.6640625" style="15" customWidth="1"/>
-    <col min="186" max="191" width="2.6640625" style="12" customWidth="1"/>
-    <col min="192" max="192" width="2.6640625" style="15" customWidth="1"/>
-    <col min="193" max="198" width="2.6640625" style="12" customWidth="1"/>
-    <col min="199" max="199" width="2.6640625" style="15" customWidth="1"/>
-    <col min="200" max="205" width="2.6640625" style="12" customWidth="1"/>
-    <col min="206" max="206" width="2.6640625" style="15" customWidth="1"/>
-    <col min="207" max="212" width="2.6640625" style="12" customWidth="1"/>
-    <col min="213" max="213" width="2.6640625" style="15" customWidth="1"/>
-    <col min="214" max="219" width="2.6640625" style="12" customWidth="1"/>
-    <col min="220" max="220" width="2.6640625" style="15" customWidth="1"/>
-    <col min="221" max="226" width="2.6640625" style="12" customWidth="1"/>
-    <col min="227" max="227" width="2.6640625" style="15" customWidth="1"/>
-    <col min="228" max="233" width="2.6640625" style="12" customWidth="1"/>
-    <col min="234" max="234" width="2.6640625" style="15" customWidth="1"/>
-    <col min="235" max="240" width="2.6640625" style="12" customWidth="1"/>
-    <col min="241" max="241" width="2.6640625" style="15" customWidth="1"/>
-    <col min="242" max="247" width="2.6640625" style="12" customWidth="1"/>
-    <col min="248" max="248" width="2.6640625" style="15" customWidth="1"/>
-    <col min="249" max="254" width="2.6640625" style="12" customWidth="1"/>
-    <col min="255" max="255" width="2.6640625" style="15" customWidth="1"/>
-    <col min="256" max="261" width="2.6640625" style="12" customWidth="1"/>
-    <col min="262" max="262" width="2.6640625" style="15" customWidth="1"/>
-    <col min="263" max="268" width="2.6640625" style="12" customWidth="1"/>
-    <col min="269" max="269" width="2.6640625" style="15" customWidth="1"/>
-    <col min="270" max="275" width="2.6640625" style="12" customWidth="1"/>
-    <col min="276" max="276" width="2.6640625" style="15" customWidth="1"/>
-    <col min="277" max="282" width="2.6640625" style="12" customWidth="1"/>
-    <col min="283" max="283" width="2.6640625" style="15" customWidth="1"/>
-    <col min="284" max="289" width="2.6640625" style="12" customWidth="1"/>
-    <col min="290" max="290" width="2.6640625" style="15" customWidth="1"/>
-    <col min="291" max="296" width="2.6640625" style="12" customWidth="1"/>
-    <col min="297" max="297" width="2.6640625" style="15" customWidth="1"/>
-    <col min="298" max="303" width="2.6640625" style="12" customWidth="1"/>
-    <col min="304" max="304" width="2.6640625" style="15" customWidth="1"/>
-    <col min="305" max="310" width="2.6640625" style="12" customWidth="1"/>
-    <col min="311" max="311" width="2.6640625" style="15" customWidth="1"/>
-    <col min="312" max="317" width="2.6640625" style="12" customWidth="1"/>
-    <col min="318" max="318" width="2.6640625" style="15" customWidth="1"/>
-    <col min="319" max="324" width="2.6640625" style="12" customWidth="1"/>
-    <col min="325" max="325" width="2.6640625" style="15" customWidth="1"/>
-    <col min="326" max="331" width="2.6640625" style="12" customWidth="1"/>
-    <col min="332" max="332" width="2.6640625" style="15" customWidth="1"/>
-    <col min="333" max="338" width="2.6640625" style="12" customWidth="1"/>
-    <col min="339" max="339" width="2.6640625" style="15" customWidth="1"/>
-    <col min="340" max="345" width="2.6640625" style="12" customWidth="1"/>
-    <col min="346" max="346" width="2.6640625" style="15" customWidth="1"/>
-    <col min="347" max="352" width="2.6640625" style="12" customWidth="1"/>
-    <col min="353" max="353" width="2.6640625" style="15" customWidth="1"/>
-    <col min="354" max="359" width="2.6640625" style="12" customWidth="1"/>
-    <col min="360" max="360" width="2.6640625" style="15" customWidth="1"/>
-    <col min="361" max="366" width="2.6640625" style="12" customWidth="1"/>
-    <col min="367" max="367" width="2.6640625" style="15" customWidth="1"/>
-    <col min="368" max="373" width="2.6640625" style="12" customWidth="1"/>
-    <col min="374" max="374" width="2.6640625" style="15" customWidth="1"/>
-    <col min="375" max="380" width="2.6640625" style="12" customWidth="1"/>
-    <col min="381" max="381" width="2.6640625" style="15" customWidth="1"/>
-    <col min="382" max="387" width="2.6640625" style="12" customWidth="1"/>
-    <col min="388" max="388" width="2.6640625" style="15" customWidth="1"/>
-    <col min="389" max="394" width="2.6640625" style="12" customWidth="1"/>
-    <col min="395" max="395" width="2.6640625" style="15" customWidth="1"/>
-    <col min="396" max="401" width="2.6640625" style="12" customWidth="1"/>
-    <col min="402" max="402" width="2.6640625" style="15" customWidth="1"/>
-    <col min="403" max="408" width="2.6640625" style="12" customWidth="1"/>
-    <col min="409" max="409" width="2.6640625" style="15" customWidth="1"/>
-    <col min="410" max="415" width="2.6640625" style="12" customWidth="1"/>
-    <col min="416" max="416" width="2.6640625" style="15" customWidth="1"/>
-    <col min="417" max="422" width="2.6640625" style="12" customWidth="1"/>
-    <col min="423" max="423" width="2.6640625" style="15" customWidth="1"/>
-    <col min="424" max="428" width="2.6640625" style="12" customWidth="1"/>
-    <col min="429" max="429" width="8.77734375" style="12" customWidth="1"/>
-    <col min="430" max="16384" width="8.77734375" style="12"/>
+    <col min="4" max="9" width="2.6328125" style="13" customWidth="1"/>
+    <col min="10" max="10" width="2.6328125" style="14" customWidth="1"/>
+    <col min="11" max="16" width="2.6328125" style="13" customWidth="1"/>
+    <col min="17" max="17" width="2.6328125" style="14" customWidth="1"/>
+    <col min="18" max="23" width="2.6328125" style="13" customWidth="1"/>
+    <col min="24" max="24" width="2.6328125" style="15" customWidth="1"/>
+    <col min="25" max="30" width="2.6328125" style="12" customWidth="1"/>
+    <col min="31" max="31" width="2.6328125" style="15" customWidth="1"/>
+    <col min="32" max="37" width="2.6328125" style="12" customWidth="1"/>
+    <col min="38" max="38" width="2.6328125" style="15" customWidth="1"/>
+    <col min="39" max="44" width="2.6328125" style="12" customWidth="1"/>
+    <col min="45" max="45" width="2.6328125" style="15" customWidth="1"/>
+    <col min="46" max="51" width="2.6328125" style="12" customWidth="1"/>
+    <col min="52" max="52" width="2.6328125" style="15" customWidth="1"/>
+    <col min="53" max="58" width="2.6328125" style="12" customWidth="1"/>
+    <col min="59" max="59" width="2.6328125" style="15" customWidth="1"/>
+    <col min="60" max="65" width="2.6328125" style="12" customWidth="1"/>
+    <col min="66" max="66" width="2.6328125" style="15" customWidth="1"/>
+    <col min="67" max="72" width="2.6328125" style="12" customWidth="1"/>
+    <col min="73" max="73" width="2.6328125" style="15" customWidth="1"/>
+    <col min="74" max="79" width="2.6328125" style="12" customWidth="1"/>
+    <col min="80" max="80" width="2.6328125" style="15" customWidth="1"/>
+    <col min="81" max="86" width="2.6328125" style="12" customWidth="1"/>
+    <col min="87" max="87" width="2.6328125" style="15" customWidth="1"/>
+    <col min="88" max="93" width="2.6328125" style="12" customWidth="1"/>
+    <col min="94" max="94" width="2.6328125" style="15" customWidth="1"/>
+    <col min="95" max="100" width="2.6328125" style="12" customWidth="1"/>
+    <col min="101" max="101" width="2.6328125" style="15" customWidth="1"/>
+    <col min="102" max="107" width="2.6328125" style="12" customWidth="1"/>
+    <col min="108" max="108" width="2.6328125" style="15" customWidth="1"/>
+    <col min="109" max="114" width="2.6328125" style="12" customWidth="1"/>
+    <col min="115" max="115" width="2.6328125" style="15" customWidth="1"/>
+    <col min="116" max="121" width="2.6328125" style="12" customWidth="1"/>
+    <col min="122" max="122" width="2.6328125" style="15" customWidth="1"/>
+    <col min="123" max="128" width="2.6328125" style="12" customWidth="1"/>
+    <col min="129" max="129" width="2.6328125" style="15" customWidth="1"/>
+    <col min="130" max="135" width="2.6328125" style="12" customWidth="1"/>
+    <col min="136" max="136" width="2.6328125" style="15" customWidth="1"/>
+    <col min="137" max="142" width="2.6328125" style="12" customWidth="1"/>
+    <col min="143" max="143" width="2.6328125" style="15" customWidth="1"/>
+    <col min="144" max="149" width="2.6328125" style="12" customWidth="1"/>
+    <col min="150" max="150" width="2.6328125" style="15" customWidth="1"/>
+    <col min="151" max="156" width="2.6328125" style="12" customWidth="1"/>
+    <col min="157" max="157" width="2.6328125" style="15" customWidth="1"/>
+    <col min="158" max="163" width="2.6328125" style="12" customWidth="1"/>
+    <col min="164" max="164" width="2.6328125" style="15" customWidth="1"/>
+    <col min="165" max="170" width="2.6328125" style="12" customWidth="1"/>
+    <col min="171" max="171" width="2.6328125" style="15" customWidth="1"/>
+    <col min="172" max="177" width="2.6328125" style="12" customWidth="1"/>
+    <col min="178" max="178" width="2.6328125" style="15" customWidth="1"/>
+    <col min="179" max="184" width="2.6328125" style="12" customWidth="1"/>
+    <col min="185" max="185" width="2.6328125" style="15" customWidth="1"/>
+    <col min="186" max="191" width="2.6328125" style="12" customWidth="1"/>
+    <col min="192" max="192" width="2.6328125" style="15" customWidth="1"/>
+    <col min="193" max="198" width="2.6328125" style="12" customWidth="1"/>
+    <col min="199" max="199" width="2.6328125" style="15" customWidth="1"/>
+    <col min="200" max="205" width="2.6328125" style="12" customWidth="1"/>
+    <col min="206" max="206" width="2.6328125" style="15" customWidth="1"/>
+    <col min="207" max="212" width="2.6328125" style="12" customWidth="1"/>
+    <col min="213" max="213" width="2.6328125" style="15" customWidth="1"/>
+    <col min="214" max="219" width="2.6328125" style="12" customWidth="1"/>
+    <col min="220" max="220" width="2.6328125" style="15" customWidth="1"/>
+    <col min="221" max="226" width="2.6328125" style="12" customWidth="1"/>
+    <col min="227" max="227" width="2.6328125" style="15" customWidth="1"/>
+    <col min="228" max="233" width="2.6328125" style="12" customWidth="1"/>
+    <col min="234" max="234" width="2.6328125" style="15" customWidth="1"/>
+    <col min="235" max="240" width="2.6328125" style="12" customWidth="1"/>
+    <col min="241" max="241" width="2.6328125" style="15" customWidth="1"/>
+    <col min="242" max="247" width="2.6328125" style="12" customWidth="1"/>
+    <col min="248" max="248" width="2.6328125" style="15" customWidth="1"/>
+    <col min="249" max="254" width="2.6328125" style="12" customWidth="1"/>
+    <col min="255" max="255" width="2.6328125" style="15" customWidth="1"/>
+    <col min="256" max="261" width="2.6328125" style="12" customWidth="1"/>
+    <col min="262" max="262" width="2.6328125" style="15" customWidth="1"/>
+    <col min="263" max="268" width="2.6328125" style="12" customWidth="1"/>
+    <col min="269" max="269" width="2.6328125" style="15" customWidth="1"/>
+    <col min="270" max="275" width="2.6328125" style="12" customWidth="1"/>
+    <col min="276" max="276" width="2.6328125" style="15" customWidth="1"/>
+    <col min="277" max="282" width="2.6328125" style="12" customWidth="1"/>
+    <col min="283" max="283" width="2.6328125" style="15" customWidth="1"/>
+    <col min="284" max="289" width="2.6328125" style="12" customWidth="1"/>
+    <col min="290" max="290" width="2.6328125" style="15" customWidth="1"/>
+    <col min="291" max="296" width="2.6328125" style="12" customWidth="1"/>
+    <col min="297" max="297" width="2.6328125" style="15" customWidth="1"/>
+    <col min="298" max="303" width="2.6328125" style="12" customWidth="1"/>
+    <col min="304" max="304" width="2.6328125" style="15" customWidth="1"/>
+    <col min="305" max="310" width="2.6328125" style="12" customWidth="1"/>
+    <col min="311" max="311" width="2.6328125" style="15" customWidth="1"/>
+    <col min="312" max="317" width="2.6328125" style="12" customWidth="1"/>
+    <col min="318" max="318" width="2.6328125" style="15" customWidth="1"/>
+    <col min="319" max="324" width="2.6328125" style="12" customWidth="1"/>
+    <col min="325" max="325" width="2.6328125" style="15" customWidth="1"/>
+    <col min="326" max="331" width="2.6328125" style="12" customWidth="1"/>
+    <col min="332" max="332" width="2.6328125" style="15" customWidth="1"/>
+    <col min="333" max="338" width="2.6328125" style="12" customWidth="1"/>
+    <col min="339" max="339" width="2.6328125" style="15" customWidth="1"/>
+    <col min="340" max="345" width="2.6328125" style="12" customWidth="1"/>
+    <col min="346" max="346" width="2.6328125" style="15" customWidth="1"/>
+    <col min="347" max="352" width="2.6328125" style="12" customWidth="1"/>
+    <col min="353" max="353" width="2.6328125" style="15" customWidth="1"/>
+    <col min="354" max="359" width="2.6328125" style="12" customWidth="1"/>
+    <col min="360" max="360" width="2.6328125" style="15" customWidth="1"/>
+    <col min="361" max="366" width="2.6328125" style="12" customWidth="1"/>
+    <col min="367" max="367" width="2.6328125" style="15" customWidth="1"/>
+    <col min="368" max="373" width="2.6328125" style="12" customWidth="1"/>
+    <col min="374" max="374" width="2.6328125" style="15" customWidth="1"/>
+    <col min="375" max="380" width="2.6328125" style="12" customWidth="1"/>
+    <col min="381" max="381" width="2.6328125" style="15" customWidth="1"/>
+    <col min="382" max="387" width="2.6328125" style="12" customWidth="1"/>
+    <col min="388" max="388" width="2.6328125" style="15" customWidth="1"/>
+    <col min="389" max="394" width="2.6328125" style="12" customWidth="1"/>
+    <col min="395" max="395" width="2.6328125" style="15" customWidth="1"/>
+    <col min="396" max="401" width="2.6328125" style="12" customWidth="1"/>
+    <col min="402" max="402" width="2.6328125" style="15" customWidth="1"/>
+    <col min="403" max="408" width="2.6328125" style="12" customWidth="1"/>
+    <col min="409" max="409" width="2.6328125" style="15" customWidth="1"/>
+    <col min="410" max="415" width="2.6328125" style="12" customWidth="1"/>
+    <col min="416" max="416" width="2.6328125" style="15" customWidth="1"/>
+    <col min="417" max="422" width="2.6328125" style="12" customWidth="1"/>
+    <col min="423" max="423" width="2.6328125" style="15" customWidth="1"/>
+    <col min="424" max="428" width="2.6328125" style="12" customWidth="1"/>
+    <col min="429" max="429" width="8.81640625" style="12" customWidth="1"/>
+    <col min="430" max="16384" width="8.81640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:429" ht="19.95" customHeight="1">
+    <row r="1" spans="2:429" ht="20" customHeight="1">
       <c r="C1" s="27"/>
-      <c r="D1" s="70">
+      <c r="D1" s="76">
         <v>46327</v>
       </c>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="71"/>
-      <c r="AA1" s="71"/>
-      <c r="AB1" s="71"/>
-      <c r="AC1" s="71"/>
-      <c r="AD1" s="71"/>
-      <c r="AE1" s="71"/>
-      <c r="AF1" s="71"/>
-      <c r="AG1" s="72"/>
-      <c r="AH1" s="70">
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="77"/>
+      <c r="W1" s="77"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="77"/>
+      <c r="Z1" s="77"/>
+      <c r="AA1" s="77"/>
+      <c r="AB1" s="77"/>
+      <c r="AC1" s="77"/>
+      <c r="AD1" s="77"/>
+      <c r="AE1" s="77"/>
+      <c r="AF1" s="77"/>
+      <c r="AG1" s="78"/>
+      <c r="AH1" s="76">
         <v>46357</v>
       </c>
-      <c r="AI1" s="71"/>
-      <c r="AJ1" s="71"/>
-      <c r="AK1" s="71"/>
-      <c r="AL1" s="71"/>
-      <c r="AM1" s="71"/>
-      <c r="AN1" s="71"/>
-      <c r="AO1" s="71"/>
-      <c r="AP1" s="71"/>
-      <c r="AQ1" s="71"/>
-      <c r="AR1" s="71"/>
-      <c r="AS1" s="71"/>
-      <c r="AT1" s="71"/>
-      <c r="AU1" s="71"/>
-      <c r="AV1" s="71"/>
-      <c r="AW1" s="71"/>
-      <c r="AX1" s="71"/>
-      <c r="AY1" s="71"/>
-      <c r="AZ1" s="71"/>
-      <c r="BA1" s="71"/>
-      <c r="BB1" s="71"/>
-      <c r="BC1" s="71"/>
-      <c r="BD1" s="71"/>
-      <c r="BE1" s="71"/>
-      <c r="BF1" s="71"/>
-      <c r="BG1" s="71"/>
-      <c r="BH1" s="71"/>
-      <c r="BI1" s="71"/>
-      <c r="BJ1" s="71"/>
-      <c r="BK1" s="71"/>
-      <c r="BL1" s="72"/>
-      <c r="BM1" s="70">
+      <c r="AI1" s="77"/>
+      <c r="AJ1" s="77"/>
+      <c r="AK1" s="77"/>
+      <c r="AL1" s="77"/>
+      <c r="AM1" s="77"/>
+      <c r="AN1" s="77"/>
+      <c r="AO1" s="77"/>
+      <c r="AP1" s="77"/>
+      <c r="AQ1" s="77"/>
+      <c r="AR1" s="77"/>
+      <c r="AS1" s="77"/>
+      <c r="AT1" s="77"/>
+      <c r="AU1" s="77"/>
+      <c r="AV1" s="77"/>
+      <c r="AW1" s="77"/>
+      <c r="AX1" s="77"/>
+      <c r="AY1" s="77"/>
+      <c r="AZ1" s="77"/>
+      <c r="BA1" s="77"/>
+      <c r="BB1" s="77"/>
+      <c r="BC1" s="77"/>
+      <c r="BD1" s="77"/>
+      <c r="BE1" s="77"/>
+      <c r="BF1" s="77"/>
+      <c r="BG1" s="77"/>
+      <c r="BH1" s="77"/>
+      <c r="BI1" s="77"/>
+      <c r="BJ1" s="77"/>
+      <c r="BK1" s="77"/>
+      <c r="BL1" s="78"/>
+      <c r="BM1" s="76">
         <v>46388</v>
       </c>
-      <c r="BN1" s="71"/>
-      <c r="BO1" s="71"/>
-      <c r="BP1" s="71"/>
-      <c r="BQ1" s="71"/>
-      <c r="BR1" s="71"/>
-      <c r="BS1" s="71"/>
-      <c r="BT1" s="71"/>
-      <c r="BU1" s="71"/>
-      <c r="BV1" s="71"/>
-      <c r="BW1" s="71"/>
-      <c r="BX1" s="71"/>
-      <c r="BY1" s="71"/>
-      <c r="BZ1" s="71"/>
-      <c r="CA1" s="71"/>
-      <c r="CB1" s="71"/>
-      <c r="CC1" s="71"/>
-      <c r="CD1" s="71"/>
-      <c r="CE1" s="71"/>
-      <c r="CF1" s="71"/>
-      <c r="CG1" s="71"/>
-      <c r="CH1" s="71"/>
-      <c r="CI1" s="71"/>
-      <c r="CJ1" s="71"/>
-      <c r="CK1" s="71"/>
-      <c r="CL1" s="71"/>
-      <c r="CM1" s="71"/>
-      <c r="CN1" s="71"/>
-      <c r="CO1" s="71"/>
-      <c r="CP1" s="71"/>
-      <c r="CQ1" s="72"/>
-      <c r="CR1" s="70">
+      <c r="BN1" s="77"/>
+      <c r="BO1" s="77"/>
+      <c r="BP1" s="77"/>
+      <c r="BQ1" s="77"/>
+      <c r="BR1" s="77"/>
+      <c r="BS1" s="77"/>
+      <c r="BT1" s="77"/>
+      <c r="BU1" s="77"/>
+      <c r="BV1" s="77"/>
+      <c r="BW1" s="77"/>
+      <c r="BX1" s="77"/>
+      <c r="BY1" s="77"/>
+      <c r="BZ1" s="77"/>
+      <c r="CA1" s="77"/>
+      <c r="CB1" s="77"/>
+      <c r="CC1" s="77"/>
+      <c r="CD1" s="77"/>
+      <c r="CE1" s="77"/>
+      <c r="CF1" s="77"/>
+      <c r="CG1" s="77"/>
+      <c r="CH1" s="77"/>
+      <c r="CI1" s="77"/>
+      <c r="CJ1" s="77"/>
+      <c r="CK1" s="77"/>
+      <c r="CL1" s="77"/>
+      <c r="CM1" s="77"/>
+      <c r="CN1" s="77"/>
+      <c r="CO1" s="77"/>
+      <c r="CP1" s="77"/>
+      <c r="CQ1" s="78"/>
+      <c r="CR1" s="76">
         <v>46419</v>
       </c>
-      <c r="CS1" s="71"/>
-      <c r="CT1" s="71"/>
-      <c r="CU1" s="71"/>
-      <c r="CV1" s="71"/>
-      <c r="CW1" s="71"/>
-      <c r="CX1" s="71"/>
-      <c r="CY1" s="71"/>
-      <c r="CZ1" s="71"/>
-      <c r="DA1" s="71"/>
-      <c r="DB1" s="71"/>
-      <c r="DC1" s="71"/>
-      <c r="DD1" s="71"/>
-      <c r="DE1" s="71"/>
-      <c r="DF1" s="71"/>
-      <c r="DG1" s="71"/>
-      <c r="DH1" s="71"/>
-      <c r="DI1" s="71"/>
-      <c r="DJ1" s="71"/>
-      <c r="DK1" s="71"/>
-      <c r="DL1" s="71"/>
-      <c r="DM1" s="71"/>
-      <c r="DN1" s="71"/>
-      <c r="DO1" s="71"/>
-      <c r="DP1" s="71"/>
-      <c r="DQ1" s="71"/>
-      <c r="DR1" s="71"/>
-      <c r="DS1" s="72"/>
-      <c r="DT1" s="70">
+      <c r="CS1" s="77"/>
+      <c r="CT1" s="77"/>
+      <c r="CU1" s="77"/>
+      <c r="CV1" s="77"/>
+      <c r="CW1" s="77"/>
+      <c r="CX1" s="77"/>
+      <c r="CY1" s="77"/>
+      <c r="CZ1" s="77"/>
+      <c r="DA1" s="77"/>
+      <c r="DB1" s="77"/>
+      <c r="DC1" s="77"/>
+      <c r="DD1" s="77"/>
+      <c r="DE1" s="77"/>
+      <c r="DF1" s="77"/>
+      <c r="DG1" s="77"/>
+      <c r="DH1" s="77"/>
+      <c r="DI1" s="77"/>
+      <c r="DJ1" s="77"/>
+      <c r="DK1" s="77"/>
+      <c r="DL1" s="77"/>
+      <c r="DM1" s="77"/>
+      <c r="DN1" s="77"/>
+      <c r="DO1" s="77"/>
+      <c r="DP1" s="77"/>
+      <c r="DQ1" s="77"/>
+      <c r="DR1" s="77"/>
+      <c r="DS1" s="78"/>
+      <c r="DT1" s="76">
         <v>46447</v>
       </c>
-      <c r="DU1" s="71"/>
-      <c r="DV1" s="71"/>
-      <c r="DW1" s="71"/>
-      <c r="DX1" s="71"/>
-      <c r="DY1" s="71"/>
-      <c r="DZ1" s="71"/>
-      <c r="EA1" s="71"/>
-      <c r="EB1" s="71"/>
-      <c r="EC1" s="71"/>
-      <c r="ED1" s="71"/>
-      <c r="EE1" s="71"/>
-      <c r="EF1" s="71"/>
-      <c r="EG1" s="71"/>
-      <c r="EH1" s="71"/>
-      <c r="EI1" s="71"/>
-      <c r="EJ1" s="71"/>
-      <c r="EK1" s="71"/>
-      <c r="EL1" s="71"/>
-      <c r="EM1" s="71"/>
-      <c r="EN1" s="71"/>
-      <c r="EO1" s="71"/>
-      <c r="EP1" s="71"/>
-      <c r="EQ1" s="71"/>
-      <c r="ER1" s="71"/>
-      <c r="ES1" s="71"/>
-      <c r="ET1" s="71"/>
-      <c r="EU1" s="71"/>
-      <c r="EV1" s="71"/>
-      <c r="EW1" s="71"/>
-      <c r="EX1" s="72"/>
-      <c r="EY1" s="70">
+      <c r="DU1" s="77"/>
+      <c r="DV1" s="77"/>
+      <c r="DW1" s="77"/>
+      <c r="DX1" s="77"/>
+      <c r="DY1" s="77"/>
+      <c r="DZ1" s="77"/>
+      <c r="EA1" s="77"/>
+      <c r="EB1" s="77"/>
+      <c r="EC1" s="77"/>
+      <c r="ED1" s="77"/>
+      <c r="EE1" s="77"/>
+      <c r="EF1" s="77"/>
+      <c r="EG1" s="77"/>
+      <c r="EH1" s="77"/>
+      <c r="EI1" s="77"/>
+      <c r="EJ1" s="77"/>
+      <c r="EK1" s="77"/>
+      <c r="EL1" s="77"/>
+      <c r="EM1" s="77"/>
+      <c r="EN1" s="77"/>
+      <c r="EO1" s="77"/>
+      <c r="EP1" s="77"/>
+      <c r="EQ1" s="77"/>
+      <c r="ER1" s="77"/>
+      <c r="ES1" s="77"/>
+      <c r="ET1" s="77"/>
+      <c r="EU1" s="77"/>
+      <c r="EV1" s="77"/>
+      <c r="EW1" s="77"/>
+      <c r="EX1" s="78"/>
+      <c r="EY1" s="76">
         <v>46478</v>
       </c>
-      <c r="EZ1" s="71"/>
-      <c r="FA1" s="71"/>
-      <c r="FB1" s="71"/>
-      <c r="FC1" s="71"/>
-      <c r="FD1" s="71"/>
-      <c r="FE1" s="71"/>
-      <c r="FF1" s="71"/>
-      <c r="FG1" s="71"/>
-      <c r="FH1" s="71"/>
-      <c r="FI1" s="71"/>
-      <c r="FJ1" s="71"/>
-      <c r="FK1" s="71"/>
-      <c r="FL1" s="71"/>
-      <c r="FM1" s="71"/>
-      <c r="FN1" s="71"/>
-      <c r="FO1" s="71"/>
-      <c r="FP1" s="71"/>
-      <c r="FQ1" s="71"/>
-      <c r="FR1" s="71"/>
-      <c r="FS1" s="71"/>
-      <c r="FT1" s="71"/>
-      <c r="FU1" s="71"/>
-      <c r="FV1" s="71"/>
-      <c r="FW1" s="71"/>
-      <c r="FX1" s="71"/>
-      <c r="FY1" s="71"/>
-      <c r="FZ1" s="71"/>
-      <c r="GA1" s="71"/>
-      <c r="GB1" s="72"/>
-      <c r="GC1" s="70">
+      <c r="EZ1" s="77"/>
+      <c r="FA1" s="77"/>
+      <c r="FB1" s="77"/>
+      <c r="FC1" s="77"/>
+      <c r="FD1" s="77"/>
+      <c r="FE1" s="77"/>
+      <c r="FF1" s="77"/>
+      <c r="FG1" s="77"/>
+      <c r="FH1" s="77"/>
+      <c r="FI1" s="77"/>
+      <c r="FJ1" s="77"/>
+      <c r="FK1" s="77"/>
+      <c r="FL1" s="77"/>
+      <c r="FM1" s="77"/>
+      <c r="FN1" s="77"/>
+      <c r="FO1" s="77"/>
+      <c r="FP1" s="77"/>
+      <c r="FQ1" s="77"/>
+      <c r="FR1" s="77"/>
+      <c r="FS1" s="77"/>
+      <c r="FT1" s="77"/>
+      <c r="FU1" s="77"/>
+      <c r="FV1" s="77"/>
+      <c r="FW1" s="77"/>
+      <c r="FX1" s="77"/>
+      <c r="FY1" s="77"/>
+      <c r="FZ1" s="77"/>
+      <c r="GA1" s="77"/>
+      <c r="GB1" s="78"/>
+      <c r="GC1" s="76">
         <v>46508</v>
       </c>
-      <c r="GD1" s="71"/>
-      <c r="GE1" s="71"/>
-      <c r="GF1" s="71"/>
-      <c r="GG1" s="71"/>
-      <c r="GH1" s="71"/>
-      <c r="GI1" s="71"/>
-      <c r="GJ1" s="71"/>
-      <c r="GK1" s="71"/>
-      <c r="GL1" s="71"/>
-      <c r="GM1" s="71"/>
-      <c r="GN1" s="71"/>
-      <c r="GO1" s="71"/>
-      <c r="GP1" s="71"/>
-      <c r="GQ1" s="71"/>
-      <c r="GR1" s="71"/>
-      <c r="GS1" s="71"/>
-      <c r="GT1" s="71"/>
-      <c r="GU1" s="71"/>
-      <c r="GV1" s="71"/>
-      <c r="GW1" s="71"/>
-      <c r="GX1" s="71"/>
-      <c r="GY1" s="71"/>
-      <c r="GZ1" s="71"/>
-      <c r="HA1" s="71"/>
-      <c r="HB1" s="71"/>
-      <c r="HC1" s="71"/>
-      <c r="HD1" s="71"/>
-      <c r="HE1" s="71"/>
-      <c r="HF1" s="71"/>
-      <c r="HG1" s="72"/>
-      <c r="HH1" s="70">
+      <c r="GD1" s="77"/>
+      <c r="GE1" s="77"/>
+      <c r="GF1" s="77"/>
+      <c r="GG1" s="77"/>
+      <c r="GH1" s="77"/>
+      <c r="GI1" s="77"/>
+      <c r="GJ1" s="77"/>
+      <c r="GK1" s="77"/>
+      <c r="GL1" s="77"/>
+      <c r="GM1" s="77"/>
+      <c r="GN1" s="77"/>
+      <c r="GO1" s="77"/>
+      <c r="GP1" s="77"/>
+      <c r="GQ1" s="77"/>
+      <c r="GR1" s="77"/>
+      <c r="GS1" s="77"/>
+      <c r="GT1" s="77"/>
+      <c r="GU1" s="77"/>
+      <c r="GV1" s="77"/>
+      <c r="GW1" s="77"/>
+      <c r="GX1" s="77"/>
+      <c r="GY1" s="77"/>
+      <c r="GZ1" s="77"/>
+      <c r="HA1" s="77"/>
+      <c r="HB1" s="77"/>
+      <c r="HC1" s="77"/>
+      <c r="HD1" s="77"/>
+      <c r="HE1" s="77"/>
+      <c r="HF1" s="77"/>
+      <c r="HG1" s="78"/>
+      <c r="HH1" s="76">
         <v>46539</v>
       </c>
-      <c r="HI1" s="71"/>
-      <c r="HJ1" s="71"/>
-      <c r="HK1" s="71"/>
-      <c r="HL1" s="71"/>
-      <c r="HM1" s="71"/>
-      <c r="HN1" s="71"/>
-      <c r="HO1" s="71"/>
-      <c r="HP1" s="71"/>
-      <c r="HQ1" s="71"/>
-      <c r="HR1" s="71"/>
-      <c r="HS1" s="71"/>
-      <c r="HT1" s="71"/>
-      <c r="HU1" s="71"/>
-      <c r="HV1" s="71"/>
-      <c r="HW1" s="71"/>
-      <c r="HX1" s="71"/>
-      <c r="HY1" s="71"/>
-      <c r="HZ1" s="71"/>
-      <c r="IA1" s="71"/>
-      <c r="IB1" s="71"/>
-      <c r="IC1" s="71"/>
-      <c r="ID1" s="71"/>
-      <c r="IE1" s="71"/>
-      <c r="IF1" s="71"/>
-      <c r="IG1" s="71"/>
-      <c r="IH1" s="71"/>
-      <c r="II1" s="71"/>
-      <c r="IJ1" s="71"/>
-      <c r="IK1" s="72"/>
-      <c r="IL1" s="70">
+      <c r="HI1" s="77"/>
+      <c r="HJ1" s="77"/>
+      <c r="HK1" s="77"/>
+      <c r="HL1" s="77"/>
+      <c r="HM1" s="77"/>
+      <c r="HN1" s="77"/>
+      <c r="HO1" s="77"/>
+      <c r="HP1" s="77"/>
+      <c r="HQ1" s="77"/>
+      <c r="HR1" s="77"/>
+      <c r="HS1" s="77"/>
+      <c r="HT1" s="77"/>
+      <c r="HU1" s="77"/>
+      <c r="HV1" s="77"/>
+      <c r="HW1" s="77"/>
+      <c r="HX1" s="77"/>
+      <c r="HY1" s="77"/>
+      <c r="HZ1" s="77"/>
+      <c r="IA1" s="77"/>
+      <c r="IB1" s="77"/>
+      <c r="IC1" s="77"/>
+      <c r="ID1" s="77"/>
+      <c r="IE1" s="77"/>
+      <c r="IF1" s="77"/>
+      <c r="IG1" s="77"/>
+      <c r="IH1" s="77"/>
+      <c r="II1" s="77"/>
+      <c r="IJ1" s="77"/>
+      <c r="IK1" s="78"/>
+      <c r="IL1" s="76">
         <v>46569</v>
       </c>
-      <c r="IM1" s="71"/>
-      <c r="IN1" s="71"/>
-      <c r="IO1" s="71"/>
-      <c r="IP1" s="71"/>
-      <c r="IQ1" s="71"/>
-      <c r="IR1" s="71"/>
-      <c r="IS1" s="71"/>
-      <c r="IT1" s="71"/>
-      <c r="IU1" s="71"/>
-      <c r="IV1" s="71"/>
-      <c r="IW1" s="71"/>
-      <c r="IX1" s="71"/>
-      <c r="IY1" s="71"/>
-      <c r="IZ1" s="71"/>
-      <c r="JA1" s="71"/>
-      <c r="JB1" s="71"/>
-      <c r="JC1" s="71"/>
-      <c r="JD1" s="71"/>
-      <c r="JE1" s="71"/>
-      <c r="JF1" s="71"/>
-      <c r="JG1" s="71"/>
-      <c r="JH1" s="71"/>
-      <c r="JI1" s="71"/>
-      <c r="JJ1" s="71"/>
-      <c r="JK1" s="71"/>
-      <c r="JL1" s="71"/>
-      <c r="JM1" s="71"/>
-      <c r="JN1" s="71"/>
-      <c r="JO1" s="71"/>
-      <c r="JP1" s="72"/>
-      <c r="JQ1" s="70">
+      <c r="IM1" s="77"/>
+      <c r="IN1" s="77"/>
+      <c r="IO1" s="77"/>
+      <c r="IP1" s="77"/>
+      <c r="IQ1" s="77"/>
+      <c r="IR1" s="77"/>
+      <c r="IS1" s="77"/>
+      <c r="IT1" s="77"/>
+      <c r="IU1" s="77"/>
+      <c r="IV1" s="77"/>
+      <c r="IW1" s="77"/>
+      <c r="IX1" s="77"/>
+      <c r="IY1" s="77"/>
+      <c r="IZ1" s="77"/>
+      <c r="JA1" s="77"/>
+      <c r="JB1" s="77"/>
+      <c r="JC1" s="77"/>
+      <c r="JD1" s="77"/>
+      <c r="JE1" s="77"/>
+      <c r="JF1" s="77"/>
+      <c r="JG1" s="77"/>
+      <c r="JH1" s="77"/>
+      <c r="JI1" s="77"/>
+      <c r="JJ1" s="77"/>
+      <c r="JK1" s="77"/>
+      <c r="JL1" s="77"/>
+      <c r="JM1" s="77"/>
+      <c r="JN1" s="77"/>
+      <c r="JO1" s="77"/>
+      <c r="JP1" s="78"/>
+      <c r="JQ1" s="76">
         <v>46600</v>
       </c>
-      <c r="JR1" s="71"/>
-      <c r="JS1" s="71"/>
-      <c r="JT1" s="71"/>
-      <c r="JU1" s="71"/>
-      <c r="JV1" s="71"/>
-      <c r="JW1" s="71"/>
-      <c r="JX1" s="71"/>
-      <c r="JY1" s="71"/>
-      <c r="JZ1" s="71"/>
-      <c r="KA1" s="71"/>
-      <c r="KB1" s="71"/>
-      <c r="KC1" s="71"/>
-      <c r="KD1" s="71"/>
-      <c r="KE1" s="71"/>
-      <c r="KF1" s="71"/>
-      <c r="KG1" s="71"/>
-      <c r="KH1" s="71"/>
-      <c r="KI1" s="71"/>
-      <c r="KJ1" s="71"/>
-      <c r="KK1" s="71"/>
-      <c r="KL1" s="71"/>
-      <c r="KM1" s="71"/>
-      <c r="KN1" s="71"/>
-      <c r="KO1" s="71"/>
-      <c r="KP1" s="71"/>
-      <c r="KQ1" s="71"/>
-      <c r="KR1" s="71"/>
-      <c r="KS1" s="71"/>
-      <c r="KT1" s="71"/>
-      <c r="KU1" s="72"/>
-      <c r="KV1" s="70">
+      <c r="JR1" s="77"/>
+      <c r="JS1" s="77"/>
+      <c r="JT1" s="77"/>
+      <c r="JU1" s="77"/>
+      <c r="JV1" s="77"/>
+      <c r="JW1" s="77"/>
+      <c r="JX1" s="77"/>
+      <c r="JY1" s="77"/>
+      <c r="JZ1" s="77"/>
+      <c r="KA1" s="77"/>
+      <c r="KB1" s="77"/>
+      <c r="KC1" s="77"/>
+      <c r="KD1" s="77"/>
+      <c r="KE1" s="77"/>
+      <c r="KF1" s="77"/>
+      <c r="KG1" s="77"/>
+      <c r="KH1" s="77"/>
+      <c r="KI1" s="77"/>
+      <c r="KJ1" s="77"/>
+      <c r="KK1" s="77"/>
+      <c r="KL1" s="77"/>
+      <c r="KM1" s="77"/>
+      <c r="KN1" s="77"/>
+      <c r="KO1" s="77"/>
+      <c r="KP1" s="77"/>
+      <c r="KQ1" s="77"/>
+      <c r="KR1" s="77"/>
+      <c r="KS1" s="77"/>
+      <c r="KT1" s="77"/>
+      <c r="KU1" s="78"/>
+      <c r="KV1" s="76">
         <v>46631</v>
       </c>
-      <c r="KW1" s="71"/>
-      <c r="KX1" s="71"/>
-      <c r="KY1" s="71"/>
-      <c r="KZ1" s="71"/>
-      <c r="LA1" s="71"/>
-      <c r="LB1" s="71"/>
-      <c r="LC1" s="71"/>
-      <c r="LD1" s="71"/>
-      <c r="LE1" s="71"/>
-      <c r="LF1" s="71"/>
-      <c r="LG1" s="71"/>
-      <c r="LH1" s="71"/>
-      <c r="LI1" s="71"/>
-      <c r="LJ1" s="71"/>
-      <c r="LK1" s="71"/>
-      <c r="LL1" s="71"/>
-      <c r="LM1" s="71"/>
-      <c r="LN1" s="71"/>
-      <c r="LO1" s="71"/>
-      <c r="LP1" s="71"/>
-      <c r="LQ1" s="71"/>
-      <c r="LR1" s="71"/>
-      <c r="LS1" s="71"/>
-      <c r="LT1" s="71"/>
-      <c r="LU1" s="71"/>
-      <c r="LV1" s="71"/>
-      <c r="LW1" s="71"/>
-      <c r="LX1" s="71"/>
-      <c r="LY1" s="72"/>
-      <c r="LZ1" s="70">
+      <c r="KW1" s="77"/>
+      <c r="KX1" s="77"/>
+      <c r="KY1" s="77"/>
+      <c r="KZ1" s="77"/>
+      <c r="LA1" s="77"/>
+      <c r="LB1" s="77"/>
+      <c r="LC1" s="77"/>
+      <c r="LD1" s="77"/>
+      <c r="LE1" s="77"/>
+      <c r="LF1" s="77"/>
+      <c r="LG1" s="77"/>
+      <c r="LH1" s="77"/>
+      <c r="LI1" s="77"/>
+      <c r="LJ1" s="77"/>
+      <c r="LK1" s="77"/>
+      <c r="LL1" s="77"/>
+      <c r="LM1" s="77"/>
+      <c r="LN1" s="77"/>
+      <c r="LO1" s="77"/>
+      <c r="LP1" s="77"/>
+      <c r="LQ1" s="77"/>
+      <c r="LR1" s="77"/>
+      <c r="LS1" s="77"/>
+      <c r="LT1" s="77"/>
+      <c r="LU1" s="77"/>
+      <c r="LV1" s="77"/>
+      <c r="LW1" s="77"/>
+      <c r="LX1" s="77"/>
+      <c r="LY1" s="78"/>
+      <c r="LZ1" s="76">
         <v>46661</v>
       </c>
-      <c r="MA1" s="71"/>
-      <c r="MB1" s="71"/>
-      <c r="MC1" s="71"/>
-      <c r="MD1" s="71"/>
-      <c r="ME1" s="71"/>
-      <c r="MF1" s="71"/>
-      <c r="MG1" s="71"/>
-      <c r="MH1" s="71"/>
-      <c r="MI1" s="71"/>
-      <c r="MJ1" s="71"/>
-      <c r="MK1" s="71"/>
-      <c r="ML1" s="71"/>
-      <c r="MM1" s="71"/>
-      <c r="MN1" s="71"/>
-      <c r="MO1" s="71"/>
-      <c r="MP1" s="71"/>
-      <c r="MQ1" s="71"/>
-      <c r="MR1" s="71"/>
-      <c r="MS1" s="71"/>
-      <c r="MT1" s="71"/>
-      <c r="MU1" s="71"/>
-      <c r="MV1" s="71"/>
-      <c r="MW1" s="71"/>
-      <c r="MX1" s="71"/>
-      <c r="MY1" s="71"/>
-      <c r="MZ1" s="71"/>
-      <c r="NA1" s="71"/>
-      <c r="NB1" s="71"/>
-      <c r="NC1" s="71"/>
-      <c r="ND1" s="72"/>
-      <c r="NE1" s="70">
+      <c r="MA1" s="77"/>
+      <c r="MB1" s="77"/>
+      <c r="MC1" s="77"/>
+      <c r="MD1" s="77"/>
+      <c r="ME1" s="77"/>
+      <c r="MF1" s="77"/>
+      <c r="MG1" s="77"/>
+      <c r="MH1" s="77"/>
+      <c r="MI1" s="77"/>
+      <c r="MJ1" s="77"/>
+      <c r="MK1" s="77"/>
+      <c r="ML1" s="77"/>
+      <c r="MM1" s="77"/>
+      <c r="MN1" s="77"/>
+      <c r="MO1" s="77"/>
+      <c r="MP1" s="77"/>
+      <c r="MQ1" s="77"/>
+      <c r="MR1" s="77"/>
+      <c r="MS1" s="77"/>
+      <c r="MT1" s="77"/>
+      <c r="MU1" s="77"/>
+      <c r="MV1" s="77"/>
+      <c r="MW1" s="77"/>
+      <c r="MX1" s="77"/>
+      <c r="MY1" s="77"/>
+      <c r="MZ1" s="77"/>
+      <c r="NA1" s="77"/>
+      <c r="NB1" s="77"/>
+      <c r="NC1" s="77"/>
+      <c r="ND1" s="78"/>
+      <c r="NE1" s="76">
         <v>46692</v>
       </c>
-      <c r="NF1" s="71"/>
-      <c r="NG1" s="71"/>
-      <c r="NH1" s="71"/>
-      <c r="NI1" s="71"/>
-      <c r="NJ1" s="71"/>
-      <c r="NK1" s="71"/>
-      <c r="NL1" s="71"/>
-      <c r="NM1" s="71"/>
-      <c r="NN1" s="71"/>
-      <c r="NO1" s="71"/>
-      <c r="NP1" s="71"/>
-      <c r="NQ1" s="71"/>
-      <c r="NR1" s="71"/>
-      <c r="NS1" s="71"/>
-      <c r="NT1" s="71"/>
-      <c r="NU1" s="71"/>
-      <c r="NV1" s="71"/>
-      <c r="NW1" s="71"/>
-      <c r="NX1" s="71"/>
-      <c r="NY1" s="71"/>
-      <c r="NZ1" s="71"/>
-      <c r="OA1" s="71"/>
-      <c r="OB1" s="71"/>
-      <c r="OC1" s="71"/>
-      <c r="OD1" s="71"/>
-      <c r="OE1" s="71"/>
-      <c r="OF1" s="71"/>
-      <c r="OG1" s="71"/>
-      <c r="OH1" s="72"/>
-      <c r="OI1" s="70">
+      <c r="NF1" s="77"/>
+      <c r="NG1" s="77"/>
+      <c r="NH1" s="77"/>
+      <c r="NI1" s="77"/>
+      <c r="NJ1" s="77"/>
+      <c r="NK1" s="77"/>
+      <c r="NL1" s="77"/>
+      <c r="NM1" s="77"/>
+      <c r="NN1" s="77"/>
+      <c r="NO1" s="77"/>
+      <c r="NP1" s="77"/>
+      <c r="NQ1" s="77"/>
+      <c r="NR1" s="77"/>
+      <c r="NS1" s="77"/>
+      <c r="NT1" s="77"/>
+      <c r="NU1" s="77"/>
+      <c r="NV1" s="77"/>
+      <c r="NW1" s="77"/>
+      <c r="NX1" s="77"/>
+      <c r="NY1" s="77"/>
+      <c r="NZ1" s="77"/>
+      <c r="OA1" s="77"/>
+      <c r="OB1" s="77"/>
+      <c r="OC1" s="77"/>
+      <c r="OD1" s="77"/>
+      <c r="OE1" s="77"/>
+      <c r="OF1" s="77"/>
+      <c r="OG1" s="77"/>
+      <c r="OH1" s="78"/>
+      <c r="OI1" s="76">
         <v>46722</v>
       </c>
-      <c r="OJ1" s="71"/>
-      <c r="OK1" s="71"/>
-      <c r="OL1" s="71"/>
-      <c r="OM1" s="71"/>
-      <c r="ON1" s="71"/>
-      <c r="OO1" s="71"/>
-      <c r="OP1" s="71"/>
-      <c r="OQ1" s="71"/>
-      <c r="OR1" s="71"/>
-      <c r="OS1" s="71"/>
-      <c r="OT1" s="71"/>
-      <c r="OU1" s="71"/>
-      <c r="OV1" s="71"/>
-      <c r="OW1" s="71"/>
-      <c r="OX1" s="71"/>
-      <c r="OY1" s="71"/>
-      <c r="OZ1" s="71"/>
-      <c r="PA1" s="71"/>
-      <c r="PB1" s="71"/>
-      <c r="PC1" s="71"/>
-      <c r="PD1" s="71"/>
-      <c r="PE1" s="71"/>
-      <c r="PF1" s="71"/>
-      <c r="PG1" s="71"/>
-      <c r="PH1" s="71"/>
-      <c r="PI1" s="71"/>
-      <c r="PJ1" s="71"/>
-      <c r="PK1" s="71"/>
-      <c r="PL1" s="71"/>
-      <c r="PM1" s="72"/>
+      <c r="OJ1" s="77"/>
+      <c r="OK1" s="77"/>
+      <c r="OL1" s="77"/>
+      <c r="OM1" s="77"/>
+      <c r="ON1" s="77"/>
+      <c r="OO1" s="77"/>
+      <c r="OP1" s="77"/>
+      <c r="OQ1" s="77"/>
+      <c r="OR1" s="77"/>
+      <c r="OS1" s="77"/>
+      <c r="OT1" s="77"/>
+      <c r="OU1" s="77"/>
+      <c r="OV1" s="77"/>
+      <c r="OW1" s="77"/>
+      <c r="OX1" s="77"/>
+      <c r="OY1" s="77"/>
+      <c r="OZ1" s="77"/>
+      <c r="PA1" s="77"/>
+      <c r="PB1" s="77"/>
+      <c r="PC1" s="77"/>
+      <c r="PD1" s="77"/>
+      <c r="PE1" s="77"/>
+      <c r="PF1" s="77"/>
+      <c r="PG1" s="77"/>
+      <c r="PH1" s="77"/>
+      <c r="PI1" s="77"/>
+      <c r="PJ1" s="77"/>
+      <c r="PK1" s="77"/>
+      <c r="PL1" s="77"/>
+      <c r="PM1" s="78"/>
     </row>
     <row r="2" spans="2:429" ht="10.5" customHeight="1">
       <c r="B2" s="25" t="s">
@@ -9874,11 +9874,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38AFB97A-96F2-4583-ACB9-D6943AFDA3A8}">
   <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" customWidth="1"/>
+    <col min="1" max="1" width="6.81640625" customWidth="1"/>
     <col min="2" max="2" width="47" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -9901,7 +9901,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.399999999999999">
+    <row r="3" spans="1:3">
       <c r="A3" s="35">
         <v>2</v>
       </c>

</xml_diff>